<commit_message>
Refine retention Excel with Qin=Qcap crossing points
Add interpolated start/end storage times (~9.4 and ~44.4 min) and
fix dynamic formula ranges for the longer hydrograph table.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +134,7 @@
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -267,12 +268,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Hydrogramme'!$A$4:$A$16</f>
+              <f>'Hydrogramme'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Hydrogramme'!$B$4:$B$16</f>
+              <f>'Hydrogramme'!$B$4:$B$18</f>
             </numRef>
           </val>
         </ser>
@@ -385,12 +386,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Calcul_A'!$A$8:$A$20</f>
+              <f>'Calcul_A'!$A$8:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcul_A'!$H$8:$H$20</f>
+              <f>'Calcul_A'!$H$8:$H$22</f>
             </numRef>
           </val>
         </ser>
@@ -503,12 +504,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Calcul_A'!$A$8:$A$20</f>
+              <f>'Calcul_A'!$A$8:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcul_A'!$B$8:$B$20</f>
+              <f>'Calcul_A'!$B$8:$B$22</f>
             </numRef>
           </val>
         </ser>
@@ -535,12 +536,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Calcul_A'!$A$8:$A$20</f>
+              <f>'Calcul_A'!$A$8:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcul_A'!$C$8:$C$20</f>
+              <f>'Calcul_A'!$C$8:$C$22</f>
             </numRef>
           </val>
         </ser>
@@ -1285,7 +1286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1337,125 +1338,151 @@
     </row>
     <row r="6">
       <c r="A6" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>1.857</v>
-      </c>
-      <c r="C6" s="4" t="inlineStr"/>
+        <v>9.369999999999999</v>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Qin = Qcap (croisement)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3.202</v>
+        <v>1.857</v>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6.309</v>
+        <v>3.202</v>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Pointe</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6.309</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>5.846</v>
-      </c>
-      <c r="C10" s="4" t="inlineStr"/>
+        <v>22.5</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Pointe</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
-        <v>32.5</v>
+        <v>27.5</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>3.857</v>
+        <v>5.846</v>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="n">
-        <v>37.5</v>
+        <v>32.5</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>2.689</v>
+        <v>3.857</v>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="n">
-        <v>42.5</v>
+        <v>37.5</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1.953</v>
+        <v>2.689</v>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="n">
-        <v>47.5</v>
+        <v>42.5</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1.462</v>
+        <v>1.953</v>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>1.121</v>
-      </c>
-      <c r="C15" s="4" t="inlineStr"/>
+        <v>44.4</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Qin = Qcap (croisement)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1.462</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1.121</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
         <v>57.5</v>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B18" s="5" t="n">
         <v>0.875</v>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Qpointe (m³/s)</t>
         </is>
       </c>
-      <c r="B18" s="17">
-        <f>MAX(B4:B16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="B20" s="18">
+        <f>MAX(B4:B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>t pointe (min)</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B21" s="19" t="n">
         <v>22.5</v>
       </c>
     </row>
@@ -1471,7 +1498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1498,7 +1525,7 @@
           <t>Qout (m³/s)</t>
         </is>
       </c>
-      <c r="B2" s="19">
+      <c r="B2" s="20">
         <f>Parametres!B13</f>
         <v/>
       </c>
@@ -1509,8 +1536,8 @@
           <t>Vmax (m³)</t>
         </is>
       </c>
-      <c r="B3" s="20">
-        <f>MAX(H8:H20)</f>
+      <c r="B3" s="21">
+        <f>MAX(H8:H22)</f>
         <v/>
       </c>
       <c r="C3" t="inlineStr">
@@ -1599,7 +1626,7 @@
         <f>Hydrogramme!B4</f>
         <v/>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1616,7 +1643,7 @@
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="23" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="4">
@@ -1633,7 +1660,7 @@
         <f>Hydrogramme!B5</f>
         <v/>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1653,7 +1680,7 @@
         <f>F9-(H9-H8)</f>
         <v/>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="24">
         <f>MAX(0,H8+0.5*(D8+D9)*E9)</f>
         <v/>
       </c>
@@ -1671,7 +1698,7 @@
         <f>Hydrogramme!B6</f>
         <v/>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1691,7 +1718,7 @@
         <f>F10-(H10-H9)</f>
         <v/>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="24">
         <f>MAX(0,H9+0.5*(D9+D10)*E10)</f>
         <v/>
       </c>
@@ -1709,7 +1736,7 @@
         <f>Hydrogramme!B7</f>
         <v/>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1729,7 +1756,7 @@
         <f>F11-(H11-H10)</f>
         <v/>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="24">
         <f>MAX(0,H10+0.5*(D10+D11)*E11)</f>
         <v/>
       </c>
@@ -1747,7 +1774,7 @@
         <f>Hydrogramme!B8</f>
         <v/>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1767,7 +1794,7 @@
         <f>F12-(H12-H11)</f>
         <v/>
       </c>
-      <c r="H12" s="23">
+      <c r="H12" s="24">
         <f>MAX(0,H11+0.5*(D11+D12)*E12)</f>
         <v/>
       </c>
@@ -1785,7 +1812,7 @@
         <f>Hydrogramme!B9</f>
         <v/>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1805,7 +1832,7 @@
         <f>F13-(H13-H12)</f>
         <v/>
       </c>
-      <c r="H13" s="23">
+      <c r="H13" s="24">
         <f>MAX(0,H12+0.5*(D12+D13)*E13)</f>
         <v/>
       </c>
@@ -1823,7 +1850,7 @@
         <f>Hydrogramme!B10</f>
         <v/>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1843,7 +1870,7 @@
         <f>F14-(H14-H13)</f>
         <v/>
       </c>
-      <c r="H14" s="23">
+      <c r="H14" s="24">
         <f>MAX(0,H13+0.5*(D13+D14)*E14)</f>
         <v/>
       </c>
@@ -1861,7 +1888,7 @@
         <f>Hydrogramme!B11</f>
         <v/>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1881,7 +1908,7 @@
         <f>F15-(H15-H14)</f>
         <v/>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="24">
         <f>MAX(0,H14+0.5*(D14+D15)*E15)</f>
         <v/>
       </c>
@@ -1899,7 +1926,7 @@
         <f>Hydrogramme!B12</f>
         <v/>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1919,7 +1946,7 @@
         <f>F16-(H16-H15)</f>
         <v/>
       </c>
-      <c r="H16" s="23">
+      <c r="H16" s="24">
         <f>MAX(0,H15+0.5*(D15+D16)*E16)</f>
         <v/>
       </c>
@@ -1937,7 +1964,7 @@
         <f>Hydrogramme!B13</f>
         <v/>
       </c>
-      <c r="C17" s="21">
+      <c r="C17" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1957,7 +1984,7 @@
         <f>F17-(H17-H16)</f>
         <v/>
       </c>
-      <c r="H17" s="23">
+      <c r="H17" s="24">
         <f>MAX(0,H16+0.5*(D16+D17)*E17)</f>
         <v/>
       </c>
@@ -1975,7 +2002,7 @@
         <f>Hydrogramme!B14</f>
         <v/>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1995,7 +2022,7 @@
         <f>F18-(H18-H17)</f>
         <v/>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="24">
         <f>MAX(0,H17+0.5*(D17+D18)*E18)</f>
         <v/>
       </c>
@@ -2013,7 +2040,7 @@
         <f>Hydrogramme!B15</f>
         <v/>
       </c>
-      <c r="C19" s="21">
+      <c r="C19" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2033,7 +2060,7 @@
         <f>F19-(H19-H18)</f>
         <v/>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="24">
         <f>MAX(0,H18+0.5*(D18+D19)*E19)</f>
         <v/>
       </c>
@@ -2051,7 +2078,7 @@
         <f>Hydrogramme!B16</f>
         <v/>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="22">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2071,12 +2098,88 @@
         <f>F20-(H20-H19)</f>
         <v/>
       </c>
-      <c r="H20" s="23">
+      <c r="H20" s="24">
         <f>MAX(0,H19+0.5*(D19+D20)*E20)</f>
         <v/>
       </c>
       <c r="I20" s="4">
         <f>IF(H20&gt;0.5,"oui","non")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16">
+        <f>Hydrogramme!A17</f>
+        <v/>
+      </c>
+      <c r="B21" s="5">
+        <f>Hydrogramme!B17</f>
+        <v/>
+      </c>
+      <c r="C21" s="22">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D21" s="5">
+        <f>B21-C21</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>(A21-A20)*60</f>
+        <v/>
+      </c>
+      <c r="F21" s="16">
+        <f>0.5*(B20+B21)*E21</f>
+        <v/>
+      </c>
+      <c r="G21" s="16">
+        <f>F21-(H21-H20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="24">
+        <f>MAX(0,H20+0.5*(D20+D21)*E21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="4">
+        <f>IF(H21&gt;0.5,"oui","non")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16">
+        <f>Hydrogramme!A18</f>
+        <v/>
+      </c>
+      <c r="B22" s="5">
+        <f>Hydrogramme!B18</f>
+        <v/>
+      </c>
+      <c r="C22" s="22">
+        <f>$B$2</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>B22-C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="16">
+        <f>(A22-A21)*60</f>
+        <v/>
+      </c>
+      <c r="F22" s="16">
+        <f>0.5*(B21+B22)*E22</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>F22-(H22-H21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="24">
+        <f>MAX(0,H21+0.5*(D21+D22)*E22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="4">
+        <f>IF(H22&gt;0.5,"oui","non")</f>
         <v/>
       </c>
     </row>
@@ -2092,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2112,7 +2215,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>H = V / Aire_bassin.  Qorifice = Cd·(πD²/4)·√(2gH).  Qout = MIN(Qcap, Qorifice) si V&gt;0; si V≈0, Qout = MIN(Qin, Qcap).  ΔV = (Qin_moyenne − Qout)·Δt.  Ajuster Cd, Aire, Qcap (jaune).</t>
         </is>
@@ -2125,7 +2228,7 @@
           <t>Cd</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n">
+      <c r="B5" s="26" t="n">
         <v>0.62</v>
       </c>
     </row>
@@ -2135,7 +2238,7 @@
           <t>D (m)</t>
         </is>
       </c>
-      <c r="B6" s="25" t="n">
+      <c r="B6" s="26" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -2145,7 +2248,7 @@
           <t>Qcap (m³/s)</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="26">
         <f>Parametres!B13</f>
         <v/>
       </c>
@@ -2156,7 +2259,7 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="26">
         <f>Parametres!B15</f>
         <v/>
       </c>
@@ -2167,8 +2270,8 @@
           <t>Vmax_B (m³)</t>
         </is>
       </c>
-      <c r="B9" s="20">
-        <f>MAX(G14:G26)</f>
+      <c r="B9" s="21">
+        <f>MAX(G14:G28)</f>
         <v/>
       </c>
     </row>
@@ -2242,7 +2345,7 @@
       <c r="F14" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="23" t="n">
+      <c r="G14" s="24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2271,7 +2374,7 @@
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="G15" s="23">
+      <c r="G15" s="24">
         <f>MAX(0,G14+(0.5*(B14+B15)-E15)*F15)</f>
         <v/>
       </c>
@@ -2301,7 +2404,7 @@
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="G16" s="23">
+      <c r="G16" s="24">
         <f>MAX(0,G15+(0.5*(B15+B16)-E16)*F16)</f>
         <v/>
       </c>
@@ -2331,7 +2434,7 @@
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="G17" s="23">
+      <c r="G17" s="24">
         <f>MAX(0,G16+(0.5*(B16+B17)-E17)*F17)</f>
         <v/>
       </c>
@@ -2361,7 +2464,7 @@
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="G18" s="23">
+      <c r="G18" s="24">
         <f>MAX(0,G17+(0.5*(B17+B18)-E18)*F18)</f>
         <v/>
       </c>
@@ -2391,7 +2494,7 @@
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="24">
         <f>MAX(0,G18+(0.5*(B18+B19)-E19)*F19)</f>
         <v/>
       </c>
@@ -2421,7 +2524,7 @@
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="24">
         <f>MAX(0,G19+(0.5*(B19+B20)-E20)*F20)</f>
         <v/>
       </c>
@@ -2451,7 +2554,7 @@
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="24">
         <f>MAX(0,G20+(0.5*(B20+B21)-E21)*F21)</f>
         <v/>
       </c>
@@ -2481,7 +2584,7 @@
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="G22" s="23">
+      <c r="G22" s="24">
         <f>MAX(0,G21+(0.5*(B21+B22)-E22)*F22)</f>
         <v/>
       </c>
@@ -2511,7 +2614,7 @@
         <f>(A23-A22)*60</f>
         <v/>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="24">
         <f>MAX(0,G22+(0.5*(B22+B23)-E23)*F23)</f>
         <v/>
       </c>
@@ -2541,7 +2644,7 @@
         <f>(A24-A23)*60</f>
         <v/>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="24">
         <f>MAX(0,G23+(0.5*(B23+B24)-E24)*F24)</f>
         <v/>
       </c>
@@ -2571,7 +2674,7 @@
         <f>(A25-A24)*60</f>
         <v/>
       </c>
-      <c r="G25" s="23">
+      <c r="G25" s="24">
         <f>MAX(0,G24+(0.5*(B24+B25)-E25)*F25)</f>
         <v/>
       </c>
@@ -2601,8 +2704,68 @@
         <f>(A26-A25)*60</f>
         <v/>
       </c>
-      <c r="G26" s="23">
+      <c r="G26" s="24">
         <f>MAX(0,G25+(0.5*(B25+B26)-E26)*F26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4">
+        <f>Hydrogramme!A17</f>
+        <v/>
+      </c>
+      <c r="B27" s="5">
+        <f>Hydrogramme!B17</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>IF($B$8&gt;0,G26/$B$8,0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="5">
+        <f>IF(C27&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C27))</f>
+        <v/>
+      </c>
+      <c r="E27" s="5">
+        <f>IF(G26&lt;=0.01,MIN(0.5*(B26+B27),$B$7),MIN($B$7,D27))</f>
+        <v/>
+      </c>
+      <c r="F27" s="16">
+        <f>(A27-A26)*60</f>
+        <v/>
+      </c>
+      <c r="G27" s="24">
+        <f>MAX(0,G26+(0.5*(B26+B27)-E27)*F27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4">
+        <f>Hydrogramme!A18</f>
+        <v/>
+      </c>
+      <c r="B28" s="5">
+        <f>Hydrogramme!B18</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>IF($B$8&gt;0,G27/$B$8,0)</f>
+        <v/>
+      </c>
+      <c r="D28" s="5">
+        <f>IF(C28&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C28))</f>
+        <v/>
+      </c>
+      <c r="E28" s="5">
+        <f>IF(G27&lt;=0.01,MIN(0.5*(B27+B28),$B$7),MIN($B$7,D28))</f>
+        <v/>
+      </c>
+      <c r="F28" s="16">
+        <f>(A28-A27)*60</f>
+        <v/>
+      </c>
+      <c r="G28" s="24">
+        <f>MAX(0,G27+(0.5*(B27+B28)-E28)*F28)</f>
         <v/>
       </c>
     </row>
@@ -2627,7 +2790,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>

</xml_diff>

<commit_message>
Document Manning n=0.013 full-pipe basis and inlet/outlet notes
Default Qout to computed Ø900 Q_plein (~1.668 m³/s); keep 1.77 as prior
office value; clarify that IC vs OC is not resolved for this estimate.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +128,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -960,12 +965,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -1086,7 +1091,7 @@
         <v>0.008489634748272452</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>1.77</v>
+        <v>1.668</v>
       </c>
     </row>
     <row r="7">
@@ -1130,151 +1135,318 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Entrées de calcul (jaune)</t>
+          <t>Capacité Ø900 — Manning pleine section (n = 0,013)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Qout_cap_900 (m³/s)</t>
+          <t>n Manning (-)</t>
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>1.77</v>
+        <v>0.013</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Débit sortant constant — Méthode A (capacité Ø900)</t>
+          <t>Fourni (béton typique ~0,012–0,015)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Facteur_securite (-)</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Marge sur Vmax (ex. 1.20 = +20%)</t>
-        </is>
+          <t>D (m)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aire_bassin_m2</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>2500</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Aire plan d'eau approximative pour estimer H = V/A (Méthode B / niveau)</t>
-        </is>
+          <t>S0 = (Zamont−Zaval)/L</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>0.008489634748272452</v>
+      </c>
+      <c r="C15">
+        <f> (34.88 − 34.45) / 50.65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A = πD²/4 (m²)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>0.6361725123519332</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Résultats (formules — feuille Calcul_A)</t>
-        </is>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>R = D/4 (m)</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Vmax (m³)</t>
-        </is>
-      </c>
-      <c r="B18" s="13">
-        <f>Calcul_A!B3</f>
-        <v/>
+          <t>Q_plein = (1/n)·A·R^(2/3)·√S0</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>1.668006465155198</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>m³/s — capacité pleine section (hypothèse actuelle)</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>V_dimensionnement = Vmax × facteur (m³)</t>
-        </is>
-      </c>
-      <c r="B19" s="13">
-        <f>B18*B14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Hmax approx (m) = Vmax / Aire</t>
-        </is>
-      </c>
-      <c r="B20" s="14">
-        <f>IF(B15&gt;0,B18/B15,0)</f>
-        <v/>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Estimation grossière si l'aire de bassin est constante</t>
+          <t>Q utilisé avant (m³/s)</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ancienne valeur bureau (~6% plus haute; même méthode)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Entrées de calcul rétention (jaune)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Qout_cap_900 (m³/s)</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Par défaut = Q_plein Manning. Mettre 1.77 pour retrouver l'ancien calcul.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• Méthode A: Qout fixe = capacité Ø900. Valable comme estimation prudente / enveloppe basse de sortie.</t>
+          <t>Facteur_securite (-)</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Marge sur Vmax (ex. 1.20 = +20%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Le stockage commence quand Qin dépasse Qout; Vmax est le maximum du volume cumulé (pas (Qp-Qout)×durée).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>• Méthode B (feuille Calcul_B): Qout augmente un peu avec la charge H (orifice plafonné), plus réaliste si disponible.</t>
+          <t>Aire_bassin_m2</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Aire plan d'eau approx. pour H = V/A (Méthode B)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>• Les capacités 1.77 et 4.93 m³/s sont prises comme données; idéalement remplacer par une courbe Q=f(H) calibrée.</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Résultats (formules — feuille Calcul_A)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Vmax (m³)</t>
+        </is>
+      </c>
+      <c r="B27" s="18">
+        <f>Calcul_A!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>V_dimensionnement = Vmax × facteur (m³)</t>
+        </is>
+      </c>
+      <c r="B28" s="18">
+        <f>B27*B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hmax approx (m) = Vmax / Aire</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>IF(B24&gt;0,B27/B24,0)</f>
+        <v/>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Estimation grossière si l'aire de bassin est constante</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Inlet control vs outlet control — qu'est-ce que ça veut dire?</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>• Inlet control (contrôle à l'entrée): le débit est limité par l'entrée du ponceau (forme d'entrée, HW/D).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Le tuyau aval « n'aspire » pas assez pour influencer — Q dépend surtout de la charge amont H, pas de L ni de n.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>• Outlet control (contrôle à la sortie / frottement): le débit dépend de la longueur, de n, de la pente et de la charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (énergie amont → aval). Manning pleine section est une hypothèse de type outlet/frottement à section pleine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>• Ici L/D = 56 (tuyau assez long) → le contrôle par frottement (outlet) est souvent plausible,</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mais sans analyse FHWA/HY-8 on ne peut pas l'affirmer. Pour dimensionner la rétention, Q_plein constant est</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  en général prudent (si la charge monte, le débit réel peut être un peu plus élevé → Vmax un peu plus bas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>• On n'a pas besoin de trancher IC/OC pour utiliser ce classeur: garder Qout = Q_plein (ou 1.77) suffit pour une 1re estimation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (n=0,013). Pas un jugement IC/OC complet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>• Le stockage commence quand Qin dépasse Qout; Vmax = max du volume stocké (pas (Qp−Qout)×durée).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>• Méthode B: orifice Q=f(H) plafonné — illustration seulement; HY-8 / HEC-RAS donnerait une vraie courbe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>• Ø1200 Q_plein ≈ 4,93 m³/s avec le même n: cohérent, mais aval du Ø900 donc non limitant pour la rétention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>• Vérifier que le radier amont Ø900 (34.88) est bien le fond de la zone de rétention étudiée.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="15">
     <mergeCell ref="A9:H10"/>
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1295,7 +1467,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Hydrogramme d'entrée (point Ø1500 / entrée rétention)</t>
         </is>
@@ -1319,7 +1491,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="21" t="n">
         <v>0</v>
       </c>
       <c r="B4" s="5" t="n">
@@ -1328,7 +1500,7 @@
       <c r="C4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="21" t="n">
         <v>5</v>
       </c>
       <c r="B5" s="5" t="n">
@@ -1337,11 +1509,11 @@
       <c r="C5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
-        <v>9.369999999999999</v>
-      </c>
-      <c r="B6" s="17" t="n">
-        <v>1.77</v>
+      <c r="A6" s="21" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="B6" s="22" t="n">
+        <v>1.668</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -1350,7 +1522,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="21" t="n">
         <v>10</v>
       </c>
       <c r="B7" s="5" t="n">
@@ -1359,7 +1531,7 @@
       <c r="C7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="21" t="n">
         <v>15</v>
       </c>
       <c r="B8" s="5" t="n">
@@ -1368,7 +1540,7 @@
       <c r="C8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="21" t="n">
         <v>20</v>
       </c>
       <c r="B9" s="5" t="n">
@@ -1377,7 +1549,7 @@
       <c r="C9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="21" t="n">
         <v>22.5</v>
       </c>
       <c r="B10" s="8" t="n">
@@ -1390,7 +1562,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="21" t="n">
         <v>27.5</v>
       </c>
       <c r="B11" s="5" t="n">
@@ -1399,7 +1571,7 @@
       <c r="C11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n">
+      <c r="A12" s="21" t="n">
         <v>32.5</v>
       </c>
       <c r="B12" s="5" t="n">
@@ -1408,7 +1580,7 @@
       <c r="C12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="21" t="n">
         <v>37.5</v>
       </c>
       <c r="B13" s="5" t="n">
@@ -1417,7 +1589,7 @@
       <c r="C13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n">
+      <c r="A14" s="21" t="n">
         <v>42.5</v>
       </c>
       <c r="B14" s="5" t="n">
@@ -1426,11 +1598,11 @@
       <c r="C14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="B15" s="17" t="n">
-        <v>1.77</v>
+      <c r="A15" s="21" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>1.668</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
@@ -1439,7 +1611,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n">
+      <c r="A16" s="21" t="n">
         <v>47.5</v>
       </c>
       <c r="B16" s="5" t="n">
@@ -1448,7 +1620,7 @@
       <c r="C16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="21" t="n">
         <v>52.5</v>
       </c>
       <c r="B17" s="5" t="n">
@@ -1457,7 +1629,7 @@
       <c r="C17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="n">
+      <c r="A18" s="21" t="n">
         <v>57.5</v>
       </c>
       <c r="B18" s="5" t="n">
@@ -1471,7 +1643,7 @@
           <t>Qpointe (m³/s)</t>
         </is>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="23">
         <f>MAX(B4:B18)</f>
         <v/>
       </c>
@@ -1482,7 +1654,7 @@
           <t>t pointe (min)</t>
         </is>
       </c>
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="24" t="n">
         <v>22.5</v>
       </c>
     </row>
@@ -1513,7 +1685,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Méthode A — Qout constant = capacité Ø900</t>
         </is>
@@ -1525,8 +1697,8 @@
           <t>Qout (m³/s)</t>
         </is>
       </c>
-      <c r="B2" s="20">
-        <f>Parametres!B13</f>
+      <c r="B2" s="25">
+        <f>Parametres!B22</f>
         <v/>
       </c>
     </row>
@@ -1536,7 +1708,7 @@
           <t>Vmax (m³)</t>
         </is>
       </c>
-      <c r="B3" s="21">
+      <c r="B3" s="26">
         <f>MAX(H8:H22)</f>
         <v/>
       </c>
@@ -1554,19 +1726,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>voir courbe / entre 5 et 10 min (~9.4 min)</t>
+          <t>croisement Qin=Qcap dans Hydrogramme (~8.6 min si Q=1.668)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>t fin stockage approx (min)</t>
+          <t>t fin accumulation nette (min)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>entre 42.5 et 47.5 min (~44.4 min)</t>
+          <t>croisement descendant (~45.4 min si Q=1.668)</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1790,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16">
+      <c r="A8" s="21">
         <f>Hydrogramme!A4</f>
         <v/>
       </c>
@@ -1626,7 +1798,7 @@
         <f>Hydrogramme!B4</f>
         <v/>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1643,7 +1815,7 @@
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="23" t="n">
+      <c r="H8" s="28" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="4">
@@ -1652,7 +1824,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16">
+      <c r="A9" s="21">
         <f>Hydrogramme!A5</f>
         <v/>
       </c>
@@ -1660,7 +1832,7 @@
         <f>Hydrogramme!B5</f>
         <v/>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1668,19 +1840,19 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="21">
         <f>(A9-A8)*60</f>
         <v/>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="21">
         <f>0.5*(B8+B9)*E9</f>
         <v/>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="21">
         <f>F9-(H9-H8)</f>
         <v/>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="29">
         <f>MAX(0,H8+0.5*(D8+D9)*E9)</f>
         <v/>
       </c>
@@ -1690,7 +1862,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16">
+      <c r="A10" s="21">
         <f>Hydrogramme!A6</f>
         <v/>
       </c>
@@ -1698,7 +1870,7 @@
         <f>Hydrogramme!B6</f>
         <v/>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1706,19 +1878,19 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="21">
         <f>(A10-A9)*60</f>
         <v/>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="21">
         <f>0.5*(B9+B10)*E10</f>
         <v/>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="21">
         <f>F10-(H10-H9)</f>
         <v/>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="29">
         <f>MAX(0,H9+0.5*(D9+D10)*E10)</f>
         <v/>
       </c>
@@ -1728,7 +1900,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16">
+      <c r="A11" s="21">
         <f>Hydrogramme!A7</f>
         <v/>
       </c>
@@ -1736,7 +1908,7 @@
         <f>Hydrogramme!B7</f>
         <v/>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1744,19 +1916,19 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="21">
         <f>(A11-A10)*60</f>
         <v/>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="21">
         <f>0.5*(B10+B11)*E11</f>
         <v/>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="21">
         <f>F11-(H11-H10)</f>
         <v/>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="29">
         <f>MAX(0,H10+0.5*(D10+D11)*E11)</f>
         <v/>
       </c>
@@ -1766,7 +1938,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16">
+      <c r="A12" s="21">
         <f>Hydrogramme!A8</f>
         <v/>
       </c>
@@ -1774,7 +1946,7 @@
         <f>Hydrogramme!B8</f>
         <v/>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1782,19 +1954,19 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="21">
         <f>(A12-A11)*60</f>
         <v/>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="21">
         <f>0.5*(B11+B12)*E12</f>
         <v/>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="21">
         <f>F12-(H12-H11)</f>
         <v/>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="29">
         <f>MAX(0,H11+0.5*(D11+D12)*E12)</f>
         <v/>
       </c>
@@ -1804,7 +1976,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16">
+      <c r="A13" s="21">
         <f>Hydrogramme!A9</f>
         <v/>
       </c>
@@ -1812,7 +1984,7 @@
         <f>Hydrogramme!B9</f>
         <v/>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1820,19 +1992,19 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="21">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="21">
         <f>0.5*(B12+B13)*E13</f>
         <v/>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="21">
         <f>F13-(H13-H12)</f>
         <v/>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="29">
         <f>MAX(0,H12+0.5*(D12+D13)*E13)</f>
         <v/>
       </c>
@@ -1842,7 +2014,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16">
+      <c r="A14" s="21">
         <f>Hydrogramme!A10</f>
         <v/>
       </c>
@@ -1850,7 +2022,7 @@
         <f>Hydrogramme!B10</f>
         <v/>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1858,19 +2030,19 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="21">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="21">
         <f>0.5*(B13+B14)*E14</f>
         <v/>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="21">
         <f>F14-(H14-H13)</f>
         <v/>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="29">
         <f>MAX(0,H13+0.5*(D13+D14)*E14)</f>
         <v/>
       </c>
@@ -1880,7 +2052,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16">
+      <c r="A15" s="21">
         <f>Hydrogramme!A11</f>
         <v/>
       </c>
@@ -1888,7 +2060,7 @@
         <f>Hydrogramme!B11</f>
         <v/>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1896,19 +2068,19 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="21">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="21">
         <f>0.5*(B14+B15)*E15</f>
         <v/>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="21">
         <f>F15-(H15-H14)</f>
         <v/>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="29">
         <f>MAX(0,H14+0.5*(D14+D15)*E15)</f>
         <v/>
       </c>
@@ -1918,7 +2090,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16">
+      <c r="A16" s="21">
         <f>Hydrogramme!A12</f>
         <v/>
       </c>
@@ -1926,7 +2098,7 @@
         <f>Hydrogramme!B12</f>
         <v/>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1934,19 +2106,19 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="21">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="21">
         <f>0.5*(B15+B16)*E16</f>
         <v/>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="21">
         <f>F16-(H16-H15)</f>
         <v/>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="29">
         <f>MAX(0,H15+0.5*(D15+D16)*E16)</f>
         <v/>
       </c>
@@ -1956,7 +2128,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16">
+      <c r="A17" s="21">
         <f>Hydrogramme!A13</f>
         <v/>
       </c>
@@ -1964,7 +2136,7 @@
         <f>Hydrogramme!B13</f>
         <v/>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -1972,19 +2144,19 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="21">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="21">
         <f>0.5*(B16+B17)*E17</f>
         <v/>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="21">
         <f>F17-(H17-H16)</f>
         <v/>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="29">
         <f>MAX(0,H16+0.5*(D16+D17)*E17)</f>
         <v/>
       </c>
@@ -1994,7 +2166,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16">
+      <c r="A18" s="21">
         <f>Hydrogramme!A14</f>
         <v/>
       </c>
@@ -2002,7 +2174,7 @@
         <f>Hydrogramme!B14</f>
         <v/>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2010,19 +2182,19 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="21">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="21">
         <f>0.5*(B17+B18)*E18</f>
         <v/>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="21">
         <f>F18-(H18-H17)</f>
         <v/>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="29">
         <f>MAX(0,H17+0.5*(D17+D18)*E18)</f>
         <v/>
       </c>
@@ -2032,7 +2204,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16">
+      <c r="A19" s="21">
         <f>Hydrogramme!A15</f>
         <v/>
       </c>
@@ -2040,7 +2212,7 @@
         <f>Hydrogramme!B15</f>
         <v/>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2048,19 +2220,19 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="21">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="21">
         <f>0.5*(B18+B19)*E19</f>
         <v/>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="21">
         <f>F19-(H19-H18)</f>
         <v/>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="29">
         <f>MAX(0,H18+0.5*(D18+D19)*E19)</f>
         <v/>
       </c>
@@ -2070,7 +2242,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16">
+      <c r="A20" s="21">
         <f>Hydrogramme!A16</f>
         <v/>
       </c>
@@ -2078,7 +2250,7 @@
         <f>Hydrogramme!B16</f>
         <v/>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2086,19 +2258,19 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="21">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="21">
         <f>0.5*(B19+B20)*E20</f>
         <v/>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="21">
         <f>F20-(H20-H19)</f>
         <v/>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="29">
         <f>MAX(0,H19+0.5*(D19+D20)*E20)</f>
         <v/>
       </c>
@@ -2108,7 +2280,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16">
+      <c r="A21" s="21">
         <f>Hydrogramme!A17</f>
         <v/>
       </c>
@@ -2116,7 +2288,7 @@
         <f>Hydrogramme!B17</f>
         <v/>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2124,19 +2296,19 @@
         <f>B21-C21</f>
         <v/>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="21">
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="21">
         <f>0.5*(B20+B21)*E21</f>
         <v/>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="21">
         <f>F21-(H21-H20)</f>
         <v/>
       </c>
-      <c r="H21" s="24">
+      <c r="H21" s="29">
         <f>MAX(0,H20+0.5*(D20+D21)*E21)</f>
         <v/>
       </c>
@@ -2146,7 +2318,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16">
+      <c r="A22" s="21">
         <f>Hydrogramme!A18</f>
         <v/>
       </c>
@@ -2154,7 +2326,7 @@
         <f>Hydrogramme!B18</f>
         <v/>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="27">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2162,19 +2334,19 @@
         <f>B22-C22</f>
         <v/>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="21">
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="21">
         <f>0.5*(B21+B22)*E22</f>
         <v/>
       </c>
-      <c r="G22" s="16">
+      <c r="G22" s="21">
         <f>F22-(H22-H21)</f>
         <v/>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="29">
         <f>MAX(0,H21+0.5*(D21+D22)*E22)</f>
         <v/>
       </c>
@@ -2208,14 +2380,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="20" t="inlineStr">
         <is>
           <t>Méthode B — routage simplifié Qout = f(H) (orifice Ø900 plafonné à Qcap)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>H = V / Aire_bassin.  Qorifice = Cd·(πD²/4)·√(2gH).  Qout = MIN(Qcap, Qorifice) si V&gt;0; si V≈0, Qout = MIN(Qin, Qcap).  ΔV = (Qin_moyenne − Qout)·Δt.  Ajuster Cd, Aire, Qcap (jaune).</t>
         </is>
@@ -2228,7 +2400,7 @@
           <t>Cd</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="31" t="n">
         <v>0.62</v>
       </c>
     </row>
@@ -2238,7 +2410,7 @@
           <t>D (m)</t>
         </is>
       </c>
-      <c r="B6" s="26" t="n">
+      <c r="B6" s="31" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -2248,8 +2420,8 @@
           <t>Qcap (m³/s)</t>
         </is>
       </c>
-      <c r="B7" s="26">
-        <f>Parametres!B13</f>
+      <c r="B7" s="31">
+        <f>Parametres!B22</f>
         <v/>
       </c>
     </row>
@@ -2259,8 +2431,8 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B8" s="26">
-        <f>Parametres!B15</f>
+      <c r="B8" s="31">
+        <f>Parametres!B24</f>
         <v/>
       </c>
     </row>
@@ -2270,7 +2442,7 @@
           <t>Vmax_B (m³)</t>
         </is>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="26">
         <f>MAX(G14:G28)</f>
         <v/>
       </c>
@@ -2281,7 +2453,7 @@
           <t>Hmax_B (m)</t>
         </is>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="19">
         <f>IF(B8&gt;0,B9/B8,0)</f>
         <v/>
       </c>
@@ -2342,10 +2514,10 @@
         <f>MIN(B14,$B$7)</f>
         <v/>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="24" t="n">
+      <c r="G14" s="29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2370,11 +2542,11 @@
         <f>IF(G14&lt;=0.01,MIN(0.5*(B14+B15),$B$7),MIN($B$7,D15))</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="21">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="29">
         <f>MAX(0,G14+(0.5*(B14+B15)-E15)*F15)</f>
         <v/>
       </c>
@@ -2400,11 +2572,11 @@
         <f>IF(G15&lt;=0.01,MIN(0.5*(B15+B16),$B$7),MIN($B$7,D16))</f>
         <v/>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="21">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="29">
         <f>MAX(0,G15+(0.5*(B15+B16)-E16)*F16)</f>
         <v/>
       </c>
@@ -2430,11 +2602,11 @@
         <f>IF(G16&lt;=0.01,MIN(0.5*(B16+B17),$B$7),MIN($B$7,D17))</f>
         <v/>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="21">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="29">
         <f>MAX(0,G16+(0.5*(B16+B17)-E17)*F17)</f>
         <v/>
       </c>
@@ -2460,11 +2632,11 @@
         <f>IF(G17&lt;=0.01,MIN(0.5*(B17+B18),$B$7),MIN($B$7,D18))</f>
         <v/>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="21">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="29">
         <f>MAX(0,G17+(0.5*(B17+B18)-E18)*F18)</f>
         <v/>
       </c>
@@ -2490,11 +2662,11 @@
         <f>IF(G18&lt;=0.01,MIN(0.5*(B18+B19),$B$7),MIN($B$7,D19))</f>
         <v/>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="21">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="29">
         <f>MAX(0,G18+(0.5*(B18+B19)-E19)*F19)</f>
         <v/>
       </c>
@@ -2520,11 +2692,11 @@
         <f>IF(G19&lt;=0.01,MIN(0.5*(B19+B20),$B$7),MIN($B$7,D20))</f>
         <v/>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="21">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="29">
         <f>MAX(0,G19+(0.5*(B19+B20)-E20)*F20)</f>
         <v/>
       </c>
@@ -2550,11 +2722,11 @@
         <f>IF(G20&lt;=0.01,MIN(0.5*(B20+B21),$B$7),MIN($B$7,D21))</f>
         <v/>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="21">
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="G21" s="24">
+      <c r="G21" s="29">
         <f>MAX(0,G20+(0.5*(B20+B21)-E21)*F21)</f>
         <v/>
       </c>
@@ -2580,11 +2752,11 @@
         <f>IF(G21&lt;=0.01,MIN(0.5*(B21+B22),$B$7),MIN($B$7,D22))</f>
         <v/>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="21">
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="G22" s="24">
+      <c r="G22" s="29">
         <f>MAX(0,G21+(0.5*(B21+B22)-E22)*F22)</f>
         <v/>
       </c>
@@ -2610,11 +2782,11 @@
         <f>IF(G22&lt;=0.01,MIN(0.5*(B22+B23),$B$7),MIN($B$7,D23))</f>
         <v/>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="21">
         <f>(A23-A22)*60</f>
         <v/>
       </c>
-      <c r="G23" s="24">
+      <c r="G23" s="29">
         <f>MAX(0,G22+(0.5*(B22+B23)-E23)*F23)</f>
         <v/>
       </c>
@@ -2640,11 +2812,11 @@
         <f>IF(G23&lt;=0.01,MIN(0.5*(B23+B24),$B$7),MIN($B$7,D24))</f>
         <v/>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="21">
         <f>(A24-A23)*60</f>
         <v/>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="29">
         <f>MAX(0,G23+(0.5*(B23+B24)-E24)*F24)</f>
         <v/>
       </c>
@@ -2670,11 +2842,11 @@
         <f>IF(G24&lt;=0.01,MIN(0.5*(B24+B25),$B$7),MIN($B$7,D25))</f>
         <v/>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="21">
         <f>(A25-A24)*60</f>
         <v/>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="29">
         <f>MAX(0,G24+(0.5*(B24+B25)-E25)*F25)</f>
         <v/>
       </c>
@@ -2700,11 +2872,11 @@
         <f>IF(G25&lt;=0.01,MIN(0.5*(B25+B26),$B$7),MIN($B$7,D26))</f>
         <v/>
       </c>
-      <c r="F26" s="16">
+      <c r="F26" s="21">
         <f>(A26-A25)*60</f>
         <v/>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="29">
         <f>MAX(0,G25+(0.5*(B25+B26)-E26)*F26)</f>
         <v/>
       </c>
@@ -2730,11 +2902,11 @@
         <f>IF(G26&lt;=0.01,MIN(0.5*(B26+B27),$B$7),MIN($B$7,D27))</f>
         <v/>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="21">
         <f>(A27-A26)*60</f>
         <v/>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="29">
         <f>MAX(0,G26+(0.5*(B26+B27)-E27)*F27)</f>
         <v/>
       </c>
@@ -2760,11 +2932,11 @@
         <f>IF(G27&lt;=0.01,MIN(0.5*(B27+B28),$B$7),MIN($B$7,D28))</f>
         <v/>
       </c>
-      <c r="F28" s="16">
+      <c r="F28" s="21">
         <f>(A28-A27)*60</f>
         <v/>
       </c>
-      <c r="G28" s="24">
+      <c r="G28" s="29">
         <f>MAX(0,G27+(0.5*(B27+B28)-E28)*F28)</f>
         <v/>
       </c>
@@ -2783,14 +2955,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>
@@ -2816,66 +2988,73 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Méthode A: Qout = constante = capacité Ø900.</t>
+          <t>3. Capacité Ø900: Manning pleine section, n=0.013:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pendant chaque pas Δt:  ΔV = 0.5 * ((Qin−Qout)_i + (Qin−Qout)_{i+1}) * Δt</t>
+          <t xml:space="preserve">   Q = (1/n)·A·R^(2/3)·√S0  avec A=πD²/4, R=D/4, S0=(Zamont−Zaval)/L.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (excès signé: positif = remplissage, négatif = vidange).</t>
+          <t xml:space="preserve">   → Q_plein ≈ 1.668 m³/s (ancienne valeur bureau 1.77 ≈ même méthode).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   V(t) = max(0, V(t−Δt) + ΔV).   Vmax = max V(t).</t>
+          <t>4. Méthode A: Qout = constante = Q_plein (jaune Parametres).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4. Volume de dimensionnement ≈ Vmax × facteur de sécurité (Parametres).</t>
+          <t xml:space="preserve">   ΔV = 0.5 * ((Qin−Qout)_i + (Qin−Qout)_{i+1}) * Δt ; V = max(0, V+ΔV); Vmax = max V.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5. Méthode B: même bilan, mais Qout dépend de H = V/Aire (orifice plafonné).</t>
+          <t>5. Inlet vs outlet control: non tranché ici. L/D≈56 → frottement souvent plausible;</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6. Le Ø1200 à 4.93 m³/s est aval: il ne augmente pas la capacité de sortie de la rétention.</t>
+          <t xml:space="preserve">   Q_plein constant reste une 1re estimation prudente pour la rétention.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6. Méthode B: orifice Q=f(H) plafonné — illustration seulement.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Limites: Q=f(H) réelle du ponceau (entrée/sortie, longueur, n) préférable à Qcap constant;</t>
+          <t>7. Le Ø1200 (~4.93 m³/s Manning) est aval: n'augmente pas la sortie de la rétention.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>aire de bassin rarement constante — remplacer par une courbe V(H) de site si disponible.</t>
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pour une courbe Q=f(H) défendable: HY-8 / HEC-RAS (inlet + outlet control FHWA).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FHWA Q=f(H) curve for Ø900 and locate prior HY-8 Excel
Replace orifice Method B with HDS-5 inlet/outlet rating (Courbe_QH_900),
route storage from that curve, and include Ponceau_Capacite_Inlet_Outlet.xlsx
plus hydraulics module so the older capacity workbook is findable again.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -10,8 +10,10 @@
     <sheet name="Parametres" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Hydrogramme" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Calcul_A" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Calcul_B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Methode" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Courbe_QH_900" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Calcul_B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Fichiers_lies" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Methode" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="0.00000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +51,11 @@
       <b val="1"/>
       <color rgb="000F5C5C"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F5C5C"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -114,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,11 +154,12 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -600,6 +608,188 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Q gouvernant vs HW (Ø900)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Courbe_QH_900'!E9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Courbe_QH_900'!$A$10:$A$70</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Courbe_QH_900'!$E$10:$E$70</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Courbe_QH_900'!C9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Courbe_QH_900'!$A$10:$A$70</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Courbe_QH_900'!$C$10:$C$70</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Courbe_QH_900'!D9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Courbe_QH_900'!$A$10:$A$70</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Courbe_QH_900'!$D$10:$D$70</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>HW (m)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Q (m³/s)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -668,6 +858,33 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -965,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1412,14 +1629,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>• Méthode B: orifice Q=f(H) plafonné — illustration seulement; HY-8 / HEC-RAS donnerait une vraie courbe.</t>
+          <t>• Méthode B: Qout = f(H) depuis feuille Courbe_QH_900 (FHWA inlet+outlet).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>• Ø1200 Q_plein ≈ 4,93 m³/s avec le même n: cohérent, mais aval du Ø900 donc non limitant pour la rétention.</t>
+          <t>• Voir feuille Fichiers_lies pour les anciens Excel HY-8 / ponceau+fossé.</t>
         </is>
       </c>
     </row>
@@ -1427,6 +1644,22 @@
       <c r="A46" t="inlineStr">
         <is>
           <t>• Vérifier que le radier amont Ø900 (34.88) est bien le fond de la zone de rétention étudiée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Vmax_B courbe FHWA (m³)</t>
+        </is>
+      </c>
+      <c r="B47" s="18">
+        <f>Calcul_B!B7</f>
+        <v/>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Routage avec Q=f(H) — dépend de Aire_bassin (B24)</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2600,1469 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:G70"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Courbe de capacité Ø900 — Q = f(H) (FHWA HDS-5 inlet + outlet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Hypothèses: n=0.013, entrée=square_edge (Ke=0.5, inconnu → conservateur), TW=0 (exutoire libre), L=50.65 m, S0=0.00849. Q_gouvernant = min(Qinlet, Qoutlet). Sur ce tuyau long, le contrôle outlet domine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q_plein Manning (réf.)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>1.668006465155198</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>m³/s — section pleine, pente S0 seulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Entrée (hypothèse)</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>square_edge</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>square_edge | beveled | groove_headwall — régénérer le xlsx si changé</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TW (m au-dessus radier aval)</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0 = libre; si TW connu, régénérer avec build_retention_excel.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>HW (m)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Qinlet</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Qoutlet</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Q gouvernant</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>34.93</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>2.6023476558891</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.01002863087169758</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>0.01002863087169758</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>3.680275348968197</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0.04343590696816653</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0.04343590696816653</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>35.03</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>4.507398358957689</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.100717292251984</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.100717292251984</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B14" s="27" t="n">
+        <v>35.08000000000001</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>5.204695311778201</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0.1806404003717619</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.1806404003717619</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>35.13</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>5.819026259655258</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.281196921681494</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0.281196921681494</v>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>35.18</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>6.374423890256198</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.3998735226147597</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0.3998735226147597</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B17" s="27" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>6.88516472241445</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.5337705973187848</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>0.5337705973187848</v>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B18" s="27" t="n">
+        <v>35.28</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>7.360550697936395</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0.6796591745176915</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0.6796591745176915</v>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="B19" s="27" t="n">
+        <v>35.33000000000001</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>7.807042967667298</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0.8340032325775992</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>0.8340032325775992</v>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B20" s="27" t="n">
+        <v>35.38</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>8.229345856209648</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0.9929557763009054</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0.9929557763009054</v>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>35.43</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>8.63101074864505</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>1.152327657120539</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>1.152327657120539</v>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="B22" s="27" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>9.014796717915377</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>1.307519216598689</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>1.307519216598689</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="B23" s="27" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>9.382897909891664</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1.453389853296119</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>1.453389853296119</v>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="B24" s="27" t="n">
+        <v>35.58000000000001</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>9.737093329611298</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>1.584005967433924</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>1.584005967433924</v>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B25" s="27" t="n">
+        <v>35.63</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>10.07884913230039</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>1.692108486639005</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>1.692108486639005</v>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="B26" s="27" t="n">
+        <v>35.68</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>10.4093906235564</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>1.767776830483624</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>1.767776830483624</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="B27" s="27" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>10.72975425980928</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>1.793744127901133</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>1.793744127901133</v>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="B28" s="27" t="n">
+        <v>35.78</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>1.967842229450993</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>1.967842229450993</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="B29" s="27" t="n">
+        <v>35.83000000000001</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>2.004490484303977</v>
+      </c>
+      <c r="E29" s="15" t="n">
+        <v>2.004490484303977</v>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="27" t="n">
+        <v>35.88</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>2.040480620667524</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <v>2.040480620667524</v>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="B31" s="27" t="n">
+        <v>35.93</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>2.075846869346162</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <v>2.075846869346162</v>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="27" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="B32" s="27" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>2.11062059277095</v>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>2.11062059277095</v>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="B33" s="27" t="n">
+        <v>36.03</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>2.144830610627173</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>2.144830610627173</v>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="B34" s="27" t="n">
+        <v>36.08000000000001</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>2.178503479441304</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>2.178503479441304</v>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B35" s="27" t="n">
+        <v>36.13</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>2.211663733842106</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>2.211663733842106</v>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="B36" s="27" t="n">
+        <v>36.18</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>2.244334095727938</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <v>2.244334095727938</v>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="B37" s="27" t="n">
+        <v>36.23</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>2.276535656408983</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>2.276535656408983</v>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="B38" s="27" t="n">
+        <v>36.28</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>2.308288035873342</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <v>2.308288035873342</v>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="B39" s="27" t="n">
+        <v>36.33000000000001</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>2.339609522593578</v>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>2.339609522593578</v>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="27" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B40" s="27" t="n">
+        <v>36.38</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>2.370517196703092</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>2.370517196703092</v>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="27" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="B41" s="27" t="n">
+        <v>36.43</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>2.401027038898067</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>2.401027038898067</v>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="27" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="B42" s="27" t="n">
+        <v>36.48</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>2.431154027036164</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>2.431154027036164</v>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="B43" s="27" t="n">
+        <v>36.53</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>2.46091222208934</v>
+      </c>
+      <c r="E43" s="15" t="n">
+        <v>2.46091222208934</v>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="27" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="B44" s="27" t="n">
+        <v>36.58000000000001</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>2.490314844850592</v>
+      </c>
+      <c r="E44" s="15" t="n">
+        <v>2.490314844850592</v>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="B45" s="27" t="n">
+        <v>36.63</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>2.519374344581957</v>
+      </c>
+      <c r="E45" s="15" t="n">
+        <v>2.519374344581957</v>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="27" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="B46" s="27" t="n">
+        <v>36.68</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>2.548102460615016</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <v>2.548102460615016</v>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="27" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="B47" s="27" t="n">
+        <v>36.73</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>2.576510277768524</v>
+      </c>
+      <c r="E47" s="15" t="n">
+        <v>2.576510277768524</v>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="B48" s="27" t="n">
+        <v>36.78</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>2.604608276325131</v>
+      </c>
+      <c r="E48" s="15" t="n">
+        <v>2.604608276325131</v>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="B49" s="27" t="n">
+        <v>36.83000000000001</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>2.632406377206207</v>
+      </c>
+      <c r="E49" s="15" t="n">
+        <v>2.632406377206207</v>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="27" t="n">
+        <v>36.88</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>2.659913982896899</v>
+      </c>
+      <c r="E50" s="15" t="n">
+        <v>2.659913982896899</v>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="27" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="B51" s="27" t="n">
+        <v>36.93</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>2.687140014600091</v>
+      </c>
+      <c r="E51" s="15" t="n">
+        <v>2.687140014600091</v>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="27" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="B52" s="27" t="n">
+        <v>36.98</v>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>2.714092946035473</v>
+      </c>
+      <c r="E52" s="15" t="n">
+        <v>2.714092946035473</v>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="B53" s="27" t="n">
+        <v>37.03</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D53" s="5" t="n">
+        <v>2.740780834246703</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>2.740780834246703</v>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="27" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="B54" s="27" t="n">
+        <v>37.08000000000001</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>2.767211347734138</v>
+      </c>
+      <c r="E54" s="15" t="n">
+        <v>2.767211347734138</v>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="27" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="B55" s="27" t="n">
+        <v>37.13</v>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D55" s="5" t="n">
+        <v>2.79339179219155</v>
+      </c>
+      <c r="E55" s="15" t="n">
+        <v>2.79339179219155</v>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="27" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="B56" s="27" t="n">
+        <v>37.18</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>2.819329134091594</v>
+      </c>
+      <c r="E56" s="15" t="n">
+        <v>2.819329134091594</v>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="27" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="B57" s="27" t="n">
+        <v>37.23</v>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D57" s="5" t="n">
+        <v>2.845030022335827</v>
+      </c>
+      <c r="E57" s="15" t="n">
+        <v>2.845030022335827</v>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="27" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="B58" s="27" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="C58" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D58" s="5" t="n">
+        <v>2.870500808159916</v>
+      </c>
+      <c r="E58" s="15" t="n">
+        <v>2.870500808159916</v>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="27" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="B59" s="27" t="n">
+        <v>37.33000000000001</v>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D59" s="5" t="n">
+        <v>2.89574756346289</v>
+      </c>
+      <c r="E59" s="15" t="n">
+        <v>2.89574756346289</v>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B60" s="27" t="n">
+        <v>37.38</v>
+      </c>
+      <c r="C60" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>2.920776097710299</v>
+      </c>
+      <c r="E60" s="15" t="n">
+        <v>2.920776097710299</v>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="27" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="B61" s="27" t="n">
+        <v>37.43</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D61" s="5" t="n">
+        <v>2.945591973544595</v>
+      </c>
+      <c r="E61" s="15" t="n">
+        <v>2.945591973544595</v>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="27" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="B62" s="27" t="n">
+        <v>37.48</v>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D62" s="5" t="n">
+        <v>2.970200521221568</v>
+      </c>
+      <c r="E62" s="15" t="n">
+        <v>2.970200521221568</v>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="27" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="B63" s="27" t="n">
+        <v>37.53</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D63" s="5" t="n">
+        <v>2.994606851978972</v>
+      </c>
+      <c r="E63" s="15" t="n">
+        <v>2.994606851978972</v>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="27" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="B64" s="27" t="n">
+        <v>37.58000000000001</v>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D64" s="5" t="n">
+        <v>3.018815870432304</v>
+      </c>
+      <c r="E64" s="15" t="n">
+        <v>3.018815870432304</v>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="27" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="B65" s="27" t="n">
+        <v>37.63</v>
+      </c>
+      <c r="C65" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D65" s="5" t="n">
+        <v>3.042832286082899</v>
+      </c>
+      <c r="E65" s="15" t="n">
+        <v>3.042832286082899</v>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="B66" s="27" t="n">
+        <v>37.68</v>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D66" s="5" t="n">
+        <v>3.066660624014829</v>
+      </c>
+      <c r="E66" s="15" t="n">
+        <v>3.066660624014829</v>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="27" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="B67" s="27" t="n">
+        <v>37.73</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D67" s="5" t="n">
+        <v>3.090305234849392</v>
+      </c>
+      <c r="E67" s="15" t="n">
+        <v>3.090305234849392</v>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="27" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="B68" s="27" t="n">
+        <v>37.78</v>
+      </c>
+      <c r="C68" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D68" s="5" t="n">
+        <v>3.113770304019243</v>
+      </c>
+      <c r="E68" s="15" t="n">
+        <v>3.113770304019243</v>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="27" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="B69" s="27" t="n">
+        <v>37.83000000000001</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D69" s="5" t="n">
+        <v>3.137059860418132</v>
+      </c>
+      <c r="E69" s="15" t="n">
+        <v>3.137059860418132</v>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B70" s="27" t="n">
+        <v>37.88</v>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>10.76126608759892</v>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>3.160177784476874</v>
+      </c>
+      <c r="E70" s="15" t="n">
+        <v>3.160177784476874</v>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>outlet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2382,14 +4077,14 @@
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>Méthode B — routage simplifié Qout = f(H) (orifice Ø900 plafonné à Qcap)</t>
+          <t>Méthode B — routage avec Qout = f(H) depuis Courbe_QH_900 (FHWA)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
-        <is>
-          <t>H = V / Aire_bassin.  Qorifice = Cd·(πD²/4)·√(2gH).  Qout = MIN(Qcap, Qorifice) si V&gt;0; si V≈0, Qout = MIN(Qin, Qcap).  ΔV = (Qin_moyenne − Qout)·Δt.  Ajuster Cd, Aire, Qcap (jaune).</t>
+      <c r="A2" s="31" t="inlineStr">
+        <is>
+          <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy − Qout)·Δt.</t>
         </is>
       </c>
     </row>
@@ -2397,149 +4092,189 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cd</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="n">
-        <v>0.62</v>
+          <t>Aire (m²)</t>
+        </is>
+      </c>
+      <c r="B5" s="30">
+        <f>Parametres!B24</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>D (m)</t>
-        </is>
-      </c>
-      <c r="B6" s="31" t="n">
-        <v>0.9</v>
+          <t>Q_plein réf. (m³/s)</t>
+        </is>
+      </c>
+      <c r="B6" s="30">
+        <f>Parametres!B22</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Qcap (m³/s)</t>
-        </is>
-      </c>
-      <c r="B7" s="31">
-        <f>Parametres!B22</f>
+          <t>Vmax_B (m³)</t>
+        </is>
+      </c>
+      <c r="B7" s="26">
+        <f>MAX(G12:G26)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aire (m²)</t>
-        </is>
-      </c>
-      <c r="B8" s="31">
-        <f>Parametres!B24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Vmax_B (m³)</t>
-        </is>
-      </c>
-      <c r="B9" s="26">
-        <f>MAX(G14:G28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
           <t>Hmax_B (m)</t>
         </is>
       </c>
-      <c r="B10" s="19">
-        <f>IF(B8&gt;0,B9/B8,0)</f>
-        <v/>
+      <c r="B8" s="19">
+        <f>IF(B5&gt;0,B7/B5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>t (min)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Qin</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>H (m)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Q_courbe</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Qout</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Δt (s)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>V (m³)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <f>Hydrogramme!A4</f>
+        <v/>
+      </c>
+      <c r="B12" s="5">
+        <f>Hydrogramme!B4</f>
+        <v/>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5">
+        <f>MIN(B12,$B$6)</f>
+        <v/>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="29" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>t (min)</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Qin</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>H (m)</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Qorifice</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Qout</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Δt (s)</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>V (m³)</t>
-        </is>
+      <c r="A13" s="4">
+        <f>Hydrogramme!A5</f>
+        <v/>
+      </c>
+      <c r="B13" s="5">
+        <f>Hydrogramme!B5</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>IF($B$5&gt;0,G12/$B$5,0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>IF(C13&lt;=0,0,IF(C13&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1))+(C13-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>IF(G12&lt;=0.01,MIN(0.5*(B12+B13),$B$6),D13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="21">
+        <f>(A13-A12)*60</f>
+        <v/>
+      </c>
+      <c r="G13" s="29">
+        <f>MAX(0,G12+(0.5*(B12+B13)-E13)*F13)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4">
-        <f>Hydrogramme!A4</f>
+        <f>Hydrogramme!A6</f>
         <v/>
       </c>
       <c r="B14" s="5">
-        <f>Hydrogramme!B4</f>
-        <v/>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>0</v>
+        <f>Hydrogramme!B6</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>IF($B$5&gt;0,G13/$B$5,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="5">
+        <f>IF(C14&lt;=0,0,IF(C14&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1))+(C14-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <v/>
       </c>
       <c r="E14" s="5">
-        <f>MIN(B14,$B$7)</f>
-        <v/>
-      </c>
-      <c r="F14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="29" t="n">
-        <v>0</v>
+        <f>IF(G13&lt;=0.01,MIN(0.5*(B13+B14),$B$6),D14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>(A14-A13)*60</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>MAX(0,G13+(0.5*(B13+B14)-E14)*F14)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4">
-        <f>Hydrogramme!A5</f>
+        <f>Hydrogramme!A7</f>
         <v/>
       </c>
       <c r="B15" s="5">
-        <f>Hydrogramme!B5</f>
+        <f>Hydrogramme!B7</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>IF($B$8&gt;0,G14/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G14/$B$5,0)</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>IF(C15&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C15))</f>
+        <f>IF(C15&lt;=0,0,IF(C15&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1))+(C15-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>IF(G14&lt;=0.01,MIN(0.5*(B14+B15),$B$7),MIN($B$7,D15))</f>
+        <f>IF(G14&lt;=0.01,MIN(0.5*(B14+B15),$B$6),D15)</f>
         <v/>
       </c>
       <c r="F15" s="21">
@@ -2553,23 +4288,23 @@
     </row>
     <row r="16">
       <c r="A16" s="4">
-        <f>Hydrogramme!A6</f>
+        <f>Hydrogramme!A8</f>
         <v/>
       </c>
       <c r="B16" s="5">
-        <f>Hydrogramme!B6</f>
+        <f>Hydrogramme!B8</f>
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>IF($B$8&gt;0,G15/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G15/$B$5,0)</f>
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>IF(C16&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C16))</f>
+        <f>IF(C16&lt;=0,0,IF(C16&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1))+(C16-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E16" s="5">
-        <f>IF(G15&lt;=0.01,MIN(0.5*(B15+B16),$B$7),MIN($B$7,D16))</f>
+        <f>IF(G15&lt;=0.01,MIN(0.5*(B15+B16),$B$6),D16)</f>
         <v/>
       </c>
       <c r="F16" s="21">
@@ -2583,23 +4318,23 @@
     </row>
     <row r="17">
       <c r="A17" s="4">
-        <f>Hydrogramme!A7</f>
+        <f>Hydrogramme!A9</f>
         <v/>
       </c>
       <c r="B17" s="5">
-        <f>Hydrogramme!B7</f>
+        <f>Hydrogramme!B9</f>
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>IF($B$8&gt;0,G16/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G16/$B$5,0)</f>
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>IF(C17&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C17))</f>
+        <f>IF(C17&lt;=0,0,IF(C17&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1))+(C17-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E17" s="5">
-        <f>IF(G16&lt;=0.01,MIN(0.5*(B16+B17),$B$7),MIN($B$7,D17))</f>
+        <f>IF(G16&lt;=0.01,MIN(0.5*(B16+B17),$B$6),D17)</f>
         <v/>
       </c>
       <c r="F17" s="21">
@@ -2613,23 +4348,23 @@
     </row>
     <row r="18">
       <c r="A18" s="4">
-        <f>Hydrogramme!A8</f>
+        <f>Hydrogramme!A10</f>
         <v/>
       </c>
       <c r="B18" s="5">
-        <f>Hydrogramme!B8</f>
+        <f>Hydrogramme!B10</f>
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>IF($B$8&gt;0,G17/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G17/$B$5,0)</f>
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>IF(C18&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C18))</f>
+        <f>IF(C18&lt;=0,0,IF(C18&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1))+(C18-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E18" s="5">
-        <f>IF(G17&lt;=0.01,MIN(0.5*(B17+B18),$B$7),MIN($B$7,D18))</f>
+        <f>IF(G17&lt;=0.01,MIN(0.5*(B17+B18),$B$6),D18)</f>
         <v/>
       </c>
       <c r="F18" s="21">
@@ -2643,23 +4378,23 @@
     </row>
     <row r="19">
       <c r="A19" s="4">
-        <f>Hydrogramme!A9</f>
+        <f>Hydrogramme!A11</f>
         <v/>
       </c>
       <c r="B19" s="5">
-        <f>Hydrogramme!B9</f>
+        <f>Hydrogramme!B11</f>
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>IF($B$8&gt;0,G18/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G18/$B$5,0)</f>
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>IF(C19&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C19))</f>
+        <f>IF(C19&lt;=0,0,IF(C19&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1))+(C19-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E19" s="5">
-        <f>IF(G18&lt;=0.01,MIN(0.5*(B18+B19),$B$7),MIN($B$7,D19))</f>
+        <f>IF(G18&lt;=0.01,MIN(0.5*(B18+B19),$B$6),D19)</f>
         <v/>
       </c>
       <c r="F19" s="21">
@@ -2673,23 +4408,23 @@
     </row>
     <row r="20">
       <c r="A20" s="4">
-        <f>Hydrogramme!A10</f>
+        <f>Hydrogramme!A12</f>
         <v/>
       </c>
       <c r="B20" s="5">
-        <f>Hydrogramme!B10</f>
+        <f>Hydrogramme!B12</f>
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>IF($B$8&gt;0,G19/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G19/$B$5,0)</f>
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>IF(C20&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C20))</f>
+        <f>IF(C20&lt;=0,0,IF(C20&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1))+(C20-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E20" s="5">
-        <f>IF(G19&lt;=0.01,MIN(0.5*(B19+B20),$B$7),MIN($B$7,D20))</f>
+        <f>IF(G19&lt;=0.01,MIN(0.5*(B19+B20),$B$6),D20)</f>
         <v/>
       </c>
       <c r="F20" s="21">
@@ -2703,23 +4438,23 @@
     </row>
     <row r="21">
       <c r="A21" s="4">
-        <f>Hydrogramme!A11</f>
+        <f>Hydrogramme!A13</f>
         <v/>
       </c>
       <c r="B21" s="5">
-        <f>Hydrogramme!B11</f>
+        <f>Hydrogramme!B13</f>
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>IF($B$8&gt;0,G20/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G20/$B$5,0)</f>
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>IF(C21&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C21))</f>
+        <f>IF(C21&lt;=0,0,IF(C21&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1))+(C21-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E21" s="5">
-        <f>IF(G20&lt;=0.01,MIN(0.5*(B20+B21),$B$7),MIN($B$7,D21))</f>
+        <f>IF(G20&lt;=0.01,MIN(0.5*(B20+B21),$B$6),D21)</f>
         <v/>
       </c>
       <c r="F21" s="21">
@@ -2733,23 +4468,23 @@
     </row>
     <row r="22">
       <c r="A22" s="4">
-        <f>Hydrogramme!A12</f>
+        <f>Hydrogramme!A14</f>
         <v/>
       </c>
       <c r="B22" s="5">
-        <f>Hydrogramme!B12</f>
+        <f>Hydrogramme!B14</f>
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>IF($B$8&gt;0,G21/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G21/$B$5,0)</f>
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>IF(C22&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C22))</f>
+        <f>IF(C22&lt;=0,0,IF(C22&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1))+(C22-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E22" s="5">
-        <f>IF(G21&lt;=0.01,MIN(0.5*(B21+B22),$B$7),MIN($B$7,D22))</f>
+        <f>IF(G21&lt;=0.01,MIN(0.5*(B21+B22),$B$6),D22)</f>
         <v/>
       </c>
       <c r="F22" s="21">
@@ -2763,23 +4498,23 @@
     </row>
     <row r="23">
       <c r="A23" s="4">
-        <f>Hydrogramme!A13</f>
+        <f>Hydrogramme!A15</f>
         <v/>
       </c>
       <c r="B23" s="5">
-        <f>Hydrogramme!B13</f>
+        <f>Hydrogramme!B15</f>
         <v/>
       </c>
       <c r="C23" s="5">
-        <f>IF($B$8&gt;0,G22/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G22/$B$5,0)</f>
         <v/>
       </c>
       <c r="D23" s="5">
-        <f>IF(C23&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C23))</f>
+        <f>IF(C23&lt;=0,0,IF(C23&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1))+(C23-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E23" s="5">
-        <f>IF(G22&lt;=0.01,MIN(0.5*(B22+B23),$B$7),MIN($B$7,D23))</f>
+        <f>IF(G22&lt;=0.01,MIN(0.5*(B22+B23),$B$6),D23)</f>
         <v/>
       </c>
       <c r="F23" s="21">
@@ -2793,23 +4528,23 @@
     </row>
     <row r="24">
       <c r="A24" s="4">
-        <f>Hydrogramme!A14</f>
+        <f>Hydrogramme!A16</f>
         <v/>
       </c>
       <c r="B24" s="5">
-        <f>Hydrogramme!B14</f>
+        <f>Hydrogramme!B16</f>
         <v/>
       </c>
       <c r="C24" s="5">
-        <f>IF($B$8&gt;0,G23/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G23/$B$5,0)</f>
         <v/>
       </c>
       <c r="D24" s="5">
-        <f>IF(C24&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C24))</f>
+        <f>IF(C24&lt;=0,0,IF(C24&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1))+(C24-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E24" s="5">
-        <f>IF(G23&lt;=0.01,MIN(0.5*(B23+B24),$B$7),MIN($B$7,D24))</f>
+        <f>IF(G23&lt;=0.01,MIN(0.5*(B23+B24),$B$6),D24)</f>
         <v/>
       </c>
       <c r="F24" s="21">
@@ -2823,23 +4558,23 @@
     </row>
     <row r="25">
       <c r="A25" s="4">
-        <f>Hydrogramme!A15</f>
+        <f>Hydrogramme!A17</f>
         <v/>
       </c>
       <c r="B25" s="5">
-        <f>Hydrogramme!B15</f>
+        <f>Hydrogramme!B17</f>
         <v/>
       </c>
       <c r="C25" s="5">
-        <f>IF($B$8&gt;0,G24/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G24/$B$5,0)</f>
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>IF(C25&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C25))</f>
+        <f>IF(C25&lt;=0,0,IF(C25&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1))+(C25-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E25" s="5">
-        <f>IF(G24&lt;=0.01,MIN(0.5*(B24+B25),$B$7),MIN($B$7,D25))</f>
+        <f>IF(G24&lt;=0.01,MIN(0.5*(B24+B25),$B$6),D25)</f>
         <v/>
       </c>
       <c r="F25" s="21">
@@ -2853,23 +4588,23 @@
     </row>
     <row r="26">
       <c r="A26" s="4">
-        <f>Hydrogramme!A16</f>
+        <f>Hydrogramme!A18</f>
         <v/>
       </c>
       <c r="B26" s="5">
-        <f>Hydrogramme!B16</f>
+        <f>Hydrogramme!B18</f>
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>IF($B$8&gt;0,G25/$B$8,0)</f>
+        <f>IF($B$5&gt;0,G25/$B$5,0)</f>
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>IF(C26&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C26))</f>
+        <f>IF(C26&lt;=0,0,IF(C26&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1))+(C26-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)))))</f>
         <v/>
       </c>
       <c r="E26" s="5">
-        <f>IF(G25&lt;=0.01,MIN(0.5*(B25+B26),$B$7),MIN($B$7,D26))</f>
+        <f>IF(G25&lt;=0.01,MIN(0.5*(B25+B26),$B$6),D26)</f>
         <v/>
       </c>
       <c r="F26" s="21">
@@ -2881,88 +4616,161 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4">
-        <f>Hydrogramme!A17</f>
-        <v/>
-      </c>
-      <c r="B27" s="5">
-        <f>Hydrogramme!B17</f>
-        <v/>
-      </c>
-      <c r="C27" s="5">
-        <f>IF($B$8&gt;0,G26/$B$8,0)</f>
-        <v/>
-      </c>
-      <c r="D27" s="5">
-        <f>IF(C27&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C27))</f>
-        <v/>
-      </c>
-      <c r="E27" s="5">
-        <f>IF(G26&lt;=0.01,MIN(0.5*(B26+B27),$B$7),MIN($B$7,D27))</f>
-        <v/>
-      </c>
-      <c r="F27" s="21">
-        <f>(A27-A26)*60</f>
-        <v/>
-      </c>
-      <c r="G27" s="29">
-        <f>MAX(0,G26+(0.5*(B26+B27)-E27)*F27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4">
-        <f>Hydrogramme!A18</f>
-        <v/>
-      </c>
-      <c r="B28" s="5">
-        <f>Hydrogramme!B18</f>
-        <v/>
-      </c>
-      <c r="C28" s="5">
-        <f>IF($B$8&gt;0,G27/$B$8,0)</f>
-        <v/>
-      </c>
-      <c r="D28" s="5">
-        <f>IF(C28&lt;=0,0,$B$5*(PI()*($B$6^2)/4)*SQRT(2*9.81*C28))</f>
-        <v/>
-      </c>
-      <c r="E28" s="5">
-        <f>IF(G27&lt;=0.01,MIN(0.5*(B27+B28),$B$7),MIN($B$7,D28))</f>
-        <v/>
-      </c>
-      <c r="F28" s="21">
-        <f>(A28-A27)*60</f>
-        <v/>
-      </c>
-      <c r="G28" s="29">
-        <f>MAX(0,G27+(0.5*(B27+B28)-E28)*F28)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:I3"/>
+    <mergeCell ref="A2:G3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>Où sont les fichiers HY-8 / capacité ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ce classeur (rétention Ø900) :</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Courbe Q=f(H) FHWA pour CE Ø900 : feuille Courbe_QH_900 (ci-dessus).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ancien Excel « type HY-8 / inlet-outlet » (autre projet / Ste-Thérèse) :</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/drainage-design/Ponceau_Capacite_Inlet_Outlet.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Branche git: cursor/culvert-excel-capacity-model-d87f</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Modèle composé ponceau Ø1050 + fossé (FHWA + remblai) — PAS le Ø900 de rétention :</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Branche git: cursor/ponceau-fosse-hydraulic-model-d87f</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HEC-RAS : pas de projet .ras/.hdf pour ce Ø900. Un DEM Ste-Thérèse est dans</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/hec-ras-data/ (données topo seulement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Donc: on n'avait pas perdu un HY-8 pour ce bassin Ø900 — on avait des outils</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>similaires pour d'autres sites. La courbe de CE classeur remplace ça pour le Ø900.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>
@@ -2988,73 +4796,59 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Capacité Ø900: Manning pleine section, n=0.013:</t>
+          <t>3. Capacité Ø900 — deux niveaux:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Q = (1/n)·A·R^(2/3)·√S0  avec A=πD²/4, R=D/4, S0=(Zamont−Zaval)/L.</t>
+          <t xml:space="preserve">   A) Q_plein Manning (n=0.013) ≈ 1.668 m³/s → Méthode A (constant).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   → Q_plein ≈ 1.668 m³/s (ancienne valeur bureau 1.77 ≈ même méthode).</t>
+          <t xml:space="preserve">   B) Courbe Q=f(H) FHWA HDS-5 (inlet + outlet) → feuille Courbe_QH_900 + Calcul_B.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4. Méthode A: Qout = constante = Q_plein (jaune Parametres).</t>
+          <t>4. Méthode A: Qout = constante = Q_plein (jaune Parametres). Bon pour 1re estimation.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ΔV = 0.5 * ((Qin−Qout)_i + (Qin−Qout)_{i+1}) * Δt ; V = max(0, V+ΔV); Vmax = max V.</t>
+          <t>5. Méthode B: Qout lu sur la courbe selon H=V/Aire (charge amont).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5. Inlet vs outlet control: non tranché ici. L/D≈56 → frottement souvent plausible;</t>
+          <t>6. Sur ce Ø900 (L/D≈56), le calcul FHWA indique surtout un contrôle outlet.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Q_plein constant reste une 1re estimation prudente pour la rétention.</t>
+          <t>7. Le Ø1200 est aval: n'augmente pas la sortie de la rétention.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>6. Méthode B: orifice Q=f(H) plafonné — illustration seulement.</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7. Le Ø1200 (~4.93 m³/s Manning) est aval: n'augmente pas la sortie de la rétention.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Pour une courbe Q=f(H) défendable: HY-8 / HEC-RAS (inlet + outlet control FHWA).</t>
+          <t>Fichiers liés / anciens Excel: voir feuille Fichiers_lies.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Ø900 FHWA capacity curve live Excel formulas
Courbe_QH_900 now recalculates Qinlet/Qoutlet/Q from yellow inputs
(n, D, L, inverts, entrance type, TW) without rerunning Python.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -121,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,10 +155,16 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -620,7 +627,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Q gouvernant vs HW (Ø900)</a:t>
+              <a:t>Q gouvernant vs HW (Ø900) — live</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -634,7 +641,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Courbe_QH_900'!E9</f>
+              <f>'Courbe_QH_900'!E23</f>
             </strRef>
           </tx>
           <spPr>
@@ -652,12 +659,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Courbe_QH_900'!$A$10:$A$70</f>
+              <f>'Courbe_QH_900'!$A$24:$A$84</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Courbe_QH_900'!$E$10:$E$70</f>
+              <f>'Courbe_QH_900'!$E$24:$E$84</f>
             </numRef>
           </val>
         </ser>
@@ -666,7 +673,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Courbe_QH_900'!C9</f>
+              <f>'Courbe_QH_900'!C23</f>
             </strRef>
           </tx>
           <spPr>
@@ -684,12 +691,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Courbe_QH_900'!$A$10:$A$70</f>
+              <f>'Courbe_QH_900'!$A$24:$A$84</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Courbe_QH_900'!$C$10:$C$70</f>
+              <f>'Courbe_QH_900'!$C$24:$C$84</f>
             </numRef>
           </val>
         </ser>
@@ -698,7 +705,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Courbe_QH_900'!D9</f>
+              <f>'Courbe_QH_900'!D23</f>
             </strRef>
           </tx>
           <spPr>
@@ -716,12 +723,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Courbe_QH_900'!$A$10:$A$70</f>
+              <f>'Courbe_QH_900'!$A$24:$A$84</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Courbe_QH_900'!$D$10:$D$70</f>
+              <f>'Courbe_QH_900'!$D$24:$D$84</f>
             </numRef>
           </val>
         </ser>
@@ -870,7 +877,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>4</row>
       <rowOff>0</rowOff>
@@ -2600,1451 +2607,1868 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>Courbe de capacité Ø900 — Q = f(H) (FHWA HDS-5 inlet + outlet)</t>
+          <t>Courbe de capacité Ø900 — Q = f(H) (FHWA HDS-5 inlet + outlet) — FORMULES LIVE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Hypothèses: n=0.013, entrée=square_edge (Ke=0.5, inconnu → conservateur), TW=0 (exutoire libre), L=50.65 m, S0=0.00849. Q_gouvernant = min(Qinlet, Qoutlet). Sur ce tuyau long, le contrôle outlet domine.</t>
+          <t>Changez les cellules JAUNES (n, D, L, radiers, entrée, TW) : toute la table se recalcule. Q_gouvernant = MIN(Qinlet, Qoutlet). Pas besoin de relancer Python.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Q_plein Manning (réf.)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n">
-        <v>1.668006465155198</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>m³/s — section pleine, pente S0 seulement</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Paramètres Ø900 (jaune = éditable)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Coeffs HDS-5 (table)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Entrée (hypothèse)</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>square_edge</t>
-        </is>
+          <t>n Manning (-)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>0.013</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>square_edge | beveled | groove_headwall — régénérer le xlsx si changé</t>
+          <t>béton typ. 0.012–0.015</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
+          <t>entrée</t>
+        </is>
+      </c>
+      <c r="F6" s="30" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="G6" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H6" s="30" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="I6" s="30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J6" s="30" t="inlineStr">
+        <is>
+          <t>Ke</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TW (m au-dessus radier aval)</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="n">
+          <t>D (m)</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>square_edge</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0.0098</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0.0398</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L (m)</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>50.65</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>beveled</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Radier amont Zin (m)</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>groove_headwall</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.0078</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Radier aval Zout (m)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>34.45</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>S0 = (Zin-Zout)/L</t>
+        </is>
+      </c>
+      <c r="B11" s="31">
+        <f>(B9-B10)/B8</f>
+        <v/>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ASCII minus; LibreOffice FR: OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TW (m au-dessus Zout)</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0 = libre; si TW connu, régénérer avec build_retention_excel.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0 = exutoire libre</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Entrée (texte exact)</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>square_edge</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>square_edge | beveled | groove_headwall</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q_plein Manning (réf.)</t>
+        </is>
+      </c>
+      <c r="B15" s="33">
+        <f>(1/B6)*(PI()*B7^2/4)*((B7/4)^(2/3))*SQRT(B11)</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>m³/s — se met à jour avec n, D, S0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>K (lu)</t>
+        </is>
+      </c>
+      <c r="B17" s="34">
+        <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,2,FALSE),0.0098)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>M (lu)</t>
+        </is>
+      </c>
+      <c r="B18" s="34">
+        <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,3,FALSE),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>c (lu)</t>
+        </is>
+      </c>
+      <c r="B19" s="34">
+        <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,4,FALSE),0.0398)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Y (lu)</t>
+        </is>
+      </c>
+      <c r="B20" s="34">
+        <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,5,FALSE),0.67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ke (lu)</t>
+        </is>
+      </c>
+      <c r="B21" s="34">
+        <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,6,FALSE),0.5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>HW (m)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>WSE (m)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Qinlet</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Qoutlet</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Q gouvernant</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Contrôle</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="B10" s="27" t="n">
-        <v>34.88</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="27" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="B11" s="27" t="n">
-        <v>34.93</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>2.6023476558891</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>0.01002863087169758</v>
-      </c>
-      <c r="E11" s="15" t="n">
-        <v>0.01002863087169758</v>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="B12" s="27" t="n">
-        <v>34.98</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>3.680275348968197</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>0.04343590696816653</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>0.04343590696816653</v>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="27" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="B13" s="27" t="n">
-        <v>35.03</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>4.507398358957689</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>0.100717292251984</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>0.100717292251984</v>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="27" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="B14" s="27" t="n">
-        <v>35.08000000000001</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>5.204695311778201</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>0.1806404003717619</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <v>0.1806404003717619</v>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="27" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="B15" s="27" t="n">
-        <v>35.13</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>5.819026259655258</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>0.281196921681494</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>0.281196921681494</v>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="27" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B16" s="27" t="n">
-        <v>35.18</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>6.374423890256198</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>0.3998735226147597</v>
-      </c>
-      <c r="E16" s="15" t="n">
-        <v>0.3998735226147597</v>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="27" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="B17" s="27" t="n">
-        <v>35.23</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>6.88516472241445</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>0.5337705973187848</v>
-      </c>
-      <c r="E17" s="15" t="n">
-        <v>0.5337705973187848</v>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="27" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="B18" s="27" t="n">
-        <v>35.28</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>7.360550697936395</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>0.6796591745176915</v>
-      </c>
-      <c r="E18" s="15" t="n">
-        <v>0.6796591745176915</v>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="27" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="B19" s="27" t="n">
-        <v>35.33000000000001</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>7.807042967667298</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>0.8340032325775992</v>
-      </c>
-      <c r="E19" s="15" t="n">
-        <v>0.8340032325775992</v>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="27" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B20" s="27" t="n">
-        <v>35.38</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>8.229345856209648</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>0.9929557763009054</v>
-      </c>
-      <c r="E20" s="15" t="n">
-        <v>0.9929557763009054</v>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="27" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="B21" s="27" t="n">
-        <v>35.43</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>8.63101074864505</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>1.152327657120539</v>
-      </c>
-      <c r="E21" s="15" t="n">
-        <v>1.152327657120539</v>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="27" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="B22" s="27" t="n">
-        <v>35.48</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>9.014796717915377</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>1.307519216598689</v>
-      </c>
-      <c r="E22" s="15" t="n">
-        <v>1.307519216598689</v>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="27" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="B23" s="27" t="n">
-        <v>35.53</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>9.382897909891664</v>
-      </c>
-      <c r="D23" s="5" t="n">
-        <v>1.453389853296119</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <v>1.453389853296119</v>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="27" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="B24" s="27" t="n">
-        <v>35.58000000000001</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>9.737093329611298</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>1.584005967433924</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>1.584005967433924</v>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="B24" s="27">
+        <f>$B$9+A24</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>IF(A24&lt;=0,0,IF(A24&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A24/($B$17*$B$7))^(1/$B$18)),IF(A24&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A24/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A24/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A24/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A24/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A24/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D24" s="5">
+        <f>IF(A24&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A24/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A24-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A24-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E24" s="15">
+        <f>MIN(C24,D24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="4">
+        <f>IF(A24&lt;=0,"—",IF(C24&lt;=D24,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="27" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="B25" s="27" t="n">
-        <v>35.63</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>10.07884913230039</v>
-      </c>
-      <c r="D25" s="5" t="n">
-        <v>1.692108486639005</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>1.692108486639005</v>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.05</v>
+      </c>
+      <c r="B25" s="27">
+        <f>$B$9+A25</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>IF(A25&lt;=0,0,IF(A25&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A25/($B$17*$B$7))^(1/$B$18)),IF(A25&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A25/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A25/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A25/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A25/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A25/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D25" s="5">
+        <f>IF(A25&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A25/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A25-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A25-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E25" s="15">
+        <f>MIN(C25,D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="4">
+        <f>IF(A25&lt;=0,"—",IF(C25&lt;=D25,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="27" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="B26" s="27" t="n">
-        <v>35.68</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>10.4093906235564</v>
-      </c>
-      <c r="D26" s="5" t="n">
-        <v>1.767776830483624</v>
-      </c>
-      <c r="E26" s="15" t="n">
-        <v>1.767776830483624</v>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.1</v>
+      </c>
+      <c r="B26" s="27">
+        <f>$B$9+A26</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>IF(A26&lt;=0,0,IF(A26&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A26/($B$17*$B$7))^(1/$B$18)),IF(A26&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A26/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A26/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A26/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A26/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A26/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D26" s="5">
+        <f>IF(A26&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A26/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A26-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A26-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E26" s="15">
+        <f>MIN(C26,D26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="4">
+        <f>IF(A26&lt;=0,"—",IF(C26&lt;=D26,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="27" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="B27" s="27" t="n">
-        <v>35.73</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>10.72975425980928</v>
-      </c>
-      <c r="D27" s="5" t="n">
-        <v>1.793744127901133</v>
-      </c>
-      <c r="E27" s="15" t="n">
-        <v>1.793744127901133</v>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.15</v>
+      </c>
+      <c r="B27" s="27">
+        <f>$B$9+A27</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>IF(A27&lt;=0,0,IF(A27&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A27/($B$17*$B$7))^(1/$B$18)),IF(A27&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A27/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A27/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A27/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A27/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A27/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D27" s="5">
+        <f>IF(A27&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A27/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A27-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A27-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E27" s="15">
+        <f>MIN(C27,D27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="4">
+        <f>IF(A27&lt;=0,"—",IF(C27&lt;=D27,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="27" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="B28" s="27" t="n">
-        <v>35.78</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>1.967842229450993</v>
-      </c>
-      <c r="E28" s="15" t="n">
-        <v>1.967842229450993</v>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.2</v>
+      </c>
+      <c r="B28" s="27">
+        <f>$B$9+A28</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>IF(A28&lt;=0,0,IF(A28&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A28/($B$17*$B$7))^(1/$B$18)),IF(A28&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A28/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A28/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A28/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A28/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A28/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D28" s="5">
+        <f>IF(A28&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A28/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A28-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A28-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E28" s="15">
+        <f>MIN(C28,D28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="4">
+        <f>IF(A28&lt;=0,"—",IF(C28&lt;=D28,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="27" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="B29" s="27" t="n">
-        <v>35.83000000000001</v>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>2.004490484303977</v>
-      </c>
-      <c r="E29" s="15" t="n">
-        <v>2.004490484303977</v>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.25</v>
+      </c>
+      <c r="B29" s="27">
+        <f>$B$9+A29</f>
+        <v/>
+      </c>
+      <c r="C29" s="5">
+        <f>IF(A29&lt;=0,0,IF(A29&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A29/($B$17*$B$7))^(1/$B$18)),IF(A29&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A29/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A29/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A29/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A29/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A29/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D29" s="5">
+        <f>IF(A29&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A29/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A29-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A29-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E29" s="15">
+        <f>MIN(C29,D29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="4">
+        <f>IF(A29&lt;=0,"—",IF(C29&lt;=D29,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" s="27" t="n">
-        <v>35.88</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D30" s="5" t="n">
-        <v>2.040480620667524</v>
-      </c>
-      <c r="E30" s="15" t="n">
-        <v>2.040480620667524</v>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.3</v>
+      </c>
+      <c r="B30" s="27">
+        <f>$B$9+A30</f>
+        <v/>
+      </c>
+      <c r="C30" s="5">
+        <f>IF(A30&lt;=0,0,IF(A30&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A30/($B$17*$B$7))^(1/$B$18)),IF(A30&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A30/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A30/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A30/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A30/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A30/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D30" s="5">
+        <f>IF(A30&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A30/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A30-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A30-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E30" s="15">
+        <f>MIN(C30,D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="4">
+        <f>IF(A30&lt;=0,"—",IF(C30&lt;=D30,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="27" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="B31" s="27" t="n">
-        <v>35.93</v>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D31" s="5" t="n">
-        <v>2.075846869346162</v>
-      </c>
-      <c r="E31" s="15" t="n">
-        <v>2.075846869346162</v>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.35</v>
+      </c>
+      <c r="B31" s="27">
+        <f>$B$9+A31</f>
+        <v/>
+      </c>
+      <c r="C31" s="5">
+        <f>IF(A31&lt;=0,0,IF(A31&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A31/($B$17*$B$7))^(1/$B$18)),IF(A31&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A31/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A31/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A31/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A31/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A31/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D31" s="5">
+        <f>IF(A31&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A31/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A31-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A31-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E31" s="15">
+        <f>MIN(C31,D31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="4">
+        <f>IF(A31&lt;=0,"—",IF(C31&lt;=D31,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="27" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="B32" s="27" t="n">
-        <v>35.98</v>
-      </c>
-      <c r="C32" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D32" s="5" t="n">
-        <v>2.11062059277095</v>
-      </c>
-      <c r="E32" s="15" t="n">
-        <v>2.11062059277095</v>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.4</v>
+      </c>
+      <c r="B32" s="27">
+        <f>$B$9+A32</f>
+        <v/>
+      </c>
+      <c r="C32" s="5">
+        <f>IF(A32&lt;=0,0,IF(A32&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A32/($B$17*$B$7))^(1/$B$18)),IF(A32&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A32/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A32/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A32/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A32/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A32/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D32" s="5">
+        <f>IF(A32&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A32/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A32-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A32-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E32" s="15">
+        <f>MIN(C32,D32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="4">
+        <f>IF(A32&lt;=0,"—",IF(C32&lt;=D32,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="27" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="B33" s="27" t="n">
-        <v>36.03</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D33" s="5" t="n">
-        <v>2.144830610627173</v>
-      </c>
-      <c r="E33" s="15" t="n">
-        <v>2.144830610627173</v>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.45</v>
+      </c>
+      <c r="B33" s="27">
+        <f>$B$9+A33</f>
+        <v/>
+      </c>
+      <c r="C33" s="5">
+        <f>IF(A33&lt;=0,0,IF(A33&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A33/($B$17*$B$7))^(1/$B$18)),IF(A33&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A33/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A33/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A33/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A33/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A33/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D33" s="5">
+        <f>IF(A33&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A33/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A33-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A33-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E33" s="15">
+        <f>MIN(C33,D33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="4">
+        <f>IF(A33&lt;=0,"—",IF(C33&lt;=D33,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="27" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="B34" s="27" t="n">
-        <v>36.08000000000001</v>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D34" s="5" t="n">
-        <v>2.178503479441304</v>
-      </c>
-      <c r="E34" s="15" t="n">
-        <v>2.178503479441304</v>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.5</v>
+      </c>
+      <c r="B34" s="27">
+        <f>$B$9+A34</f>
+        <v/>
+      </c>
+      <c r="C34" s="5">
+        <f>IF(A34&lt;=0,0,IF(A34&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A34/($B$17*$B$7))^(1/$B$18)),IF(A34&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A34/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A34/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A34/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A34/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A34/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D34" s="5">
+        <f>IF(A34&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A34/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A34-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A34-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E34" s="15">
+        <f>MIN(C34,D34)</f>
+        <v/>
+      </c>
+      <c r="F34" s="4">
+        <f>IF(A34&lt;=0,"—",IF(C34&lt;=D34,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="27" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="B35" s="27" t="n">
-        <v>36.13</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D35" s="5" t="n">
-        <v>2.211663733842106</v>
-      </c>
-      <c r="E35" s="15" t="n">
-        <v>2.211663733842106</v>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.55</v>
+      </c>
+      <c r="B35" s="27">
+        <f>$B$9+A35</f>
+        <v/>
+      </c>
+      <c r="C35" s="5">
+        <f>IF(A35&lt;=0,0,IF(A35&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A35/($B$17*$B$7))^(1/$B$18)),IF(A35&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A35/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A35/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A35/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A35/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A35/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D35" s="5">
+        <f>IF(A35&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A35/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A35-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A35-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E35" s="15">
+        <f>MIN(C35,D35)</f>
+        <v/>
+      </c>
+      <c r="F35" s="4">
+        <f>IF(A35&lt;=0,"—",IF(C35&lt;=D35,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="27" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="B36" s="27" t="n">
-        <v>36.18</v>
-      </c>
-      <c r="C36" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D36" s="5" t="n">
-        <v>2.244334095727938</v>
-      </c>
-      <c r="E36" s="15" t="n">
-        <v>2.244334095727938</v>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.6</v>
+      </c>
+      <c r="B36" s="27">
+        <f>$B$9+A36</f>
+        <v/>
+      </c>
+      <c r="C36" s="5">
+        <f>IF(A36&lt;=0,0,IF(A36&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A36/($B$17*$B$7))^(1/$B$18)),IF(A36&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A36/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A36/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A36/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A36/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A36/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D36" s="5">
+        <f>IF(A36&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A36/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A36-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A36-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E36" s="15">
+        <f>MIN(C36,D36)</f>
+        <v/>
+      </c>
+      <c r="F36" s="4">
+        <f>IF(A36&lt;=0,"—",IF(C36&lt;=D36,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="27" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="B37" s="27" t="n">
-        <v>36.23</v>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>2.276535656408983</v>
-      </c>
-      <c r="E37" s="15" t="n">
-        <v>2.276535656408983</v>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.65</v>
+      </c>
+      <c r="B37" s="27">
+        <f>$B$9+A37</f>
+        <v/>
+      </c>
+      <c r="C37" s="5">
+        <f>IF(A37&lt;=0,0,IF(A37&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A37/($B$17*$B$7))^(1/$B$18)),IF(A37&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A37/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A37/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A37/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A37/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A37/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D37" s="5">
+        <f>IF(A37&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A37/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A37-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A37-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E37" s="15">
+        <f>MIN(C37,D37)</f>
+        <v/>
+      </c>
+      <c r="F37" s="4">
+        <f>IF(A37&lt;=0,"—",IF(C37&lt;=D37,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="27" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="B38" s="27" t="n">
-        <v>36.28</v>
-      </c>
-      <c r="C38" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D38" s="5" t="n">
-        <v>2.308288035873342</v>
-      </c>
-      <c r="E38" s="15" t="n">
-        <v>2.308288035873342</v>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.7</v>
+      </c>
+      <c r="B38" s="27">
+        <f>$B$9+A38</f>
+        <v/>
+      </c>
+      <c r="C38" s="5">
+        <f>IF(A38&lt;=0,0,IF(A38&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A38/($B$17*$B$7))^(1/$B$18)),IF(A38&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A38/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A38/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A38/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A38/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A38/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D38" s="5">
+        <f>IF(A38&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A38/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A38-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A38-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>MIN(C38,D38)</f>
+        <v/>
+      </c>
+      <c r="F38" s="4">
+        <f>IF(A38&lt;=0,"—",IF(C38&lt;=D38,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="27" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="B39" s="27" t="n">
-        <v>36.33000000000001</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D39" s="5" t="n">
-        <v>2.339609522593578</v>
-      </c>
-      <c r="E39" s="15" t="n">
-        <v>2.339609522593578</v>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.75</v>
+      </c>
+      <c r="B39" s="27">
+        <f>$B$9+A39</f>
+        <v/>
+      </c>
+      <c r="C39" s="5">
+        <f>IF(A39&lt;=0,0,IF(A39&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A39/($B$17*$B$7))^(1/$B$18)),IF(A39&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A39/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A39/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A39/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A39/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A39/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D39" s="5">
+        <f>IF(A39&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A39/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A39-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A39-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E39" s="15">
+        <f>MIN(C39,D39)</f>
+        <v/>
+      </c>
+      <c r="F39" s="4">
+        <f>IF(A39&lt;=0,"—",IF(C39&lt;=D39,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="27" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="B40" s="27" t="n">
-        <v>36.38</v>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D40" s="5" t="n">
-        <v>2.370517196703092</v>
-      </c>
-      <c r="E40" s="15" t="n">
-        <v>2.370517196703092</v>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.8</v>
+      </c>
+      <c r="B40" s="27">
+        <f>$B$9+A40</f>
+        <v/>
+      </c>
+      <c r="C40" s="5">
+        <f>IF(A40&lt;=0,0,IF(A40&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A40/($B$17*$B$7))^(1/$B$18)),IF(A40&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A40/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A40/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A40/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A40/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A40/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D40" s="5">
+        <f>IF(A40&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A40/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A40-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A40-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E40" s="15">
+        <f>MIN(C40,D40)</f>
+        <v/>
+      </c>
+      <c r="F40" s="4">
+        <f>IF(A40&lt;=0,"—",IF(C40&lt;=D40,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="27" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="B41" s="27" t="n">
-        <v>36.43</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D41" s="5" t="n">
-        <v>2.401027038898067</v>
-      </c>
-      <c r="E41" s="15" t="n">
-        <v>2.401027038898067</v>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.85</v>
+      </c>
+      <c r="B41" s="27">
+        <f>$B$9+A41</f>
+        <v/>
+      </c>
+      <c r="C41" s="5">
+        <f>IF(A41&lt;=0,0,IF(A41&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A41/($B$17*$B$7))^(1/$B$18)),IF(A41&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A41/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A41/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A41/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A41/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A41/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D41" s="5">
+        <f>IF(A41&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A41/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A41-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A41-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E41" s="15">
+        <f>MIN(C41,D41)</f>
+        <v/>
+      </c>
+      <c r="F41" s="4">
+        <f>IF(A41&lt;=0,"—",IF(C41&lt;=D41,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="27" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="B42" s="27" t="n">
-        <v>36.48</v>
-      </c>
-      <c r="C42" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D42" s="5" t="n">
-        <v>2.431154027036164</v>
-      </c>
-      <c r="E42" s="15" t="n">
-        <v>2.431154027036164</v>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.9</v>
+      </c>
+      <c r="B42" s="27">
+        <f>$B$9+A42</f>
+        <v/>
+      </c>
+      <c r="C42" s="5">
+        <f>IF(A42&lt;=0,0,IF(A42&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A42/($B$17*$B$7))^(1/$B$18)),IF(A42&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A42/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A42/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A42/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A42/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A42/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D42" s="5">
+        <f>IF(A42&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A42/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A42-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A42-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E42" s="15">
+        <f>MIN(C42,D42)</f>
+        <v/>
+      </c>
+      <c r="F42" s="4">
+        <f>IF(A42&lt;=0,"—",IF(C42&lt;=D42,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="27" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="B43" s="27" t="n">
-        <v>36.53</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D43" s="5" t="n">
-        <v>2.46091222208934</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <v>2.46091222208934</v>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>0.95</v>
+      </c>
+      <c r="B43" s="27">
+        <f>$B$9+A43</f>
+        <v/>
+      </c>
+      <c r="C43" s="5">
+        <f>IF(A43&lt;=0,0,IF(A43&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A43/($B$17*$B$7))^(1/$B$18)),IF(A43&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A43/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A43/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A43/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A43/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A43/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D43" s="5">
+        <f>IF(A43&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A43/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A43-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A43-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E43" s="15">
+        <f>MIN(C43,D43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="4">
+        <f>IF(A43&lt;=0,"—",IF(C43&lt;=D43,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="27" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="B44" s="27" t="n">
-        <v>36.58000000000001</v>
-      </c>
-      <c r="C44" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D44" s="5" t="n">
-        <v>2.490314844850592</v>
-      </c>
-      <c r="E44" s="15" t="n">
-        <v>2.490314844850592</v>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="B44" s="27">
+        <f>$B$9+A44</f>
+        <v/>
+      </c>
+      <c r="C44" s="5">
+        <f>IF(A44&lt;=0,0,IF(A44&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A44/($B$17*$B$7))^(1/$B$18)),IF(A44&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A44/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A44/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A44/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A44/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A44/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D44" s="5">
+        <f>IF(A44&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A44/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A44-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A44-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E44" s="15">
+        <f>MIN(C44,D44)</f>
+        <v/>
+      </c>
+      <c r="F44" s="4">
+        <f>IF(A44&lt;=0,"—",IF(C44&lt;=D44,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="27" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="B45" s="27" t="n">
-        <v>36.63</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D45" s="5" t="n">
-        <v>2.519374344581957</v>
-      </c>
-      <c r="E45" s="15" t="n">
-        <v>2.519374344581957</v>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.05</v>
+      </c>
+      <c r="B45" s="27">
+        <f>$B$9+A45</f>
+        <v/>
+      </c>
+      <c r="C45" s="5">
+        <f>IF(A45&lt;=0,0,IF(A45&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A45/($B$17*$B$7))^(1/$B$18)),IF(A45&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A45/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A45/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A45/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A45/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A45/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D45" s="5">
+        <f>IF(A45&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A45/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A45-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A45-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E45" s="15">
+        <f>MIN(C45,D45)</f>
+        <v/>
+      </c>
+      <c r="F45" s="4">
+        <f>IF(A45&lt;=0,"—",IF(C45&lt;=D45,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="27" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="B46" s="27" t="n">
-        <v>36.68</v>
-      </c>
-      <c r="C46" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D46" s="5" t="n">
-        <v>2.548102460615016</v>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>2.548102460615016</v>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.1</v>
+      </c>
+      <c r="B46" s="27">
+        <f>$B$9+A46</f>
+        <v/>
+      </c>
+      <c r="C46" s="5">
+        <f>IF(A46&lt;=0,0,IF(A46&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A46/($B$17*$B$7))^(1/$B$18)),IF(A46&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A46/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A46/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A46/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A46/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A46/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D46" s="5">
+        <f>IF(A46&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A46/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A46-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A46-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E46" s="15">
+        <f>MIN(C46,D46)</f>
+        <v/>
+      </c>
+      <c r="F46" s="4">
+        <f>IF(A46&lt;=0,"—",IF(C46&lt;=D46,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="27" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="B47" s="27" t="n">
-        <v>36.73</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>2.576510277768524</v>
-      </c>
-      <c r="E47" s="15" t="n">
-        <v>2.576510277768524</v>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.15</v>
+      </c>
+      <c r="B47" s="27">
+        <f>$B$9+A47</f>
+        <v/>
+      </c>
+      <c r="C47" s="5">
+        <f>IF(A47&lt;=0,0,IF(A47&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A47/($B$17*$B$7))^(1/$B$18)),IF(A47&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A47/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A47/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A47/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A47/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A47/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D47" s="5">
+        <f>IF(A47&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A47/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A47-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A47-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E47" s="15">
+        <f>MIN(C47,D47)</f>
+        <v/>
+      </c>
+      <c r="F47" s="4">
+        <f>IF(A47&lt;=0,"—",IF(C47&lt;=D47,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="27" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="B48" s="27" t="n">
-        <v>36.78</v>
-      </c>
-      <c r="C48" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D48" s="5" t="n">
-        <v>2.604608276325131</v>
-      </c>
-      <c r="E48" s="15" t="n">
-        <v>2.604608276325131</v>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.2</v>
+      </c>
+      <c r="B48" s="27">
+        <f>$B$9+A48</f>
+        <v/>
+      </c>
+      <c r="C48" s="5">
+        <f>IF(A48&lt;=0,0,IF(A48&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A48/($B$17*$B$7))^(1/$B$18)),IF(A48&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A48/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A48/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A48/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A48/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A48/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D48" s="5">
+        <f>IF(A48&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A48/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A48-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A48-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E48" s="15">
+        <f>MIN(C48,D48)</f>
+        <v/>
+      </c>
+      <c r="F48" s="4">
+        <f>IF(A48&lt;=0,"—",IF(C48&lt;=D48,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="27" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="B49" s="27" t="n">
-        <v>36.83000000000001</v>
-      </c>
-      <c r="C49" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D49" s="5" t="n">
-        <v>2.632406377206207</v>
-      </c>
-      <c r="E49" s="15" t="n">
-        <v>2.632406377206207</v>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.25</v>
+      </c>
+      <c r="B49" s="27">
+        <f>$B$9+A49</f>
+        <v/>
+      </c>
+      <c r="C49" s="5">
+        <f>IF(A49&lt;=0,0,IF(A49&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A49/($B$17*$B$7))^(1/$B$18)),IF(A49&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A49/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A49/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A49/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A49/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A49/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D49" s="5">
+        <f>IF(A49&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A49/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A49-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A49-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E49" s="15">
+        <f>MIN(C49,D49)</f>
+        <v/>
+      </c>
+      <c r="F49" s="4">
+        <f>IF(A49&lt;=0,"—",IF(C49&lt;=D49,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="B50" s="27" t="n">
-        <v>36.88</v>
-      </c>
-      <c r="C50" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D50" s="5" t="n">
-        <v>2.659913982896899</v>
-      </c>
-      <c r="E50" s="15" t="n">
-        <v>2.659913982896899</v>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.3</v>
+      </c>
+      <c r="B50" s="27">
+        <f>$B$9+A50</f>
+        <v/>
+      </c>
+      <c r="C50" s="5">
+        <f>IF(A50&lt;=0,0,IF(A50&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A50/($B$17*$B$7))^(1/$B$18)),IF(A50&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A50/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A50/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A50/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A50/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A50/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D50" s="5">
+        <f>IF(A50&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A50/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A50-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A50-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E50" s="15">
+        <f>MIN(C50,D50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="4">
+        <f>IF(A50&lt;=0,"—",IF(C50&lt;=D50,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="27" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="B51" s="27" t="n">
-        <v>36.93</v>
-      </c>
-      <c r="C51" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D51" s="5" t="n">
-        <v>2.687140014600091</v>
-      </c>
-      <c r="E51" s="15" t="n">
-        <v>2.687140014600091</v>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.35</v>
+      </c>
+      <c r="B51" s="27">
+        <f>$B$9+A51</f>
+        <v/>
+      </c>
+      <c r="C51" s="5">
+        <f>IF(A51&lt;=0,0,IF(A51&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A51/($B$17*$B$7))^(1/$B$18)),IF(A51&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A51/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A51/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A51/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A51/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A51/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D51" s="5">
+        <f>IF(A51&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A51/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A51-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A51-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E51" s="15">
+        <f>MIN(C51,D51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="4">
+        <f>IF(A51&lt;=0,"—",IF(C51&lt;=D51,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="27" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="B52" s="27" t="n">
-        <v>36.98</v>
-      </c>
-      <c r="C52" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D52" s="5" t="n">
-        <v>2.714092946035473</v>
-      </c>
-      <c r="E52" s="15" t="n">
-        <v>2.714092946035473</v>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.4</v>
+      </c>
+      <c r="B52" s="27">
+        <f>$B$9+A52</f>
+        <v/>
+      </c>
+      <c r="C52" s="5">
+        <f>IF(A52&lt;=0,0,IF(A52&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A52/($B$17*$B$7))^(1/$B$18)),IF(A52&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A52/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A52/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A52/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A52/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A52/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D52" s="5">
+        <f>IF(A52&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A52/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A52-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A52-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E52" s="15">
+        <f>MIN(C52,D52)</f>
+        <v/>
+      </c>
+      <c r="F52" s="4">
+        <f>IF(A52&lt;=0,"—",IF(C52&lt;=D52,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="27" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="B53" s="27" t="n">
-        <v>37.03</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D53" s="5" t="n">
-        <v>2.740780834246703</v>
-      </c>
-      <c r="E53" s="15" t="n">
-        <v>2.740780834246703</v>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.45</v>
+      </c>
+      <c r="B53" s="27">
+        <f>$B$9+A53</f>
+        <v/>
+      </c>
+      <c r="C53" s="5">
+        <f>IF(A53&lt;=0,0,IF(A53&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A53/($B$17*$B$7))^(1/$B$18)),IF(A53&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A53/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A53/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A53/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A53/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A53/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D53" s="5">
+        <f>IF(A53&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A53/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A53-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A53-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E53" s="15">
+        <f>MIN(C53,D53)</f>
+        <v/>
+      </c>
+      <c r="F53" s="4">
+        <f>IF(A53&lt;=0,"—",IF(C53&lt;=D53,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="27" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="B54" s="27" t="n">
-        <v>37.08000000000001</v>
-      </c>
-      <c r="C54" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D54" s="5" t="n">
-        <v>2.767211347734138</v>
-      </c>
-      <c r="E54" s="15" t="n">
-        <v>2.767211347734138</v>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.5</v>
+      </c>
+      <c r="B54" s="27">
+        <f>$B$9+A54</f>
+        <v/>
+      </c>
+      <c r="C54" s="5">
+        <f>IF(A54&lt;=0,0,IF(A54&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A54/($B$17*$B$7))^(1/$B$18)),IF(A54&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A54/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A54/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A54/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A54/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A54/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D54" s="5">
+        <f>IF(A54&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A54/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A54-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A54-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E54" s="15">
+        <f>MIN(C54,D54)</f>
+        <v/>
+      </c>
+      <c r="F54" s="4">
+        <f>IF(A54&lt;=0,"—",IF(C54&lt;=D54,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="27" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="B55" s="27" t="n">
-        <v>37.13</v>
-      </c>
-      <c r="C55" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D55" s="5" t="n">
-        <v>2.79339179219155</v>
-      </c>
-      <c r="E55" s="15" t="n">
-        <v>2.79339179219155</v>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.55</v>
+      </c>
+      <c r="B55" s="27">
+        <f>$B$9+A55</f>
+        <v/>
+      </c>
+      <c r="C55" s="5">
+        <f>IF(A55&lt;=0,0,IF(A55&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A55/($B$17*$B$7))^(1/$B$18)),IF(A55&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A55/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A55/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A55/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A55/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A55/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D55" s="5">
+        <f>IF(A55&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A55/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A55-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A55-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E55" s="15">
+        <f>MIN(C55,D55)</f>
+        <v/>
+      </c>
+      <c r="F55" s="4">
+        <f>IF(A55&lt;=0,"—",IF(C55&lt;=D55,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="27" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="B56" s="27" t="n">
-        <v>37.18</v>
-      </c>
-      <c r="C56" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D56" s="5" t="n">
-        <v>2.819329134091594</v>
-      </c>
-      <c r="E56" s="15" t="n">
-        <v>2.819329134091594</v>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.6</v>
+      </c>
+      <c r="B56" s="27">
+        <f>$B$9+A56</f>
+        <v/>
+      </c>
+      <c r="C56" s="5">
+        <f>IF(A56&lt;=0,0,IF(A56&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A56/($B$17*$B$7))^(1/$B$18)),IF(A56&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A56/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A56/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A56/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A56/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A56/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D56" s="5">
+        <f>IF(A56&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A56/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A56-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A56-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E56" s="15">
+        <f>MIN(C56,D56)</f>
+        <v/>
+      </c>
+      <c r="F56" s="4">
+        <f>IF(A56&lt;=0,"—",IF(C56&lt;=D56,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="27" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="B57" s="27" t="n">
-        <v>37.23</v>
-      </c>
-      <c r="C57" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D57" s="5" t="n">
-        <v>2.845030022335827</v>
-      </c>
-      <c r="E57" s="15" t="n">
-        <v>2.845030022335827</v>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.65</v>
+      </c>
+      <c r="B57" s="27">
+        <f>$B$9+A57</f>
+        <v/>
+      </c>
+      <c r="C57" s="5">
+        <f>IF(A57&lt;=0,0,IF(A57&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A57/($B$17*$B$7))^(1/$B$18)),IF(A57&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A57/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A57/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A57/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A57/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A57/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D57" s="5">
+        <f>IF(A57&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A57/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A57-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A57-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E57" s="15">
+        <f>MIN(C57,D57)</f>
+        <v/>
+      </c>
+      <c r="F57" s="4">
+        <f>IF(A57&lt;=0,"—",IF(C57&lt;=D57,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="27" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="B58" s="27" t="n">
-        <v>37.28</v>
-      </c>
-      <c r="C58" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D58" s="5" t="n">
-        <v>2.870500808159916</v>
-      </c>
-      <c r="E58" s="15" t="n">
-        <v>2.870500808159916</v>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.7</v>
+      </c>
+      <c r="B58" s="27">
+        <f>$B$9+A58</f>
+        <v/>
+      </c>
+      <c r="C58" s="5">
+        <f>IF(A58&lt;=0,0,IF(A58&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A58/($B$17*$B$7))^(1/$B$18)),IF(A58&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A58/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A58/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A58/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A58/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A58/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D58" s="5">
+        <f>IF(A58&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A58/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A58-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A58-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E58" s="15">
+        <f>MIN(C58,D58)</f>
+        <v/>
+      </c>
+      <c r="F58" s="4">
+        <f>IF(A58&lt;=0,"—",IF(C58&lt;=D58,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="27" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="B59" s="27" t="n">
-        <v>37.33000000000001</v>
-      </c>
-      <c r="C59" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D59" s="5" t="n">
-        <v>2.89574756346289</v>
-      </c>
-      <c r="E59" s="15" t="n">
-        <v>2.89574756346289</v>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.75</v>
+      </c>
+      <c r="B59" s="27">
+        <f>$B$9+A59</f>
+        <v/>
+      </c>
+      <c r="C59" s="5">
+        <f>IF(A59&lt;=0,0,IF(A59&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A59/($B$17*$B$7))^(1/$B$18)),IF(A59&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A59/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A59/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A59/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A59/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A59/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D59" s="5">
+        <f>IF(A59&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A59/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A59-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A59-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E59" s="15">
+        <f>MIN(C59,D59)</f>
+        <v/>
+      </c>
+      <c r="F59" s="4">
+        <f>IF(A59&lt;=0,"—",IF(C59&lt;=D59,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="27" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="B60" s="27" t="n">
-        <v>37.38</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D60" s="5" t="n">
-        <v>2.920776097710299</v>
-      </c>
-      <c r="E60" s="15" t="n">
-        <v>2.920776097710299</v>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.8</v>
+      </c>
+      <c r="B60" s="27">
+        <f>$B$9+A60</f>
+        <v/>
+      </c>
+      <c r="C60" s="5">
+        <f>IF(A60&lt;=0,0,IF(A60&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A60/($B$17*$B$7))^(1/$B$18)),IF(A60&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A60/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A60/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A60/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A60/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A60/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D60" s="5">
+        <f>IF(A60&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A60/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A60-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A60-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E60" s="15">
+        <f>MIN(C60,D60)</f>
+        <v/>
+      </c>
+      <c r="F60" s="4">
+        <f>IF(A60&lt;=0,"—",IF(C60&lt;=D60,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="27" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="B61" s="27" t="n">
-        <v>37.43</v>
-      </c>
-      <c r="C61" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D61" s="5" t="n">
-        <v>2.945591973544595</v>
-      </c>
-      <c r="E61" s="15" t="n">
-        <v>2.945591973544595</v>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.85</v>
+      </c>
+      <c r="B61" s="27">
+        <f>$B$9+A61</f>
+        <v/>
+      </c>
+      <c r="C61" s="5">
+        <f>IF(A61&lt;=0,0,IF(A61&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A61/($B$17*$B$7))^(1/$B$18)),IF(A61&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A61/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A61/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A61/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A61/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A61/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D61" s="5">
+        <f>IF(A61&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A61/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A61-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A61-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E61" s="15">
+        <f>MIN(C61,D61)</f>
+        <v/>
+      </c>
+      <c r="F61" s="4">
+        <f>IF(A61&lt;=0,"—",IF(C61&lt;=D61,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="27" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="B62" s="27" t="n">
-        <v>37.48</v>
-      </c>
-      <c r="C62" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D62" s="5" t="n">
-        <v>2.970200521221568</v>
-      </c>
-      <c r="E62" s="15" t="n">
-        <v>2.970200521221568</v>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.9</v>
+      </c>
+      <c r="B62" s="27">
+        <f>$B$9+A62</f>
+        <v/>
+      </c>
+      <c r="C62" s="5">
+        <f>IF(A62&lt;=0,0,IF(A62&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A62/($B$17*$B$7))^(1/$B$18)),IF(A62&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A62/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A62/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A62/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A62/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A62/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D62" s="5">
+        <f>IF(A62&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A62/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A62-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A62-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E62" s="15">
+        <f>MIN(C62,D62)</f>
+        <v/>
+      </c>
+      <c r="F62" s="4">
+        <f>IF(A62&lt;=0,"—",IF(C62&lt;=D62,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="27" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="B63" s="27" t="n">
-        <v>37.53</v>
-      </c>
-      <c r="C63" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D63" s="5" t="n">
-        <v>2.994606851978972</v>
-      </c>
-      <c r="E63" s="15" t="n">
-        <v>2.994606851978972</v>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>1.95</v>
+      </c>
+      <c r="B63" s="27">
+        <f>$B$9+A63</f>
+        <v/>
+      </c>
+      <c r="C63" s="5">
+        <f>IF(A63&lt;=0,0,IF(A63&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A63/($B$17*$B$7))^(1/$B$18)),IF(A63&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A63/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A63/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A63/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A63/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A63/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D63" s="5">
+        <f>IF(A63&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A63/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A63-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A63-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E63" s="15">
+        <f>MIN(C63,D63)</f>
+        <v/>
+      </c>
+      <c r="F63" s="4">
+        <f>IF(A63&lt;=0,"—",IF(C63&lt;=D63,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="27" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="B64" s="27" t="n">
-        <v>37.58000000000001</v>
-      </c>
-      <c r="C64" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D64" s="5" t="n">
-        <v>3.018815870432304</v>
-      </c>
-      <c r="E64" s="15" t="n">
-        <v>3.018815870432304</v>
-      </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="B64" s="27">
+        <f>$B$9+A64</f>
+        <v/>
+      </c>
+      <c r="C64" s="5">
+        <f>IF(A64&lt;=0,0,IF(A64&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A64/($B$17*$B$7))^(1/$B$18)),IF(A64&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A64/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A64/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A64/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A64/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A64/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D64" s="5">
+        <f>IF(A64&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A64/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A64-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A64-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E64" s="15">
+        <f>MIN(C64,D64)</f>
+        <v/>
+      </c>
+      <c r="F64" s="4">
+        <f>IF(A64&lt;=0,"—",IF(C64&lt;=D64,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="27" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="B65" s="27" t="n">
-        <v>37.63</v>
-      </c>
-      <c r="C65" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D65" s="5" t="n">
-        <v>3.042832286082899</v>
-      </c>
-      <c r="E65" s="15" t="n">
-        <v>3.042832286082899</v>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>2.05</v>
+      </c>
+      <c r="B65" s="27">
+        <f>$B$9+A65</f>
+        <v/>
+      </c>
+      <c r="C65" s="5">
+        <f>IF(A65&lt;=0,0,IF(A65&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A65/($B$17*$B$7))^(1/$B$18)),IF(A65&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A65/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A65/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A65/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A65/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A65/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D65" s="5">
+        <f>IF(A65&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A65/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A65-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A65-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E65" s="15">
+        <f>MIN(C65,D65)</f>
+        <v/>
+      </c>
+      <c r="F65" s="4">
+        <f>IF(A65&lt;=0,"—",IF(C65&lt;=D65,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="27" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="B66" s="27" t="n">
-        <v>37.68</v>
-      </c>
-      <c r="C66" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D66" s="5" t="n">
-        <v>3.066660624014829</v>
-      </c>
-      <c r="E66" s="15" t="n">
-        <v>3.066660624014829</v>
-      </c>
-      <c r="F66" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>2.1</v>
+      </c>
+      <c r="B66" s="27">
+        <f>$B$9+A66</f>
+        <v/>
+      </c>
+      <c r="C66" s="5">
+        <f>IF(A66&lt;=0,0,IF(A66&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A66/($B$17*$B$7))^(1/$B$18)),IF(A66&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A66/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A66/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A66/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A66/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A66/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D66" s="5">
+        <f>IF(A66&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A66/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A66-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A66-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E66" s="15">
+        <f>MIN(C66,D66)</f>
+        <v/>
+      </c>
+      <c r="F66" s="4">
+        <f>IF(A66&lt;=0,"—",IF(C66&lt;=D66,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="27" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="B67" s="27" t="n">
-        <v>37.73</v>
-      </c>
-      <c r="C67" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D67" s="5" t="n">
-        <v>3.090305234849392</v>
-      </c>
-      <c r="E67" s="15" t="n">
-        <v>3.090305234849392</v>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>2.15</v>
+      </c>
+      <c r="B67" s="27">
+        <f>$B$9+A67</f>
+        <v/>
+      </c>
+      <c r="C67" s="5">
+        <f>IF(A67&lt;=0,0,IF(A67&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A67/($B$17*$B$7))^(1/$B$18)),IF(A67&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A67/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A67/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A67/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A67/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A67/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D67" s="5">
+        <f>IF(A67&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A67/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A67-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A67-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E67" s="15">
+        <f>MIN(C67,D67)</f>
+        <v/>
+      </c>
+      <c r="F67" s="4">
+        <f>IF(A67&lt;=0,"—",IF(C67&lt;=D67,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="27" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="B68" s="27" t="n">
-        <v>37.78</v>
-      </c>
-      <c r="C68" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D68" s="5" t="n">
-        <v>3.113770304019243</v>
-      </c>
-      <c r="E68" s="15" t="n">
-        <v>3.113770304019243</v>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>2.2</v>
+      </c>
+      <c r="B68" s="27">
+        <f>$B$9+A68</f>
+        <v/>
+      </c>
+      <c r="C68" s="5">
+        <f>IF(A68&lt;=0,0,IF(A68&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A68/($B$17*$B$7))^(1/$B$18)),IF(A68&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A68/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A68/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A68/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A68/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A68/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D68" s="5">
+        <f>IF(A68&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A68/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A68-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A68-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E68" s="15">
+        <f>MIN(C68,D68)</f>
+        <v/>
+      </c>
+      <c r="F68" s="4">
+        <f>IF(A68&lt;=0,"—",IF(C68&lt;=D68,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="27" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="B69" s="27" t="n">
-        <v>37.83000000000001</v>
-      </c>
-      <c r="C69" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D69" s="5" t="n">
-        <v>3.137059860418132</v>
-      </c>
-      <c r="E69" s="15" t="n">
-        <v>3.137059860418132</v>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+        <v>2.25</v>
+      </c>
+      <c r="B69" s="27">
+        <f>$B$9+A69</f>
+        <v/>
+      </c>
+      <c r="C69" s="5">
+        <f>IF(A69&lt;=0,0,IF(A69&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A69/($B$17*$B$7))^(1/$B$18)),IF(A69&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A69/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A69/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A69/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A69/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A69/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D69" s="5">
+        <f>IF(A69&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A69/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A69-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A69-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E69" s="15">
+        <f>MIN(C69,D69)</f>
+        <v/>
+      </c>
+      <c r="F69" s="4">
+        <f>IF(A69&lt;=0,"—",IF(C69&lt;=D69,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="27" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="B70" s="27">
+        <f>$B$9+A70</f>
+        <v/>
+      </c>
+      <c r="C70" s="5">
+        <f>IF(A70&lt;=0,0,IF(A70&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A70/($B$17*$B$7))^(1/$B$18)),IF(A70&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A70/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A70/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A70/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A70/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A70/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D70" s="5">
+        <f>IF(A70&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A70/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A70-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A70-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E70" s="15">
+        <f>MIN(C70,D70)</f>
+        <v/>
+      </c>
+      <c r="F70" s="4">
+        <f>IF(A70&lt;=0,"—",IF(C70&lt;=D70,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="27" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="B71" s="27">
+        <f>$B$9+A71</f>
+        <v/>
+      </c>
+      <c r="C71" s="5">
+        <f>IF(A71&lt;=0,0,IF(A71&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A71/($B$17*$B$7))^(1/$B$18)),IF(A71&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A71/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A71/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A71/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A71/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A71/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D71" s="5">
+        <f>IF(A71&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A71/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A71-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A71-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E71" s="15">
+        <f>MIN(C71,D71)</f>
+        <v/>
+      </c>
+      <c r="F71" s="4">
+        <f>IF(A71&lt;=0,"—",IF(C71&lt;=D71,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="B72" s="35">
+        <f>$B$9+A72</f>
+        <v/>
+      </c>
+      <c r="C72" s="8">
+        <f>IF(A72&lt;=0,0,IF(A72&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A72/($B$17*$B$7))^(1/$B$18)),IF(A72&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A72/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A72/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A72/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A72/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A72/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D72" s="8">
+        <f>IF(A72&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A72/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A72-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A72-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E72" s="8">
+        <f>MIN(C72,D72)</f>
+        <v/>
+      </c>
+      <c r="F72" s="7">
+        <f>IF(A72&lt;=0,"—",IF(C72&lt;=D72,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="27" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="B73" s="27">
+        <f>$B$9+A73</f>
+        <v/>
+      </c>
+      <c r="C73" s="5">
+        <f>IF(A73&lt;=0,0,IF(A73&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A73/($B$17*$B$7))^(1/$B$18)),IF(A73&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A73/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A73/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A73/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A73/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A73/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D73" s="5">
+        <f>IF(A73&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A73/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A73-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A73-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E73" s="15">
+        <f>MIN(C73,D73)</f>
+        <v/>
+      </c>
+      <c r="F73" s="4">
+        <f>IF(A73&lt;=0,"—",IF(C73&lt;=D73,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B74" s="27">
+        <f>$B$9+A74</f>
+        <v/>
+      </c>
+      <c r="C74" s="5">
+        <f>IF(A74&lt;=0,0,IF(A74&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A74/($B$17*$B$7))^(1/$B$18)),IF(A74&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A74/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A74/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A74/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A74/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A74/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D74" s="5">
+        <f>IF(A74&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A74/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A74-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A74-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E74" s="15">
+        <f>MIN(C74,D74)</f>
+        <v/>
+      </c>
+      <c r="F74" s="4">
+        <f>IF(A74&lt;=0,"—",IF(C74&lt;=D74,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="27" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="B75" s="27">
+        <f>$B$9+A75</f>
+        <v/>
+      </c>
+      <c r="C75" s="5">
+        <f>IF(A75&lt;=0,0,IF(A75&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A75/($B$17*$B$7))^(1/$B$18)),IF(A75&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A75/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A75/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A75/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A75/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A75/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D75" s="5">
+        <f>IF(A75&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A75/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A75-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A75-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E75" s="15">
+        <f>MIN(C75,D75)</f>
+        <v/>
+      </c>
+      <c r="F75" s="4">
+        <f>IF(A75&lt;=0,"—",IF(C75&lt;=D75,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="27" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="B76" s="27">
+        <f>$B$9+A76</f>
+        <v/>
+      </c>
+      <c r="C76" s="5">
+        <f>IF(A76&lt;=0,0,IF(A76&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A76/($B$17*$B$7))^(1/$B$18)),IF(A76&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A76/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A76/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A76/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A76/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A76/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D76" s="5">
+        <f>IF(A76&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A76/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A76-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A76-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E76" s="15">
+        <f>MIN(C76,D76)</f>
+        <v/>
+      </c>
+      <c r="F76" s="4">
+        <f>IF(A76&lt;=0,"—",IF(C76&lt;=D76,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="27" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="B77" s="27">
+        <f>$B$9+A77</f>
+        <v/>
+      </c>
+      <c r="C77" s="5">
+        <f>IF(A77&lt;=0,0,IF(A77&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A77/($B$17*$B$7))^(1/$B$18)),IF(A77&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A77/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A77/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A77/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A77/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A77/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D77" s="5">
+        <f>IF(A77&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A77/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A77-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A77-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E77" s="15">
+        <f>MIN(C77,D77)</f>
+        <v/>
+      </c>
+      <c r="F77" s="4">
+        <f>IF(A77&lt;=0,"—",IF(C77&lt;=D77,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="27" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="B78" s="27">
+        <f>$B$9+A78</f>
+        <v/>
+      </c>
+      <c r="C78" s="5">
+        <f>IF(A78&lt;=0,0,IF(A78&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A78/($B$17*$B$7))^(1/$B$18)),IF(A78&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A78/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A78/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A78/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A78/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A78/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D78" s="5">
+        <f>IF(A78&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A78/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A78-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A78-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E78" s="15">
+        <f>MIN(C78,D78)</f>
+        <v/>
+      </c>
+      <c r="F78" s="4">
+        <f>IF(A78&lt;=0,"—",IF(C78&lt;=D78,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="27" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="B79" s="27">
+        <f>$B$9+A79</f>
+        <v/>
+      </c>
+      <c r="C79" s="5">
+        <f>IF(A79&lt;=0,0,IF(A79&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A79/($B$17*$B$7))^(1/$B$18)),IF(A79&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A79/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A79/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A79/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A79/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A79/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D79" s="5">
+        <f>IF(A79&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A79/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A79-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A79-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E79" s="15">
+        <f>MIN(C79,D79)</f>
+        <v/>
+      </c>
+      <c r="F79" s="4">
+        <f>IF(A79&lt;=0,"—",IF(C79&lt;=D79,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="B80" s="27">
+        <f>$B$9+A80</f>
+        <v/>
+      </c>
+      <c r="C80" s="5">
+        <f>IF(A80&lt;=0,0,IF(A80&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A80/($B$17*$B$7))^(1/$B$18)),IF(A80&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A80/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A80/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A80/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A80/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A80/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D80" s="5">
+        <f>IF(A80&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A80/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A80-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A80-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E80" s="15">
+        <f>MIN(C80,D80)</f>
+        <v/>
+      </c>
+      <c r="F80" s="4">
+        <f>IF(A80&lt;=0,"—",IF(C80&lt;=D80,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="27" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="B81" s="27">
+        <f>$B$9+A81</f>
+        <v/>
+      </c>
+      <c r="C81" s="5">
+        <f>IF(A81&lt;=0,0,IF(A81&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A81/($B$17*$B$7))^(1/$B$18)),IF(A81&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A81/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A81/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A81/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A81/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A81/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D81" s="5">
+        <f>IF(A81&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A81/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A81-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A81-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E81" s="15">
+        <f>MIN(C81,D81)</f>
+        <v/>
+      </c>
+      <c r="F81" s="4">
+        <f>IF(A81&lt;=0,"—",IF(C81&lt;=D81,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="27" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="B82" s="27">
+        <f>$B$9+A82</f>
+        <v/>
+      </c>
+      <c r="C82" s="5">
+        <f>IF(A82&lt;=0,0,IF(A82&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A82/($B$17*$B$7))^(1/$B$18)),IF(A82&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A82/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A82/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A82/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A82/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A82/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D82" s="5">
+        <f>IF(A82&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A82/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A82-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A82-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E82" s="15">
+        <f>MIN(C82,D82)</f>
+        <v/>
+      </c>
+      <c r="F82" s="4">
+        <f>IF(A82&lt;=0,"—",IF(C82&lt;=D82,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="27" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="B83" s="27">
+        <f>$B$9+A83</f>
+        <v/>
+      </c>
+      <c r="C83" s="5">
+        <f>IF(A83&lt;=0,0,IF(A83&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A83/($B$17*$B$7))^(1/$B$18)),IF(A83&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A83/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A83/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A83/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A83/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A83/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D83" s="5">
+        <f>IF(A83&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A83/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A83-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A83-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E83" s="15">
+        <f>MIN(C83,D83)</f>
+        <v/>
+      </c>
+      <c r="F83" s="4">
+        <f>IF(A83&lt;=0,"—",IF(C83&lt;=D83,"inlet","outlet"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B70" s="27" t="n">
-        <v>37.88</v>
-      </c>
-      <c r="C70" s="5" t="n">
-        <v>10.76126608759892</v>
-      </c>
-      <c r="D70" s="5" t="n">
-        <v>3.160177784476874</v>
-      </c>
-      <c r="E70" s="15" t="n">
-        <v>3.160177784476874</v>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>outlet</t>
-        </is>
+      <c r="B84" s="27">
+        <f>$B$9+A84</f>
+        <v/>
+      </c>
+      <c r="C84" s="5">
+        <f>IF(A84&lt;=0,0,IF(A84&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A84/($B$17*$B$7))^(1/$B$18)),IF(A84&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A84/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A84/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A84/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A84/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A84/$B$7-$B$20)/$B$19))))))</f>
+        <v/>
+      </c>
+      <c r="D84" s="5">
+        <f>IF(A84&lt;$B$7,IF($B$6&lt;=0,0,(1/$B$6)*((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7)))))))*IF((IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7))))))))&lt;=0,0,(IF((($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7))))))&lt;=0,0,((($B$7/2)^2/2)*((2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7)))))-SIN(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7)))))))/(($B$7/2)*(2*ACOS(1-2*(MIN(0.999,MAX(1E-6,A84/$B$7))))))))^(2/3))*SQRT($B$11)),IF((A84-$B$12+$B$11*$B$8)&lt;=0,0,(PI()*($B$7/2)^2)*SQRT((A84-$B$12+$B$11*$B$8)/((1+$B$21)/(2*9.81)+($B$6^2)*$B$8/(($B$7/4)^(4/3))))))</f>
+        <v/>
+      </c>
+      <c r="E84" s="15">
+        <f>MIN(C84,D84)</f>
+        <v/>
+      </c>
+      <c r="F84" s="4">
+        <f>IF(A84&lt;=0,"—",IF(C84&lt;=D84,"inlet","outlet"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4082,9 +4506,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="31" t="inlineStr">
-        <is>
-          <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy − Qout)·Δt.</t>
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. La courbe Courbe_QH_900 est en formules live (changer n/L/entrée/TW).</t>
         </is>
       </c>
     </row>
@@ -4095,7 +4519,7 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="37">
         <f>Parametres!B24</f>
         <v/>
       </c>
@@ -4106,7 +4530,7 @@
           <t>Q_plein réf. (m³/s)</t>
         </is>
       </c>
-      <c r="B6" s="30">
+      <c r="B6" s="37">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -4210,7 +4634,7 @@
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>IF(C13&lt;=0,0,IF(C13&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1))+(C13-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C13,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C13&lt;=0,0,IF(C13&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C13,Courbe_QH_900!$A$24:$A$84,1))+(C13-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C13,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C13,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C13,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C13,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C13,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E13" s="5">
@@ -4240,7 +4664,7 @@
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>IF(C14&lt;=0,0,IF(C14&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1))+(C14-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C14,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C14&lt;=0,0,IF(C14&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C14,Courbe_QH_900!$A$24:$A$84,1))+(C14-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C14,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C14,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C14,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C14,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C14,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E14" s="5">
@@ -4270,7 +4694,7 @@
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>IF(C15&lt;=0,0,IF(C15&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1))+(C15-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C15,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C15&lt;=0,0,IF(C15&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C15,Courbe_QH_900!$A$24:$A$84,1))+(C15-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C15,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C15,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C15,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C15,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C15,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E15" s="5">
@@ -4300,7 +4724,7 @@
         <v/>
       </c>
       <c r="D16" s="5">
-        <f>IF(C16&lt;=0,0,IF(C16&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1))+(C16-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C16,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C16&lt;=0,0,IF(C16&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C16,Courbe_QH_900!$A$24:$A$84,1))+(C16-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C16,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C16,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C16,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C16,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C16,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E16" s="5">
@@ -4330,7 +4754,7 @@
         <v/>
       </c>
       <c r="D17" s="5">
-        <f>IF(C17&lt;=0,0,IF(C17&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1))+(C17-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C17,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C17&lt;=0,0,IF(C17&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C17,Courbe_QH_900!$A$24:$A$84,1))+(C17-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C17,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C17,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C17,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C17,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C17,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E17" s="5">
@@ -4360,7 +4784,7 @@
         <v/>
       </c>
       <c r="D18" s="5">
-        <f>IF(C18&lt;=0,0,IF(C18&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1))+(C18-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C18,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C18&lt;=0,0,IF(C18&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C18,Courbe_QH_900!$A$24:$A$84,1))+(C18-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C18,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C18,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C18,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C18,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C18,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E18" s="5">
@@ -4390,7 +4814,7 @@
         <v/>
       </c>
       <c r="D19" s="5">
-        <f>IF(C19&lt;=0,0,IF(C19&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1))+(C19-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C19,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C19&lt;=0,0,IF(C19&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C19,Courbe_QH_900!$A$24:$A$84,1))+(C19-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C19,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C19,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C19,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C19,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C19,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E19" s="5">
@@ -4420,7 +4844,7 @@
         <v/>
       </c>
       <c r="D20" s="5">
-        <f>IF(C20&lt;=0,0,IF(C20&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1))+(C20-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C20,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C20&lt;=0,0,IF(C20&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C20,Courbe_QH_900!$A$24:$A$84,1))+(C20-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C20,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C20,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C20,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C20,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C20,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E20" s="5">
@@ -4450,7 +4874,7 @@
         <v/>
       </c>
       <c r="D21" s="5">
-        <f>IF(C21&lt;=0,0,IF(C21&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1))+(C21-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C21,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C21&lt;=0,0,IF(C21&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C21,Courbe_QH_900!$A$24:$A$84,1))+(C21-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C21,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C21,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C21,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C21,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C21,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E21" s="5">
@@ -4480,7 +4904,7 @@
         <v/>
       </c>
       <c r="D22" s="5">
-        <f>IF(C22&lt;=0,0,IF(C22&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1))+(C22-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C22,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C22&lt;=0,0,IF(C22&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C22,Courbe_QH_900!$A$24:$A$84,1))+(C22-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C22,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C22,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C22,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C22,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C22,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E22" s="5">
@@ -4510,7 +4934,7 @@
         <v/>
       </c>
       <c r="D23" s="5">
-        <f>IF(C23&lt;=0,0,IF(C23&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1))+(C23-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C23,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C23&lt;=0,0,IF(C23&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C23,Courbe_QH_900!$A$24:$A$84,1))+(C23-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C23,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C23,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C23,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C23,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C23,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E23" s="5">
@@ -4540,7 +4964,7 @@
         <v/>
       </c>
       <c r="D24" s="5">
-        <f>IF(C24&lt;=0,0,IF(C24&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1))+(C24-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C24,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C24&lt;=0,0,IF(C24&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C24,Courbe_QH_900!$A$24:$A$84,1))+(C24-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C24,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C24,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C24,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C24,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C24,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E24" s="5">
@@ -4570,7 +4994,7 @@
         <v/>
       </c>
       <c r="D25" s="5">
-        <f>IF(C25&lt;=0,0,IF(C25&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1))+(C25-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C25,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C25&lt;=0,0,IF(C25&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1))+(C25-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E25" s="5">
@@ -4600,7 +5024,7 @@
         <v/>
       </c>
       <c r="D26" s="5">
-        <f>IF(C26&lt;=0,0,IF(C26&gt;=INDEX(Courbe_QH_900!$A$10:$A$70,ROWS(Courbe_QH_900!$A$10:$A$70)),INDEX(Courbe_QH_900!$E$10:$E$70,ROWS(Courbe_QH_900!$E$10:$E$70)),INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1))+(C26-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)))/(INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$A$10:$A$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)))*(INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)+1)-INDEX(Courbe_QH_900!$E$10:$E$70,MATCH(C26,Courbe_QH_900!$A$10:$A$70,1)))))</f>
+        <f>IF(C26&lt;=0,0,IF(C26&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1))+(C26-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)))))</f>
         <v/>
       </c>
       <c r="E26" s="5">
@@ -4637,7 +5061,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="38" t="inlineStr">
         <is>
           <t>Où sont les fichiers HY-8 / capacité ?</t>
         </is>
@@ -4770,7 +5194,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="33" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>

</xml_diff>

<commit_message>
Fix Qinlet chart dip at submerged transition on Courbe_QH_900
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -2629,7 +2629,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Changez les cellules JAUNES (n, D, L, radiers, entrée, TW) : toute la table se recalcule. Q_gouvernant = MIN(Qinlet, Qoutlet). Pas besoin de relancer Python.</t>
+          <t>Changez les cellules JAUNES (n, D, L, radiers, entrée, TW) : toute la table se recalcule. Q_gouvernant = MIN(Qinlet, Qoutlet) = debit retenu pour le design. Sur ce tuyau long, Q_gouvernant suit Qoutlet (courbe verte). Qinlet (rouge) est seulement la capacite d'entree — souvent plus haute.</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
         <v/>
       </c>
       <c r="C24" s="5">
-        <f>IF(A24&lt;=0,0,IF(A24&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A24/($B$17*$B$7))^(1/$B$18)),IF(A24&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A24/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A24/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A24/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A24/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A24/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A24&lt;=0,0,IF(A24&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A24/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A24/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D24" s="5">
@@ -2980,7 +2980,7 @@
         <v/>
       </c>
       <c r="C25" s="5">
-        <f>IF(A25&lt;=0,0,IF(A25&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A25/($B$17*$B$7))^(1/$B$18)),IF(A25&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A25/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A25/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A25/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A25/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A25/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A25&lt;=0,0,IF(A25&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A25/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A25/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D25" s="5">
@@ -3005,7 +3005,7 @@
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>IF(A26&lt;=0,0,IF(A26&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A26/($B$17*$B$7))^(1/$B$18)),IF(A26&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A26/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A26/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A26/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A26/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A26/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A26&lt;=0,0,IF(A26&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A26/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A26/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D26" s="5">
@@ -3030,7 +3030,7 @@
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>IF(A27&lt;=0,0,IF(A27&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A27/($B$17*$B$7))^(1/$B$18)),IF(A27&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A27/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A27/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A27/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A27/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A27/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A27&lt;=0,0,IF(A27&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A27/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A27/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D27" s="5">
@@ -3055,7 +3055,7 @@
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>IF(A28&lt;=0,0,IF(A28&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A28/($B$17*$B$7))^(1/$B$18)),IF(A28&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A28/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A28/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A28/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A28/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A28/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A28&lt;=0,0,IF(A28&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A28/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A28/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D28" s="5">
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="C29" s="5">
-        <f>IF(A29&lt;=0,0,IF(A29&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A29/($B$17*$B$7))^(1/$B$18)),IF(A29&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A29/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A29/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A29/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A29/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A29/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A29&lt;=0,0,IF(A29&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A29/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A29/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D29" s="5">
@@ -3105,7 +3105,7 @@
         <v/>
       </c>
       <c r="C30" s="5">
-        <f>IF(A30&lt;=0,0,IF(A30&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A30/($B$17*$B$7))^(1/$B$18)),IF(A30&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A30/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A30/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A30/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A30/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A30/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A30&lt;=0,0,IF(A30&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A30/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A30/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D30" s="5">
@@ -3130,7 +3130,7 @@
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>IF(A31&lt;=0,0,IF(A31&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A31/($B$17*$B$7))^(1/$B$18)),IF(A31&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A31/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A31/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A31/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A31/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A31/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A31&lt;=0,0,IF(A31&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A31/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A31/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D31" s="5">
@@ -3155,7 +3155,7 @@
         <v/>
       </c>
       <c r="C32" s="5">
-        <f>IF(A32&lt;=0,0,IF(A32&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A32/($B$17*$B$7))^(1/$B$18)),IF(A32&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A32/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A32/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A32/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A32/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A32/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A32&lt;=0,0,IF(A32&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A32/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A32/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D32" s="5">
@@ -3180,7 +3180,7 @@
         <v/>
       </c>
       <c r="C33" s="5">
-        <f>IF(A33&lt;=0,0,IF(A33&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A33/($B$17*$B$7))^(1/$B$18)),IF(A33&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A33/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A33/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A33/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A33/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A33/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A33&lt;=0,0,IF(A33&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A33/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A33/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D33" s="5">
@@ -3205,7 +3205,7 @@
         <v/>
       </c>
       <c r="C34" s="5">
-        <f>IF(A34&lt;=0,0,IF(A34&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A34/($B$17*$B$7))^(1/$B$18)),IF(A34&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A34/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A34/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A34/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A34/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A34/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A34&lt;=0,0,IF(A34&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A34/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A34/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D34" s="5">
@@ -3230,7 +3230,7 @@
         <v/>
       </c>
       <c r="C35" s="5">
-        <f>IF(A35&lt;=0,0,IF(A35&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A35/($B$17*$B$7))^(1/$B$18)),IF(A35&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A35/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A35/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A35/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A35/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A35/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A35&lt;=0,0,IF(A35&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A35/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A35/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D35" s="5">
@@ -3255,7 +3255,7 @@
         <v/>
       </c>
       <c r="C36" s="5">
-        <f>IF(A36&lt;=0,0,IF(A36&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A36/($B$17*$B$7))^(1/$B$18)),IF(A36&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A36/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A36/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A36/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A36/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A36/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A36&lt;=0,0,IF(A36&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A36/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A36/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D36" s="5">
@@ -3280,7 +3280,7 @@
         <v/>
       </c>
       <c r="C37" s="5">
-        <f>IF(A37&lt;=0,0,IF(A37&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A37/($B$17*$B$7))^(1/$B$18)),IF(A37&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A37/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A37/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A37/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A37/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A37/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A37&lt;=0,0,IF(A37&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A37/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A37/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D37" s="5">
@@ -3305,7 +3305,7 @@
         <v/>
       </c>
       <c r="C38" s="5">
-        <f>IF(A38&lt;=0,0,IF(A38&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A38/($B$17*$B$7))^(1/$B$18)),IF(A38&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A38/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A38/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A38/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A38/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A38/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A38&lt;=0,0,IF(A38&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A38/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A38/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D38" s="5">
@@ -3330,7 +3330,7 @@
         <v/>
       </c>
       <c r="C39" s="5">
-        <f>IF(A39&lt;=0,0,IF(A39&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A39/($B$17*$B$7))^(1/$B$18)),IF(A39&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A39/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A39/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A39/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A39/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A39/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A39&lt;=0,0,IF(A39&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A39/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A39/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D39" s="5">
@@ -3355,7 +3355,7 @@
         <v/>
       </c>
       <c r="C40" s="5">
-        <f>IF(A40&lt;=0,0,IF(A40&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A40/($B$17*$B$7))^(1/$B$18)),IF(A40&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A40/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A40/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A40/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A40/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A40/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A40&lt;=0,0,IF(A40&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A40/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A40/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D40" s="5">
@@ -3380,7 +3380,7 @@
         <v/>
       </c>
       <c r="C41" s="5">
-        <f>IF(A41&lt;=0,0,IF(A41&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A41/($B$17*$B$7))^(1/$B$18)),IF(A41&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A41/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A41/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A41/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A41/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A41/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A41&lt;=0,0,IF(A41&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A41/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A41/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D41" s="5">
@@ -3405,7 +3405,7 @@
         <v/>
       </c>
       <c r="C42" s="5">
-        <f>IF(A42&lt;=0,0,IF(A42&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A42/($B$17*$B$7))^(1/$B$18)),IF(A42&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A42/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A42/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A42/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A42/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A42/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A42&lt;=0,0,IF(A42&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A42/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A42/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D42" s="5">
@@ -3430,7 +3430,7 @@
         <v/>
       </c>
       <c r="C43" s="5">
-        <f>IF(A43&lt;=0,0,IF(A43&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A43/($B$17*$B$7))^(1/$B$18)),IF(A43&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A43/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A43/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A43/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A43/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A43/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A43&lt;=0,0,IF(A43&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A43/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A43/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D43" s="5">
@@ -3455,7 +3455,7 @@
         <v/>
       </c>
       <c r="C44" s="5">
-        <f>IF(A44&lt;=0,0,IF(A44&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A44/($B$17*$B$7))^(1/$B$18)),IF(A44&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A44/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A44/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A44/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A44/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A44/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A44&lt;=0,0,IF(A44&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A44/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A44/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D44" s="5">
@@ -3480,7 +3480,7 @@
         <v/>
       </c>
       <c r="C45" s="5">
-        <f>IF(A45&lt;=0,0,IF(A45&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A45/($B$17*$B$7))^(1/$B$18)),IF(A45&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A45/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A45/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A45/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A45/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A45/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A45&lt;=0,0,IF(A45&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A45/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A45/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D45" s="5">
@@ -3505,7 +3505,7 @@
         <v/>
       </c>
       <c r="C46" s="5">
-        <f>IF(A46&lt;=0,0,IF(A46&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A46/($B$17*$B$7))^(1/$B$18)),IF(A46&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A46/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A46/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A46/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A46/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A46/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A46&lt;=0,0,IF(A46&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A46/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A46/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D46" s="5">
@@ -3530,7 +3530,7 @@
         <v/>
       </c>
       <c r="C47" s="5">
-        <f>IF(A47&lt;=0,0,IF(A47&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A47/($B$17*$B$7))^(1/$B$18)),IF(A47&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A47/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A47/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A47/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A47/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A47/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A47&lt;=0,0,IF(A47&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A47/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A47/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D47" s="5">
@@ -3555,7 +3555,7 @@
         <v/>
       </c>
       <c r="C48" s="5">
-        <f>IF(A48&lt;=0,0,IF(A48&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A48/($B$17*$B$7))^(1/$B$18)),IF(A48&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A48/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A48/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A48/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A48/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A48/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A48&lt;=0,0,IF(A48&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A48/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A48/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D48" s="5">
@@ -3580,7 +3580,7 @@
         <v/>
       </c>
       <c r="C49" s="5">
-        <f>IF(A49&lt;=0,0,IF(A49&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A49/($B$17*$B$7))^(1/$B$18)),IF(A49&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A49/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A49/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A49/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A49/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A49/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A49&lt;=0,0,IF(A49&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A49/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A49/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D49" s="5">
@@ -3605,7 +3605,7 @@
         <v/>
       </c>
       <c r="C50" s="5">
-        <f>IF(A50&lt;=0,0,IF(A50&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A50/($B$17*$B$7))^(1/$B$18)),IF(A50&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A50/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A50/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A50/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A50/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A50/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A50&lt;=0,0,IF(A50&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A50/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A50/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D50" s="5">
@@ -3630,7 +3630,7 @@
         <v/>
       </c>
       <c r="C51" s="5">
-        <f>IF(A51&lt;=0,0,IF(A51&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A51/($B$17*$B$7))^(1/$B$18)),IF(A51&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A51/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A51/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A51/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A51/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A51/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A51&lt;=0,0,IF(A51&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A51/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A51/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D51" s="5">
@@ -3655,7 +3655,7 @@
         <v/>
       </c>
       <c r="C52" s="5">
-        <f>IF(A52&lt;=0,0,IF(A52&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A52/($B$17*$B$7))^(1/$B$18)),IF(A52&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A52/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A52/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A52/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A52/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A52/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A52&lt;=0,0,IF(A52&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A52/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A52/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D52" s="5">
@@ -3680,7 +3680,7 @@
         <v/>
       </c>
       <c r="C53" s="5">
-        <f>IF(A53&lt;=0,0,IF(A53&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A53/($B$17*$B$7))^(1/$B$18)),IF(A53&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A53/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A53/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A53/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A53/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A53/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A53&lt;=0,0,IF(A53&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A53/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A53/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D53" s="5">
@@ -3705,7 +3705,7 @@
         <v/>
       </c>
       <c r="C54" s="5">
-        <f>IF(A54&lt;=0,0,IF(A54&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A54/($B$17*$B$7))^(1/$B$18)),IF(A54&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A54/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A54/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A54/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A54/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A54/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A54&lt;=0,0,IF(A54&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A54/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A54/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D54" s="5">
@@ -3730,7 +3730,7 @@
         <v/>
       </c>
       <c r="C55" s="5">
-        <f>IF(A55&lt;=0,0,IF(A55&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A55/($B$17*$B$7))^(1/$B$18)),IF(A55&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A55/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A55/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A55/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A55/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A55/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A55&lt;=0,0,IF(A55&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A55/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A55/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D55" s="5">
@@ -3755,7 +3755,7 @@
         <v/>
       </c>
       <c r="C56" s="5">
-        <f>IF(A56&lt;=0,0,IF(A56&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A56/($B$17*$B$7))^(1/$B$18)),IF(A56&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A56/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A56/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A56/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A56/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A56/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A56&lt;=0,0,IF(A56&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A56/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A56/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D56" s="5">
@@ -3780,7 +3780,7 @@
         <v/>
       </c>
       <c r="C57" s="5">
-        <f>IF(A57&lt;=0,0,IF(A57&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A57/($B$17*$B$7))^(1/$B$18)),IF(A57&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A57/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A57/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A57/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A57/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A57/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A57&lt;=0,0,IF(A57&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A57/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A57/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D57" s="5">
@@ -3805,7 +3805,7 @@
         <v/>
       </c>
       <c r="C58" s="5">
-        <f>IF(A58&lt;=0,0,IF(A58&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A58/($B$17*$B$7))^(1/$B$18)),IF(A58&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A58/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A58/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A58/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A58/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A58/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A58&lt;=0,0,IF(A58&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A58/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A58/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D58" s="5">
@@ -3830,7 +3830,7 @@
         <v/>
       </c>
       <c r="C59" s="5">
-        <f>IF(A59&lt;=0,0,IF(A59&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A59/($B$17*$B$7))^(1/$B$18)),IF(A59&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A59/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A59/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A59/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A59/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A59/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A59&lt;=0,0,IF(A59&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A59/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A59/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D59" s="5">
@@ -3855,7 +3855,7 @@
         <v/>
       </c>
       <c r="C60" s="5">
-        <f>IF(A60&lt;=0,0,IF(A60&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A60/($B$17*$B$7))^(1/$B$18)),IF(A60&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A60/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A60/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A60/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A60/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A60/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A60&lt;=0,0,IF(A60&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A60/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A60/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D60" s="5">
@@ -3880,7 +3880,7 @@
         <v/>
       </c>
       <c r="C61" s="5">
-        <f>IF(A61&lt;=0,0,IF(A61&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A61/($B$17*$B$7))^(1/$B$18)),IF(A61&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A61/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A61/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A61/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A61/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A61/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A61&lt;=0,0,IF(A61&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A61/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A61/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D61" s="5">
@@ -3905,7 +3905,7 @@
         <v/>
       </c>
       <c r="C62" s="5">
-        <f>IF(A62&lt;=0,0,IF(A62&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A62/($B$17*$B$7))^(1/$B$18)),IF(A62&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A62/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A62/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A62/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A62/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A62/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A62&lt;=0,0,IF(A62&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A62/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A62/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D62" s="5">
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="C63" s="5">
-        <f>IF(A63&lt;=0,0,IF(A63&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A63/($B$17*$B$7))^(1/$B$18)),IF(A63&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A63/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A63/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A63/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A63/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A63/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A63&lt;=0,0,IF(A63&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A63/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A63/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D63" s="5">
@@ -3955,7 +3955,7 @@
         <v/>
       </c>
       <c r="C64" s="5">
-        <f>IF(A64&lt;=0,0,IF(A64&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A64/($B$17*$B$7))^(1/$B$18)),IF(A64&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A64/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A64/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A64/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A64/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A64/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A64&lt;=0,0,IF(A64&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A64/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A64/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D64" s="5">
@@ -3980,7 +3980,7 @@
         <v/>
       </c>
       <c r="C65" s="5">
-        <f>IF(A65&lt;=0,0,IF(A65&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A65/($B$17*$B$7))^(1/$B$18)),IF(A65&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A65/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A65/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A65/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A65/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A65/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A65&lt;=0,0,IF(A65&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A65/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A65/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D65" s="5">
@@ -4005,7 +4005,7 @@
         <v/>
       </c>
       <c r="C66" s="5">
-        <f>IF(A66&lt;=0,0,IF(A66&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A66/($B$17*$B$7))^(1/$B$18)),IF(A66&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A66/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A66/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A66/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A66/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A66/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A66&lt;=0,0,IF(A66&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A66/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A66/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D66" s="5">
@@ -4030,7 +4030,7 @@
         <v/>
       </c>
       <c r="C67" s="5">
-        <f>IF(A67&lt;=0,0,IF(A67&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A67/($B$17*$B$7))^(1/$B$18)),IF(A67&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A67/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A67/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A67/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A67/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A67/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A67&lt;=0,0,IF(A67&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A67/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A67/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D67" s="5">
@@ -4055,7 +4055,7 @@
         <v/>
       </c>
       <c r="C68" s="5">
-        <f>IF(A68&lt;=0,0,IF(A68&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A68/($B$17*$B$7))^(1/$B$18)),IF(A68&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A68/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A68/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A68/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A68/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A68/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A68&lt;=0,0,IF(A68&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A68/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A68/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D68" s="5">
@@ -4080,7 +4080,7 @@
         <v/>
       </c>
       <c r="C69" s="5">
-        <f>IF(A69&lt;=0,0,IF(A69&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A69/($B$17*$B$7))^(1/$B$18)),IF(A69&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A69/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A69/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A69/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A69/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A69/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A69&lt;=0,0,IF(A69&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A69/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A69/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D69" s="5">
@@ -4105,7 +4105,7 @@
         <v/>
       </c>
       <c r="C70" s="5">
-        <f>IF(A70&lt;=0,0,IF(A70&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A70/($B$17*$B$7))^(1/$B$18)),IF(A70&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A70/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A70/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A70/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A70/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A70/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A70&lt;=0,0,IF(A70&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A70/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A70/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D70" s="5">
@@ -4130,7 +4130,7 @@
         <v/>
       </c>
       <c r="C71" s="5">
-        <f>IF(A71&lt;=0,0,IF(A71&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A71/($B$17*$B$7))^(1/$B$18)),IF(A71&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A71/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A71/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A71/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A71/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A71/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A71&lt;=0,0,IF(A71&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A71/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A71/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D71" s="5">
@@ -4155,7 +4155,7 @@
         <v/>
       </c>
       <c r="C72" s="8">
-        <f>IF(A72&lt;=0,0,IF(A72&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A72/($B$17*$B$7))^(1/$B$18)),IF(A72&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A72/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A72/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A72/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A72/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A72/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A72&lt;=0,0,IF(A72&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A72/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A72/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D72" s="8">
@@ -4180,7 +4180,7 @@
         <v/>
       </c>
       <c r="C73" s="5">
-        <f>IF(A73&lt;=0,0,IF(A73&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A73/($B$17*$B$7))^(1/$B$18)),IF(A73&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A73/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A73/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A73/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A73/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A73/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A73&lt;=0,0,IF(A73&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A73/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A73/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D73" s="5">
@@ -4205,7 +4205,7 @@
         <v/>
       </c>
       <c r="C74" s="5">
-        <f>IF(A74&lt;=0,0,IF(A74&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A74/($B$17*$B$7))^(1/$B$18)),IF(A74&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A74/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A74/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A74/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A74/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A74/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A74&lt;=0,0,IF(A74&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A74/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A74/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D74" s="5">
@@ -4230,7 +4230,7 @@
         <v/>
       </c>
       <c r="C75" s="5">
-        <f>IF(A75&lt;=0,0,IF(A75&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A75/($B$17*$B$7))^(1/$B$18)),IF(A75&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A75/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A75/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A75/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A75/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A75/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A75&lt;=0,0,IF(A75&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A75/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A75/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D75" s="5">
@@ -4255,7 +4255,7 @@
         <v/>
       </c>
       <c r="C76" s="5">
-        <f>IF(A76&lt;=0,0,IF(A76&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A76/($B$17*$B$7))^(1/$B$18)),IF(A76&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A76/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A76/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A76/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A76/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A76/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A76&lt;=0,0,IF(A76&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A76/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A76/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D76" s="5">
@@ -4280,7 +4280,7 @@
         <v/>
       </c>
       <c r="C77" s="5">
-        <f>IF(A77&lt;=0,0,IF(A77&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A77/($B$17*$B$7))^(1/$B$18)),IF(A77&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A77/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A77/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A77/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A77/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A77/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A77&lt;=0,0,IF(A77&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A77/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A77/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D77" s="5">
@@ -4305,7 +4305,7 @@
         <v/>
       </c>
       <c r="C78" s="5">
-        <f>IF(A78&lt;=0,0,IF(A78&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A78/($B$17*$B$7))^(1/$B$18)),IF(A78&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A78/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A78/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A78/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A78/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A78/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A78&lt;=0,0,IF(A78&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A78/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A78/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D78" s="5">
@@ -4330,7 +4330,7 @@
         <v/>
       </c>
       <c r="C79" s="5">
-        <f>IF(A79&lt;=0,0,IF(A79&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A79/($B$17*$B$7))^(1/$B$18)),IF(A79&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A79/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A79/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A79/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A79/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A79/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A79&lt;=0,0,IF(A79&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A79/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A79/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D79" s="5">
@@ -4355,7 +4355,7 @@
         <v/>
       </c>
       <c r="C80" s="5">
-        <f>IF(A80&lt;=0,0,IF(A80&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A80/($B$17*$B$7))^(1/$B$18)),IF(A80&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A80/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A80/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A80/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A80/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A80/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A80&lt;=0,0,IF(A80&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A80/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A80/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D80" s="5">
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="C81" s="5">
-        <f>IF(A81&lt;=0,0,IF(A81&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A81/($B$17*$B$7))^(1/$B$18)),IF(A81&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A81/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A81/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A81/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A81/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A81/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A81&lt;=0,0,IF(A81&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A81/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A81/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D81" s="5">
@@ -4405,7 +4405,7 @@
         <v/>
       </c>
       <c r="C82" s="5">
-        <f>IF(A82&lt;=0,0,IF(A82&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A82/($B$17*$B$7))^(1/$B$18)),IF(A82&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A82/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A82/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A82/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A82/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A82/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A82&lt;=0,0,IF(A82&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A82/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A82/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D82" s="5">
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="C83" s="5">
-        <f>IF(A83&lt;=0,0,IF(A83&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A83/($B$17*$B$7))^(1/$B$18)),IF(A83&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A83/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A83/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A83/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A83/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A83/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A83&lt;=0,0,IF(A83&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A83/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A83/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D83" s="5">
@@ -4455,7 +4455,7 @@
         <v/>
       </c>
       <c r="C84" s="5">
-        <f>IF(A84&lt;=0,0,IF(A84&lt;0.95*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A84/($B$17*$B$7))^(1/$B$18)),IF(A84&gt;1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A84/$B$7-$B$20)/$B$19)),(1-(MIN(1,MAX(0,(A84/$B$7-0.95)/(1.2-0.95)))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A84/($B$17*$B$7))^(1/$B$18)))+(MIN(1,MAX(0,(A84/$B$7-0.95)/(1.2-0.95))))*(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A84/$B$7-$B$20)/$B$19))))))</f>
+        <f>IF(A84&lt;=0,0,IF(A84&lt;=1.2*$B$7,1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,(A84/($B$17*$B$7))^(1/$B$18)),MAX(1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*IF($B$17*$B$7&lt;=0,0,((1.2*$B$7)/($B$17*$B$7))^(1/$B$18)),1.811*(PI()*($B$7/2)^2)*SQRT($B$7)*SQRT(MAX(0,(A84/$B$7-$B$20)/$B$19)))))</f>
         <v/>
       </c>
       <c r="D84" s="5">

</xml_diff>

<commit_message>
Automate hydrograph: Qin scales with editable Qpointe
Hydrogramme sheet stores dimensionless ratios from the original shape;
Qin = ratio × Qpointe (yellow). Calcul_A/B follow live. Documents why
t=0 is 0.081×Qpointe (0.778 at Qp=9.6), not zero.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,10 +146,10 @@
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,7 +158,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -256,7 +255,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Hydrogramme Qin</a:t>
+              <a:t>Hydrogramme Qin (scalé par Qpointe)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -270,7 +269,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Hydrogramme'!B3</f>
+              <f>'Hydrogramme'!C7</f>
             </strRef>
           </tx>
           <spPr>
@@ -288,12 +287,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Hydrogramme'!$A$4:$A$18</f>
+              <f>'Hydrogramme'!$A$8:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Hydrogramme'!$B$4:$B$18</f>
+              <f>'Hydrogramme'!$C$8:$C$20</f>
             </numRef>
           </val>
         </ser>
@@ -406,12 +405,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Calcul_A'!$A$8:$A$22</f>
+              <f>'Calcul_A'!$A$8:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcul_A'!$H$8:$H$22</f>
+              <f>'Calcul_A'!$H$8:$H$20</f>
             </numRef>
           </val>
         </ser>
@@ -524,12 +523,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Calcul_A'!$A$8:$A$22</f>
+              <f>'Calcul_A'!$A$8:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcul_A'!$B$8:$B$22</f>
+              <f>'Calcul_A'!$B$8:$B$20</f>
             </numRef>
           </val>
         </ser>
@@ -556,12 +555,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Calcul_A'!$A$8:$A$22</f>
+              <f>'Calcul_A'!$A$8:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Calcul_A'!$C$8:$C$22</f>
+              <f>'Calcul_A'!$C$8:$C$20</f>
             </numRef>
           </val>
         </ser>
@@ -801,9 +800,9 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>6</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2700000"/>
@@ -1698,207 +1697,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>Hydrogramme d'entrée (point Ø1500 / entrée rétention)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+          <t>Hydrogramme d'entrée (point Ø1500 / entrée rétention) — FORMULES LIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Qin(t) = ratio(t) × Qpointe. Changez Qpointe (jaune B4) : toute la colonne Qin et Calcul_A/B se mettent à jour. Les ratios viennent de votre hydrogramme d'origine (pointe 9,6). À t=0, ratio≈0,081 → Qin=0,778 si Qpointe=9,6 (débit de départ du projet, pas zéro).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Qpointe (m³/s) ← ÉDITER</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ex. 9.6 = pointe projet / capacité Ø1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>t pointe (min)</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Forme temporelle inchangée si vous changez seulement Qpointe</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>t (min)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ratio Q/Qp_ref</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Qin (m³/s)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Remarque</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="21" t="n">
+    <row r="8">
+      <c r="A8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>0.778</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="21" t="n">
+      <c r="B8" s="23" t="n">
+        <v>0.081042</v>
+      </c>
+      <c r="C8" s="5">
+        <f>B8*$B$4</f>
+        <v/>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Départ: ≈0.081 × Qpointe (0.778 si Qp=9.6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="21" t="n">
-        <v>8.619999999999999</v>
-      </c>
-      <c r="B6" s="22" t="n">
-        <v>1.668</v>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Qin = Qcap (croisement)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="n">
+      <c r="B9" s="23" t="n">
+        <v>0.121875</v>
+      </c>
+      <c r="C9" s="5">
+        <f>B9*$B$4</f>
+        <v/>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>1.857</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="21" t="n">
+      <c r="B10" s="23" t="n">
+        <v>0.193438</v>
+      </c>
+      <c r="C10" s="5">
+        <f>B10*$B$4</f>
+        <v/>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>3.202</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="n">
+      <c r="B11" s="23" t="n">
+        <v>0.333542</v>
+      </c>
+      <c r="C11" s="5">
+        <f>B11*$B$4</f>
+        <v/>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="n">
         <v>20</v>
       </c>
-      <c r="B9" s="5" t="n">
-        <v>6.309</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="n">
+      <c r="B12" s="23" t="n">
+        <v>0.657188</v>
+      </c>
+      <c r="C12" s="5">
+        <f>B12*$B$4</f>
+        <v/>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="n">
         <v>22.5</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Pointe</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="n">
+      <c r="B13" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="8">
+        <f>B13*$B$4</f>
+        <v/>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Pointe (ratio = 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="n">
         <v>27.5</v>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>5.846</v>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="n">
+      <c r="B14" s="23" t="n">
+        <v>0.608958</v>
+      </c>
+      <c r="C14" s="5">
+        <f>B14*$B$4</f>
+        <v/>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="n">
         <v>32.5</v>
       </c>
-      <c r="B12" s="5" t="n">
-        <v>3.857</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="n">
+      <c r="B15" s="23" t="n">
+        <v>0.401771</v>
+      </c>
+      <c r="C15" s="5">
+        <f>B15*$B$4</f>
+        <v/>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="n">
         <v>37.5</v>
       </c>
-      <c r="B13" s="5" t="n">
-        <v>2.689</v>
-      </c>
-      <c r="C13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="n">
+      <c r="B16" s="23" t="n">
+        <v>0.280104</v>
+      </c>
+      <c r="C16" s="5">
+        <f>B16*$B$4</f>
+        <v/>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="n">
         <v>42.5</v>
       </c>
-      <c r="B14" s="5" t="n">
-        <v>1.953</v>
-      </c>
-      <c r="C14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="B15" s="22" t="n">
-        <v>1.668</v>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Qin = Qcap (croisement)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="n">
+      <c r="B17" s="23" t="n">
+        <v>0.203438</v>
+      </c>
+      <c r="C17" s="5">
+        <f>B17*$B$4</f>
+        <v/>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="n">
         <v>47.5</v>
       </c>
-      <c r="B16" s="5" t="n">
-        <v>1.462</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="n">
+      <c r="B18" s="23" t="n">
+        <v>0.152292</v>
+      </c>
+      <c r="C18" s="5">
+        <f>B18*$B$4</f>
+        <v/>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="n">
         <v>52.5</v>
       </c>
-      <c r="B17" s="5" t="n">
-        <v>1.121</v>
-      </c>
-      <c r="C17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="21" t="n">
+      <c r="B19" s="23" t="n">
+        <v>0.116771</v>
+      </c>
+      <c r="C19" s="5">
+        <f>B19*$B$4</f>
+        <v/>
+      </c>
+      <c r="D19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="n">
         <v>57.5</v>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Qpointe (m³/s)</t>
-        </is>
-      </c>
-      <c r="B20" s="23">
-        <f>MAX(B4:B18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>t pointe (min)</t>
-        </is>
-      </c>
-      <c r="B21" s="24" t="n">
-        <v>22.5</v>
+      <c r="B20" s="23" t="n">
+        <v>0.091146</v>
+      </c>
+      <c r="C20" s="5">
+        <f>B20*$B$4</f>
+        <v/>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Qin max (contrôle)</t>
+        </is>
+      </c>
+      <c r="B22" s="24">
+        <f>MAX(C8:C20)</f>
+        <v/>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>doit égaler Qpointe</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Qcap Ø900 (réf.)</t>
+        </is>
+      </c>
+      <c r="B23" s="14">
+        <f>Parametres!B22</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1910,7 +1992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1949,7 +2031,7 @@
         </is>
       </c>
       <c r="B3" s="26">
-        <f>MAX(H8:H22)</f>
+        <f>MAX(H8:H20)</f>
         <v/>
       </c>
       <c r="C3" t="inlineStr">
@@ -1966,7 +2048,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>croisement Qin=Qcap dans Hydrogramme (~8.6 min si Q=1.668)</t>
+          <t>quand Qin dépasse Qout (dépend de Qpointe et Qcap)</t>
         </is>
       </c>
     </row>
@@ -1978,7 +2060,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>croisement descendant (~45.4 min si Q=1.668)</t>
+          <t>quand Qin redescend sous Qout</t>
         </is>
       </c>
     </row>
@@ -2030,12 +2112,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21">
-        <f>Hydrogramme!A4</f>
+      <c r="A8" s="22">
+        <f>Hydrogramme!A8</f>
         <v/>
       </c>
       <c r="B8" s="5">
-        <f>Hydrogramme!B4</f>
+        <f>Hydrogramme!C8</f>
         <v/>
       </c>
       <c r="C8" s="27">
@@ -2064,12 +2146,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21">
-        <f>Hydrogramme!A5</f>
+      <c r="A9" s="22">
+        <f>Hydrogramme!A9</f>
         <v/>
       </c>
       <c r="B9" s="5">
-        <f>Hydrogramme!B5</f>
+        <f>Hydrogramme!C9</f>
         <v/>
       </c>
       <c r="C9" s="27">
@@ -2080,15 +2162,15 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="22">
         <f>(A9-A8)*60</f>
         <v/>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="22">
         <f>0.5*(B8+B9)*E9</f>
         <v/>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="22">
         <f>F9-(H9-H8)</f>
         <v/>
       </c>
@@ -2102,12 +2184,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21">
-        <f>Hydrogramme!A6</f>
+      <c r="A10" s="22">
+        <f>Hydrogramme!A10</f>
         <v/>
       </c>
       <c r="B10" s="5">
-        <f>Hydrogramme!B6</f>
+        <f>Hydrogramme!C10</f>
         <v/>
       </c>
       <c r="C10" s="27">
@@ -2118,15 +2200,15 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="22">
         <f>(A10-A9)*60</f>
         <v/>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="22">
         <f>0.5*(B9+B10)*E10</f>
         <v/>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="22">
         <f>F10-(H10-H9)</f>
         <v/>
       </c>
@@ -2140,12 +2222,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21">
-        <f>Hydrogramme!A7</f>
+      <c r="A11" s="22">
+        <f>Hydrogramme!A11</f>
         <v/>
       </c>
       <c r="B11" s="5">
-        <f>Hydrogramme!B7</f>
+        <f>Hydrogramme!C11</f>
         <v/>
       </c>
       <c r="C11" s="27">
@@ -2156,15 +2238,15 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="22">
         <f>(A11-A10)*60</f>
         <v/>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="22">
         <f>0.5*(B10+B11)*E11</f>
         <v/>
       </c>
-      <c r="G11" s="21">
+      <c r="G11" s="22">
         <f>F11-(H11-H10)</f>
         <v/>
       </c>
@@ -2178,12 +2260,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21">
-        <f>Hydrogramme!A8</f>
+      <c r="A12" s="22">
+        <f>Hydrogramme!A12</f>
         <v/>
       </c>
       <c r="B12" s="5">
-        <f>Hydrogramme!B8</f>
+        <f>Hydrogramme!C12</f>
         <v/>
       </c>
       <c r="C12" s="27">
@@ -2194,15 +2276,15 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="22">
         <f>(A12-A11)*60</f>
         <v/>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="22">
         <f>0.5*(B11+B12)*E12</f>
         <v/>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="22">
         <f>F12-(H12-H11)</f>
         <v/>
       </c>
@@ -2216,12 +2298,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21">
-        <f>Hydrogramme!A9</f>
+      <c r="A13" s="22">
+        <f>Hydrogramme!A13</f>
         <v/>
       </c>
       <c r="B13" s="5">
-        <f>Hydrogramme!B9</f>
+        <f>Hydrogramme!C13</f>
         <v/>
       </c>
       <c r="C13" s="27">
@@ -2232,15 +2314,15 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="22">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="22">
         <f>0.5*(B12+B13)*E13</f>
         <v/>
       </c>
-      <c r="G13" s="21">
+      <c r="G13" s="22">
         <f>F13-(H13-H12)</f>
         <v/>
       </c>
@@ -2254,12 +2336,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21">
-        <f>Hydrogramme!A10</f>
+      <c r="A14" s="22">
+        <f>Hydrogramme!A14</f>
         <v/>
       </c>
       <c r="B14" s="5">
-        <f>Hydrogramme!B10</f>
+        <f>Hydrogramme!C14</f>
         <v/>
       </c>
       <c r="C14" s="27">
@@ -2270,15 +2352,15 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="21">
+      <c r="E14" s="22">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="22">
         <f>0.5*(B13+B14)*E14</f>
         <v/>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="22">
         <f>F14-(H14-H13)</f>
         <v/>
       </c>
@@ -2292,12 +2374,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21">
-        <f>Hydrogramme!A11</f>
+      <c r="A15" s="22">
+        <f>Hydrogramme!A15</f>
         <v/>
       </c>
       <c r="B15" s="5">
-        <f>Hydrogramme!B11</f>
+        <f>Hydrogramme!C15</f>
         <v/>
       </c>
       <c r="C15" s="27">
@@ -2308,15 +2390,15 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="22">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="22">
         <f>0.5*(B14+B15)*E15</f>
         <v/>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="22">
         <f>F15-(H15-H14)</f>
         <v/>
       </c>
@@ -2330,12 +2412,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21">
-        <f>Hydrogramme!A12</f>
+      <c r="A16" s="22">
+        <f>Hydrogramme!A16</f>
         <v/>
       </c>
       <c r="B16" s="5">
-        <f>Hydrogramme!B12</f>
+        <f>Hydrogramme!C16</f>
         <v/>
       </c>
       <c r="C16" s="27">
@@ -2346,15 +2428,15 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="21">
+      <c r="E16" s="22">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="22">
         <f>0.5*(B15+B16)*E16</f>
         <v/>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="22">
         <f>F16-(H16-H15)</f>
         <v/>
       </c>
@@ -2368,12 +2450,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21">
-        <f>Hydrogramme!A13</f>
+      <c r="A17" s="22">
+        <f>Hydrogramme!A17</f>
         <v/>
       </c>
       <c r="B17" s="5">
-        <f>Hydrogramme!B13</f>
+        <f>Hydrogramme!C17</f>
         <v/>
       </c>
       <c r="C17" s="27">
@@ -2384,15 +2466,15 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="22">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="22">
         <f>0.5*(B16+B17)*E17</f>
         <v/>
       </c>
-      <c r="G17" s="21">
+      <c r="G17" s="22">
         <f>F17-(H17-H16)</f>
         <v/>
       </c>
@@ -2406,12 +2488,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21">
-        <f>Hydrogramme!A14</f>
+      <c r="A18" s="22">
+        <f>Hydrogramme!A18</f>
         <v/>
       </c>
       <c r="B18" s="5">
-        <f>Hydrogramme!B14</f>
+        <f>Hydrogramme!C18</f>
         <v/>
       </c>
       <c r="C18" s="27">
@@ -2422,15 +2504,15 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="21">
+      <c r="E18" s="22">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="F18" s="21">
+      <c r="F18" s="22">
         <f>0.5*(B17+B18)*E18</f>
         <v/>
       </c>
-      <c r="G18" s="21">
+      <c r="G18" s="22">
         <f>F18-(H18-H17)</f>
         <v/>
       </c>
@@ -2444,12 +2526,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21">
-        <f>Hydrogramme!A15</f>
+      <c r="A19" s="22">
+        <f>Hydrogramme!A19</f>
         <v/>
       </c>
       <c r="B19" s="5">
-        <f>Hydrogramme!B15</f>
+        <f>Hydrogramme!C19</f>
         <v/>
       </c>
       <c r="C19" s="27">
@@ -2460,15 +2542,15 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="22">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="22">
         <f>0.5*(B18+B19)*E19</f>
         <v/>
       </c>
-      <c r="G19" s="21">
+      <c r="G19" s="22">
         <f>F19-(H19-H18)</f>
         <v/>
       </c>
@@ -2482,12 +2564,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21">
-        <f>Hydrogramme!A16</f>
+      <c r="A20" s="22">
+        <f>Hydrogramme!A20</f>
         <v/>
       </c>
       <c r="B20" s="5">
-        <f>Hydrogramme!B16</f>
+        <f>Hydrogramme!C20</f>
         <v/>
       </c>
       <c r="C20" s="27">
@@ -2498,15 +2580,15 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="22">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="22">
         <f>0.5*(B19+B20)*E20</f>
         <v/>
       </c>
-      <c r="G20" s="21">
+      <c r="G20" s="22">
         <f>F20-(H20-H19)</f>
         <v/>
       </c>
@@ -2516,82 +2598,6 @@
       </c>
       <c r="I20" s="4">
         <f>IF(H20&gt;0.5,"oui","non")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="21">
-        <f>Hydrogramme!A17</f>
-        <v/>
-      </c>
-      <c r="B21" s="5">
-        <f>Hydrogramme!B17</f>
-        <v/>
-      </c>
-      <c r="C21" s="27">
-        <f>$B$2</f>
-        <v/>
-      </c>
-      <c r="D21" s="5">
-        <f>B21-C21</f>
-        <v/>
-      </c>
-      <c r="E21" s="21">
-        <f>(A21-A20)*60</f>
-        <v/>
-      </c>
-      <c r="F21" s="21">
-        <f>0.5*(B20+B21)*E21</f>
-        <v/>
-      </c>
-      <c r="G21" s="21">
-        <f>F21-(H21-H20)</f>
-        <v/>
-      </c>
-      <c r="H21" s="29">
-        <f>MAX(0,H20+0.5*(D20+D21)*E21)</f>
-        <v/>
-      </c>
-      <c r="I21" s="4">
-        <f>IF(H21&gt;0.5,"oui","non")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="21">
-        <f>Hydrogramme!A18</f>
-        <v/>
-      </c>
-      <c r="B22" s="5">
-        <f>Hydrogramme!B18</f>
-        <v/>
-      </c>
-      <c r="C22" s="27">
-        <f>$B$2</f>
-        <v/>
-      </c>
-      <c r="D22" s="5">
-        <f>B22-C22</f>
-        <v/>
-      </c>
-      <c r="E22" s="21">
-        <f>(A22-A21)*60</f>
-        <v/>
-      </c>
-      <c r="F22" s="21">
-        <f>0.5*(B21+B22)*E22</f>
-        <v/>
-      </c>
-      <c r="G22" s="21">
-        <f>F22-(H22-H21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="29">
-        <f>MAX(0,H21+0.5*(D21+D22)*E22)</f>
-        <v/>
-      </c>
-      <c r="I22" s="4">
-        <f>IF(H22&gt;0.5,"oui","non")</f>
         <v/>
       </c>
     </row>
@@ -2849,7 +2855,7 @@
           <t>Q_plein Manning (réf.)</t>
         </is>
       </c>
-      <c r="B15" s="33">
+      <c r="B15" s="24">
         <f>(1/B6)*(PI()*B7^2/4)*((B7/4)^(2/3))*SQRT(B11)</f>
         <v/>
       </c>
@@ -2865,7 +2871,7 @@
           <t>K (lu)</t>
         </is>
       </c>
-      <c r="B17" s="34">
+      <c r="B17" s="33">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,2,FALSE),0.0098)</f>
         <v/>
       </c>
@@ -2876,7 +2882,7 @@
           <t>M (lu)</t>
         </is>
       </c>
-      <c r="B18" s="34">
+      <c r="B18" s="33">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,3,FALSE),2)</f>
         <v/>
       </c>
@@ -2887,7 +2893,7 @@
           <t>c (lu)</t>
         </is>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="33">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,4,FALSE),0.0398)</f>
         <v/>
       </c>
@@ -2898,7 +2904,7 @@
           <t>Y (lu)</t>
         </is>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="33">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,5,FALSE),0.67)</f>
         <v/>
       </c>
@@ -2909,7 +2915,7 @@
           <t>Ke (lu)</t>
         </is>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="33">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,6,FALSE),0.5)</f>
         <v/>
       </c>
@@ -4147,10 +4153,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="35" t="n">
+      <c r="A72" s="34" t="n">
         <v>2.4</v>
       </c>
-      <c r="B72" s="35">
+      <c r="B72" s="34">
         <f>$B$9+A72</f>
         <v/>
       </c>
@@ -4486,7 +4492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4506,7 +4512,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="36" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. La courbe Courbe_QH_900 est en formules live (changer n/L/entrée/TW).</t>
         </is>
@@ -4519,7 +4525,7 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B5" s="37">
+      <c r="B5" s="36">
         <f>Parametres!B24</f>
         <v/>
       </c>
@@ -4530,7 +4536,7 @@
           <t>Q_plein réf. (m³/s)</t>
         </is>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="36">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -4542,7 +4548,7 @@
         </is>
       </c>
       <c r="B7" s="26">
-        <f>MAX(G12:G26)</f>
+        <f>MAX(G12:G24)</f>
         <v/>
       </c>
     </row>
@@ -4596,11 +4602,11 @@
     </row>
     <row r="12">
       <c r="A12" s="4">
-        <f>Hydrogramme!A4</f>
+        <f>Hydrogramme!A8</f>
         <v/>
       </c>
       <c r="B12" s="5">
-        <f>Hydrogramme!B4</f>
+        <f>Hydrogramme!C8</f>
         <v/>
       </c>
       <c r="C12" s="5" t="n">
@@ -4613,7 +4619,7 @@
         <f>MIN(B12,$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="21" t="n">
+      <c r="F12" s="22" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="29" t="n">
@@ -4622,11 +4628,11 @@
     </row>
     <row r="13">
       <c r="A13" s="4">
-        <f>Hydrogramme!A5</f>
+        <f>Hydrogramme!A9</f>
         <v/>
       </c>
       <c r="B13" s="5">
-        <f>Hydrogramme!B5</f>
+        <f>Hydrogramme!C9</f>
         <v/>
       </c>
       <c r="C13" s="5">
@@ -4641,7 +4647,7 @@
         <f>IF(G12&lt;=0.01,MIN(0.5*(B12+B13),$B$6),D13)</f>
         <v/>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="22">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
@@ -4652,11 +4658,11 @@
     </row>
     <row r="14">
       <c r="A14" s="4">
-        <f>Hydrogramme!A6</f>
+        <f>Hydrogramme!A10</f>
         <v/>
       </c>
       <c r="B14" s="5">
-        <f>Hydrogramme!B6</f>
+        <f>Hydrogramme!C10</f>
         <v/>
       </c>
       <c r="C14" s="5">
@@ -4671,7 +4677,7 @@
         <f>IF(G13&lt;=0.01,MIN(0.5*(B13+B14),$B$6),D14)</f>
         <v/>
       </c>
-      <c r="F14" s="21">
+      <c r="F14" s="22">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
@@ -4682,11 +4688,11 @@
     </row>
     <row r="15">
       <c r="A15" s="4">
-        <f>Hydrogramme!A7</f>
+        <f>Hydrogramme!A11</f>
         <v/>
       </c>
       <c r="B15" s="5">
-        <f>Hydrogramme!B7</f>
+        <f>Hydrogramme!C11</f>
         <v/>
       </c>
       <c r="C15" s="5">
@@ -4701,7 +4707,7 @@
         <f>IF(G14&lt;=0.01,MIN(0.5*(B14+B15),$B$6),D15)</f>
         <v/>
       </c>
-      <c r="F15" s="21">
+      <c r="F15" s="22">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
@@ -4712,11 +4718,11 @@
     </row>
     <row r="16">
       <c r="A16" s="4">
-        <f>Hydrogramme!A8</f>
+        <f>Hydrogramme!A12</f>
         <v/>
       </c>
       <c r="B16" s="5">
-        <f>Hydrogramme!B8</f>
+        <f>Hydrogramme!C12</f>
         <v/>
       </c>
       <c r="C16" s="5">
@@ -4731,7 +4737,7 @@
         <f>IF(G15&lt;=0.01,MIN(0.5*(B15+B16),$B$6),D16)</f>
         <v/>
       </c>
-      <c r="F16" s="21">
+      <c r="F16" s="22">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
@@ -4742,11 +4748,11 @@
     </row>
     <row r="17">
       <c r="A17" s="4">
-        <f>Hydrogramme!A9</f>
+        <f>Hydrogramme!A13</f>
         <v/>
       </c>
       <c r="B17" s="5">
-        <f>Hydrogramme!B9</f>
+        <f>Hydrogramme!C13</f>
         <v/>
       </c>
       <c r="C17" s="5">
@@ -4761,7 +4767,7 @@
         <f>IF(G16&lt;=0.01,MIN(0.5*(B16+B17),$B$6),D17)</f>
         <v/>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="22">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
@@ -4772,11 +4778,11 @@
     </row>
     <row r="18">
       <c r="A18" s="4">
-        <f>Hydrogramme!A10</f>
+        <f>Hydrogramme!A14</f>
         <v/>
       </c>
       <c r="B18" s="5">
-        <f>Hydrogramme!B10</f>
+        <f>Hydrogramme!C14</f>
         <v/>
       </c>
       <c r="C18" s="5">
@@ -4791,7 +4797,7 @@
         <f>IF(G17&lt;=0.01,MIN(0.5*(B17+B18),$B$6),D18)</f>
         <v/>
       </c>
-      <c r="F18" s="21">
+      <c r="F18" s="22">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
@@ -4802,11 +4808,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4">
-        <f>Hydrogramme!A11</f>
+        <f>Hydrogramme!A15</f>
         <v/>
       </c>
       <c r="B19" s="5">
-        <f>Hydrogramme!B11</f>
+        <f>Hydrogramme!C15</f>
         <v/>
       </c>
       <c r="C19" s="5">
@@ -4821,7 +4827,7 @@
         <f>IF(G18&lt;=0.01,MIN(0.5*(B18+B19),$B$6),D19)</f>
         <v/>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="22">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
@@ -4832,11 +4838,11 @@
     </row>
     <row r="20">
       <c r="A20" s="4">
-        <f>Hydrogramme!A12</f>
+        <f>Hydrogramme!A16</f>
         <v/>
       </c>
       <c r="B20" s="5">
-        <f>Hydrogramme!B12</f>
+        <f>Hydrogramme!C16</f>
         <v/>
       </c>
       <c r="C20" s="5">
@@ -4851,7 +4857,7 @@
         <f>IF(G19&lt;=0.01,MIN(0.5*(B19+B20),$B$6),D20)</f>
         <v/>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="22">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
@@ -4862,11 +4868,11 @@
     </row>
     <row r="21">
       <c r="A21" s="4">
-        <f>Hydrogramme!A13</f>
+        <f>Hydrogramme!A17</f>
         <v/>
       </c>
       <c r="B21" s="5">
-        <f>Hydrogramme!B13</f>
+        <f>Hydrogramme!C17</f>
         <v/>
       </c>
       <c r="C21" s="5">
@@ -4881,7 +4887,7 @@
         <f>IF(G20&lt;=0.01,MIN(0.5*(B20+B21),$B$6),D21)</f>
         <v/>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="22">
         <f>(A21-A20)*60</f>
         <v/>
       </c>
@@ -4892,11 +4898,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4">
-        <f>Hydrogramme!A14</f>
+        <f>Hydrogramme!A18</f>
         <v/>
       </c>
       <c r="B22" s="5">
-        <f>Hydrogramme!B14</f>
+        <f>Hydrogramme!C18</f>
         <v/>
       </c>
       <c r="C22" s="5">
@@ -4911,7 +4917,7 @@
         <f>IF(G21&lt;=0.01,MIN(0.5*(B21+B22),$B$6),D22)</f>
         <v/>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="22">
         <f>(A22-A21)*60</f>
         <v/>
       </c>
@@ -4922,11 +4928,11 @@
     </row>
     <row r="23">
       <c r="A23" s="4">
-        <f>Hydrogramme!A15</f>
+        <f>Hydrogramme!A19</f>
         <v/>
       </c>
       <c r="B23" s="5">
-        <f>Hydrogramme!B15</f>
+        <f>Hydrogramme!C19</f>
         <v/>
       </c>
       <c r="C23" s="5">
@@ -4941,7 +4947,7 @@
         <f>IF(G22&lt;=0.01,MIN(0.5*(B22+B23),$B$6),D23)</f>
         <v/>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="22">
         <f>(A23-A22)*60</f>
         <v/>
       </c>
@@ -4952,11 +4958,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4">
-        <f>Hydrogramme!A16</f>
+        <f>Hydrogramme!A20</f>
         <v/>
       </c>
       <c r="B24" s="5">
-        <f>Hydrogramme!B16</f>
+        <f>Hydrogramme!C20</f>
         <v/>
       </c>
       <c r="C24" s="5">
@@ -4971,72 +4977,12 @@
         <f>IF(G23&lt;=0.01,MIN(0.5*(B23+B24),$B$6),D24)</f>
         <v/>
       </c>
-      <c r="F24" s="21">
+      <c r="F24" s="22">
         <f>(A24-A23)*60</f>
         <v/>
       </c>
       <c r="G24" s="29">
         <f>MAX(0,G23+(0.5*(B23+B24)-E24)*F24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4">
-        <f>Hydrogramme!A17</f>
-        <v/>
-      </c>
-      <c r="B25" s="5">
-        <f>Hydrogramme!B17</f>
-        <v/>
-      </c>
-      <c r="C25" s="5">
-        <f>IF($B$5&gt;0,G24/$B$5,0)</f>
-        <v/>
-      </c>
-      <c r="D25" s="5">
-        <f>IF(C25&lt;=0,0,IF(C25&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1))+(C25-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C25,Courbe_QH_900!$A$24:$A$84,1)))))</f>
-        <v/>
-      </c>
-      <c r="E25" s="5">
-        <f>IF(G24&lt;=0.01,MIN(0.5*(B24+B25),$B$6),D25)</f>
-        <v/>
-      </c>
-      <c r="F25" s="21">
-        <f>(A25-A24)*60</f>
-        <v/>
-      </c>
-      <c r="G25" s="29">
-        <f>MAX(0,G24+(0.5*(B24+B25)-E25)*F25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4">
-        <f>Hydrogramme!A18</f>
-        <v/>
-      </c>
-      <c r="B26" s="5">
-        <f>Hydrogramme!B18</f>
-        <v/>
-      </c>
-      <c r="C26" s="5">
-        <f>IF($B$5&gt;0,G25/$B$5,0)</f>
-        <v/>
-      </c>
-      <c r="D26" s="5">
-        <f>IF(C26&lt;=0,0,IF(C26&gt;=INDEX(Courbe_QH_900!$A$24:$A$84,ROWS(Courbe_QH_900!$A$24:$A$84)),INDEX(Courbe_QH_900!$E$24:$E$84,ROWS(Courbe_QH_900!$E$24:$E$84)),INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1))+(C26-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)))/(INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$A$24:$A$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)))*(INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)+1)-INDEX(Courbe_QH_900!$E$24:$E$84,MATCH(C26,Courbe_QH_900!$A$24:$A$84,1)))))</f>
-        <v/>
-      </c>
-      <c r="E26" s="5">
-        <f>IF(G25&lt;=0.01,MIN(0.5*(B25+B26),$B$6),D26)</f>
-        <v/>
-      </c>
-      <c r="F26" s="21">
-        <f>(A26-A25)*60</f>
-        <v/>
-      </c>
-      <c r="G26" s="29">
-        <f>MAX(0,G25+(0.5*(B25+B26)-E26)*F26)</f>
         <v/>
       </c>
     </row>
@@ -5061,7 +5007,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Où sont les fichiers HY-8 / capacité ?</t>
         </is>
@@ -5194,7 +5140,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="38" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>

</xml_diff>

<commit_message>
Fix Stage_Storage Excel build (Parametres merge conflict)
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Calcul_A" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Courbe_QH_900" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Calcul_B" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Fichiers_lies" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Methode" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Stage_Storage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fichiers_lies" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Methode" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -122,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +146,8 @@
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,6 +167,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -796,6 +801,124 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>V cumulé vs WSE (levé)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Stage_Storage'!E10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Stage_Storage'!$A$11:$A$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Stage_Storage'!$E$11:$E$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>WSE (m)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>V (m³)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -879,6 +1002,33 @@
       <col>11</col>
       <colOff>0</colOff>
       <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2700000"/>
@@ -1188,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1548,143 +1698,199 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>WSEmax depuis levé (m) — feuille Stage_Storage</t>
+        </is>
+      </c>
+      <c r="B30" s="20">
+        <f>IF(B27&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B27&gt;=Stage_Storage!E18,"Hors table (&gt;=39.5 m — étendre levé)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B27,Stage_Storage!$E$11:$E$18,1))+(B27-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B27,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B27,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B27,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B27,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B27,Stage_Storage!$E$11:$E$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Niveau d'eau max lu sur courbe volume–cote du levé (recommandé)</t>
+        </is>
+      </c>
+    </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HW max = WSEmax − radier Ø900 (m)</t>
+        </is>
+      </c>
+      <c r="B31" s="20">
+        <f>IF(ISNUMBER(B30),B30-34.88,"")</f>
+        <v/>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Comparer à 2.40 m (limite patron = +1.5 m au-dessus du crown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Inlet control vs outlet control — qu'est-ce que ça veut dire?</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>• Inlet control (contrôle à l'entrée): le débit est limité par l'entrée du ponceau (forme d'entrée, HW/D).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Le tuyau aval « n'aspire » pas assez pour influencer — Q dépend surtout de la charge amont H, pas de L ni de n.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>• Outlet control (contrôle à la sortie / frottement): le débit dépend de la longueur, de n, de la pente et de la charge</t>
+          <t>• Inlet control (contrôle à l'entrée): le débit est limité par l'entrée du ponceau (forme d'entrée, HW/D).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (énergie amont → aval). Manning pleine section est une hypothèse de type outlet/frottement à section pleine.</t>
+          <t xml:space="preserve">  Le tuyau aval « n'aspire » pas assez pour influencer — Q dépend surtout de la charge amont H, pas de L ni de n.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>• Ici L/D = 56 (tuyau assez long) → le contrôle par frottement (outlet) est souvent plausible,</t>
+          <t>• Outlet control (contrôle à la sortie / frottement): le débit dépend de la longueur, de n, de la pente et de la charge</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  mais sans analyse FHWA/HY-8 on ne peut pas l'affirmer. Pour dimensionner la rétention, Q_plein constant est</t>
+          <t xml:space="preserve">  (énergie amont → aval). Manning pleine section est une hypothèse de type outlet/frottement à section pleine.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  en général prudent (si la charge monte, le débit réel peut être un peu plus élevé → Vmax un peu plus bas).</t>
+          <t>• Ici L/D = 56 (tuyau assez long) → le contrôle par frottement (outlet) est souvent plausible,</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t xml:space="preserve">  mais sans analyse FHWA/HY-8 on ne peut pas l'affirmer. Pour dimensionner la rétention, Q_plein constant est</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  en général prudent (si la charge monte, le débit réel peut être un peu plus élevé → Vmax un peu plus bas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>• On n'a pas besoin de trancher IC/OC pour utiliser ce classeur: garder Qout = Q_plein (ou 1.77) suffit pour une 1re estimation.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (n=0,013). Pas un jugement IC/OC complet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>• Le stockage commence quand Qin dépasse Qout; Vmax = max du volume stocké (pas (Qp−Qout)×durée).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>• Méthode B: Qout = f(H) depuis feuille Courbe_QH_900 (FHWA inlet+outlet).</t>
+          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (n=0,013). Pas un jugement IC/OC complet.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>• Voir feuille Fichiers_lies pour les anciens Excel HY-8 / ponceau+fossé.</t>
+          <t>• Le stockage commence quand Qin dépasse Qout; Vmax = max du volume stocké (pas (Qp−Qout)×durée).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>• Vérifier que le radier amont Ø900 (34.88) est bien le fond de la zone de rétention étudiée.</t>
+          <t>• Méthode B: Qout = f(H) depuis feuille Courbe_QH_900 (FHWA inlet+outlet).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>• Voir feuille Fichiers_lies pour les anciens Excel HY-8 / ponceau+fossé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>• Vérifier que le radier amont Ø900 (34.88) est bien le fond de la zone de rétention étudiée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>• Niveau max (WSEmax): feuille Stage_Storage + case Parametres!B30 (Vmax → cote du levé).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>Vmax_B courbe FHWA (m³)</t>
         </is>
       </c>
-      <c r="B47" s="18">
+      <c r="B50" s="18">
         <f>Calcul_B!B7</f>
         <v/>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Routage avec Q=f(H) — dépend de Aire_bassin (B24)</t>
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>WSEmax (rappel)</t>
+        </is>
+      </c>
+      <c r="B51" s="21">
+        <f>B30</f>
+        <v/>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Même valeur que B30 — niveau max depuis levé Stage_Storage</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="A9:H10"/>
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="A46:H46"/>
     <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A42:H42"/>
-    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A41:H41"/>
     <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A49:H49"/>
     <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A47:H47"/>
     <mergeCell ref="A45:H45"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A32:H32"/>
     <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1707,7 +1913,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Hydrogramme d'entrée (point Ø1500 / entrée rétention) — FORMULES LIVE</t>
         </is>
@@ -1742,7 +1948,7 @@
           <t>t pointe (min)</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="23" t="n">
         <v>22.5</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1774,10 +1980,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n">
+      <c r="A8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="25" t="n">
         <v>0.081042</v>
       </c>
       <c r="C8" s="5">
@@ -1791,10 +1997,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n">
+      <c r="A9" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="25" t="n">
         <v>0.121875</v>
       </c>
       <c r="C9" s="5">
@@ -1804,10 +2010,10 @@
       <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n">
+      <c r="A10" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="25" t="n">
         <v>0.193438</v>
       </c>
       <c r="C10" s="5">
@@ -1817,10 +2023,10 @@
       <c r="D10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n">
+      <c r="A11" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="25" t="n">
         <v>0.333542</v>
       </c>
       <c r="C11" s="5">
@@ -1830,10 +2036,10 @@
       <c r="D11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="n">
+      <c r="A12" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="25" t="n">
         <v>0.657188</v>
       </c>
       <c r="C12" s="5">
@@ -1843,10 +2049,10 @@
       <c r="D12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="n">
+      <c r="A13" s="24" t="n">
         <v>22.5</v>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="25" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="8">
@@ -1860,10 +2066,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="n">
+      <c r="A14" s="24" t="n">
         <v>27.5</v>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="25" t="n">
         <v>0.608958</v>
       </c>
       <c r="C14" s="5">
@@ -1873,10 +2079,10 @@
       <c r="D14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="n">
+      <c r="A15" s="24" t="n">
         <v>32.5</v>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="25" t="n">
         <v>0.401771</v>
       </c>
       <c r="C15" s="5">
@@ -1886,10 +2092,10 @@
       <c r="D15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="n">
+      <c r="A16" s="24" t="n">
         <v>37.5</v>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="25" t="n">
         <v>0.280104</v>
       </c>
       <c r="C16" s="5">
@@ -1899,10 +2105,10 @@
       <c r="D16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="n">
+      <c r="A17" s="24" t="n">
         <v>42.5</v>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="25" t="n">
         <v>0.203438</v>
       </c>
       <c r="C17" s="5">
@@ -1912,10 +2118,10 @@
       <c r="D17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="n">
+      <c r="A18" s="24" t="n">
         <v>47.5</v>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="25" t="n">
         <v>0.152292</v>
       </c>
       <c r="C18" s="5">
@@ -1925,10 +2131,10 @@
       <c r="D18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="n">
+      <c r="A19" s="24" t="n">
         <v>52.5</v>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="25" t="n">
         <v>0.116771</v>
       </c>
       <c r="C19" s="5">
@@ -1938,10 +2144,10 @@
       <c r="D19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="n">
+      <c r="A20" s="24" t="n">
         <v>57.5</v>
       </c>
-      <c r="B20" s="23" t="n">
+      <c r="B20" s="25" t="n">
         <v>0.091146</v>
       </c>
       <c r="C20" s="5">
@@ -1956,7 +2162,7 @@
           <t>Qin max (contrôle)</t>
         </is>
       </c>
-      <c r="B22" s="24">
+      <c r="B22" s="26">
         <f>MAX(C8:C20)</f>
         <v/>
       </c>
@@ -2007,7 +2213,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Méthode A — Qout constant = capacité Ø900</t>
         </is>
@@ -2019,7 +2225,7 @@
           <t>Qout (m³/s)</t>
         </is>
       </c>
-      <c r="B2" s="25">
+      <c r="B2" s="27">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -2030,7 +2236,7 @@
           <t>Vmax (m³)</t>
         </is>
       </c>
-      <c r="B3" s="26">
+      <c r="B3" s="28">
         <f>MAX(H8:H20)</f>
         <v/>
       </c>
@@ -2112,7 +2318,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22">
+      <c r="A8" s="24">
         <f>Hydrogramme!A8</f>
         <v/>
       </c>
@@ -2120,7 +2326,7 @@
         <f>Hydrogramme!C8</f>
         <v/>
       </c>
-      <c r="C8" s="27">
+      <c r="C8" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2137,7 +2343,7 @@
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="30" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="4">
@@ -2146,7 +2352,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22">
+      <c r="A9" s="24">
         <f>Hydrogramme!A9</f>
         <v/>
       </c>
@@ -2154,7 +2360,7 @@
         <f>Hydrogramme!C9</f>
         <v/>
       </c>
-      <c r="C9" s="27">
+      <c r="C9" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2162,19 +2368,19 @@
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="24">
         <f>(A9-A8)*60</f>
         <v/>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="24">
         <f>0.5*(B8+B9)*E9</f>
         <v/>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="24">
         <f>F9-(H9-H8)</f>
         <v/>
       </c>
-      <c r="H9" s="29">
+      <c r="H9" s="31">
         <f>MAX(0,H8+0.5*(D8+D9)*E9)</f>
         <v/>
       </c>
@@ -2184,7 +2390,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22">
+      <c r="A10" s="24">
         <f>Hydrogramme!A10</f>
         <v/>
       </c>
@@ -2192,7 +2398,7 @@
         <f>Hydrogramme!C10</f>
         <v/>
       </c>
-      <c r="C10" s="27">
+      <c r="C10" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2200,19 +2406,19 @@
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="24">
         <f>(A10-A9)*60</f>
         <v/>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="24">
         <f>0.5*(B9+B10)*E10</f>
         <v/>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="24">
         <f>F10-(H10-H9)</f>
         <v/>
       </c>
-      <c r="H10" s="29">
+      <c r="H10" s="31">
         <f>MAX(0,H9+0.5*(D9+D10)*E10)</f>
         <v/>
       </c>
@@ -2222,7 +2428,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22">
+      <c r="A11" s="24">
         <f>Hydrogramme!A11</f>
         <v/>
       </c>
@@ -2230,7 +2436,7 @@
         <f>Hydrogramme!C11</f>
         <v/>
       </c>
-      <c r="C11" s="27">
+      <c r="C11" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2238,19 +2444,19 @@
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="24">
         <f>(A11-A10)*60</f>
         <v/>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="24">
         <f>0.5*(B10+B11)*E11</f>
         <v/>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="24">
         <f>F11-(H11-H10)</f>
         <v/>
       </c>
-      <c r="H11" s="29">
+      <c r="H11" s="31">
         <f>MAX(0,H10+0.5*(D10+D11)*E11)</f>
         <v/>
       </c>
@@ -2260,7 +2466,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22">
+      <c r="A12" s="24">
         <f>Hydrogramme!A12</f>
         <v/>
       </c>
@@ -2268,7 +2474,7 @@
         <f>Hydrogramme!C12</f>
         <v/>
       </c>
-      <c r="C12" s="27">
+      <c r="C12" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2276,19 +2482,19 @@
         <f>B12-C12</f>
         <v/>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="24">
         <f>(A12-A11)*60</f>
         <v/>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="24">
         <f>0.5*(B11+B12)*E12</f>
         <v/>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="24">
         <f>F12-(H12-H11)</f>
         <v/>
       </c>
-      <c r="H12" s="29">
+      <c r="H12" s="31">
         <f>MAX(0,H11+0.5*(D11+D12)*E12)</f>
         <v/>
       </c>
@@ -2298,7 +2504,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22">
+      <c r="A13" s="24">
         <f>Hydrogramme!A13</f>
         <v/>
       </c>
@@ -2306,7 +2512,7 @@
         <f>Hydrogramme!C13</f>
         <v/>
       </c>
-      <c r="C13" s="27">
+      <c r="C13" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2314,19 +2520,19 @@
         <f>B13-C13</f>
         <v/>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="24">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="24">
         <f>0.5*(B12+B13)*E13</f>
         <v/>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="24">
         <f>F13-(H13-H12)</f>
         <v/>
       </c>
-      <c r="H13" s="29">
+      <c r="H13" s="31">
         <f>MAX(0,H12+0.5*(D12+D13)*E13)</f>
         <v/>
       </c>
@@ -2336,7 +2542,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22">
+      <c r="A14" s="24">
         <f>Hydrogramme!A14</f>
         <v/>
       </c>
@@ -2344,7 +2550,7 @@
         <f>Hydrogramme!C14</f>
         <v/>
       </c>
-      <c r="C14" s="27">
+      <c r="C14" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2352,19 +2558,19 @@
         <f>B14-C14</f>
         <v/>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="24">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="24">
         <f>0.5*(B13+B14)*E14</f>
         <v/>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="24">
         <f>F14-(H14-H13)</f>
         <v/>
       </c>
-      <c r="H14" s="29">
+      <c r="H14" s="31">
         <f>MAX(0,H13+0.5*(D13+D14)*E14)</f>
         <v/>
       </c>
@@ -2374,7 +2580,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22">
+      <c r="A15" s="24">
         <f>Hydrogramme!A15</f>
         <v/>
       </c>
@@ -2382,7 +2588,7 @@
         <f>Hydrogramme!C15</f>
         <v/>
       </c>
-      <c r="C15" s="27">
+      <c r="C15" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2390,19 +2596,19 @@
         <f>B15-C15</f>
         <v/>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="24">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="24">
         <f>0.5*(B14+B15)*E15</f>
         <v/>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="24">
         <f>F15-(H15-H14)</f>
         <v/>
       </c>
-      <c r="H15" s="29">
+      <c r="H15" s="31">
         <f>MAX(0,H14+0.5*(D14+D15)*E15)</f>
         <v/>
       </c>
@@ -2412,7 +2618,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22">
+      <c r="A16" s="24">
         <f>Hydrogramme!A16</f>
         <v/>
       </c>
@@ -2420,7 +2626,7 @@
         <f>Hydrogramme!C16</f>
         <v/>
       </c>
-      <c r="C16" s="27">
+      <c r="C16" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2428,19 +2634,19 @@
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="24">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="24">
         <f>0.5*(B15+B16)*E16</f>
         <v/>
       </c>
-      <c r="G16" s="22">
+      <c r="G16" s="24">
         <f>F16-(H16-H15)</f>
         <v/>
       </c>
-      <c r="H16" s="29">
+      <c r="H16" s="31">
         <f>MAX(0,H15+0.5*(D15+D16)*E16)</f>
         <v/>
       </c>
@@ -2450,7 +2656,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22">
+      <c r="A17" s="24">
         <f>Hydrogramme!A17</f>
         <v/>
       </c>
@@ -2458,7 +2664,7 @@
         <f>Hydrogramme!C17</f>
         <v/>
       </c>
-      <c r="C17" s="27">
+      <c r="C17" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2466,19 +2672,19 @@
         <f>B17-C17</f>
         <v/>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="24">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="24">
         <f>0.5*(B16+B17)*E17</f>
         <v/>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="24">
         <f>F17-(H17-H16)</f>
         <v/>
       </c>
-      <c r="H17" s="29">
+      <c r="H17" s="31">
         <f>MAX(0,H16+0.5*(D16+D17)*E17)</f>
         <v/>
       </c>
@@ -2488,7 +2694,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22">
+      <c r="A18" s="24">
         <f>Hydrogramme!A18</f>
         <v/>
       </c>
@@ -2496,7 +2702,7 @@
         <f>Hydrogramme!C18</f>
         <v/>
       </c>
-      <c r="C18" s="27">
+      <c r="C18" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2504,19 +2710,19 @@
         <f>B18-C18</f>
         <v/>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="24">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="24">
         <f>0.5*(B17+B18)*E18</f>
         <v/>
       </c>
-      <c r="G18" s="22">
+      <c r="G18" s="24">
         <f>F18-(H18-H17)</f>
         <v/>
       </c>
-      <c r="H18" s="29">
+      <c r="H18" s="31">
         <f>MAX(0,H17+0.5*(D17+D18)*E18)</f>
         <v/>
       </c>
@@ -2526,7 +2732,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22">
+      <c r="A19" s="24">
         <f>Hydrogramme!A19</f>
         <v/>
       </c>
@@ -2534,7 +2740,7 @@
         <f>Hydrogramme!C19</f>
         <v/>
       </c>
-      <c r="C19" s="27">
+      <c r="C19" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2542,19 +2748,19 @@
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="24">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="24">
         <f>0.5*(B18+B19)*E19</f>
         <v/>
       </c>
-      <c r="G19" s="22">
+      <c r="G19" s="24">
         <f>F19-(H19-H18)</f>
         <v/>
       </c>
-      <c r="H19" s="29">
+      <c r="H19" s="31">
         <f>MAX(0,H18+0.5*(D18+D19)*E19)</f>
         <v/>
       </c>
@@ -2564,7 +2770,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22">
+      <c r="A20" s="24">
         <f>Hydrogramme!A20</f>
         <v/>
       </c>
@@ -2572,7 +2778,7 @@
         <f>Hydrogramme!C20</f>
         <v/>
       </c>
-      <c r="C20" s="27">
+      <c r="C20" s="29">
         <f>$B$2</f>
         <v/>
       </c>
@@ -2580,19 +2786,19 @@
         <f>B20-C20</f>
         <v/>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="24">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="24">
         <f>0.5*(B19+B20)*E20</f>
         <v/>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="24">
         <f>F20-(H20-H19)</f>
         <v/>
       </c>
-      <c r="H20" s="29">
+      <c r="H20" s="31">
         <f>MAX(0,H19+0.5*(D19+D20)*E20)</f>
         <v/>
       </c>
@@ -2626,7 +2832,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Courbe de capacité Ø900 — Q = f(H) (FHWA HDS-5 inlet + outlet) — FORMULES LIVE</t>
         </is>
@@ -2666,32 +2872,32 @@
           <t>béton typ. 0.012–0.015</t>
         </is>
       </c>
-      <c r="E6" s="30" t="inlineStr">
+      <c r="E6" s="32" t="inlineStr">
         <is>
           <t>entrée</t>
         </is>
       </c>
-      <c r="F6" s="30" t="inlineStr">
+      <c r="F6" s="32" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="G6" s="30" t="inlineStr">
+      <c r="G6" s="32" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H6" s="30" t="inlineStr">
+      <c r="H6" s="32" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="I6" s="30" t="inlineStr">
+      <c r="I6" s="32" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J6" s="30" t="inlineStr">
+      <c r="J6" s="32" t="inlineStr">
         <is>
           <t>Ke</t>
         </is>
@@ -2807,7 +3013,7 @@
           <t>S0 = (Zin-Zout)/L</t>
         </is>
       </c>
-      <c r="B11" s="31">
+      <c r="B11" s="33">
         <f>(B9-B10)/B8</f>
         <v/>
       </c>
@@ -2838,7 +3044,7 @@
           <t>Entrée (texte exact)</t>
         </is>
       </c>
-      <c r="B13" s="32" t="inlineStr">
+      <c r="B13" s="34" t="inlineStr">
         <is>
           <t>square_edge</t>
         </is>
@@ -2855,7 +3061,7 @@
           <t>Q_plein Manning (réf.)</t>
         </is>
       </c>
-      <c r="B15" s="24">
+      <c r="B15" s="26">
         <f>(1/B6)*(PI()*B7^2/4)*((B7/4)^(2/3))*SQRT(B11)</f>
         <v/>
       </c>
@@ -2871,7 +3077,7 @@
           <t>K (lu)</t>
         </is>
       </c>
-      <c r="B17" s="33">
+      <c r="B17" s="35">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,2,FALSE),0.0098)</f>
         <v/>
       </c>
@@ -2882,7 +3088,7 @@
           <t>M (lu)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="35">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,3,FALSE),2)</f>
         <v/>
       </c>
@@ -2893,7 +3099,7 @@
           <t>c (lu)</t>
         </is>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="35">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,4,FALSE),0.0398)</f>
         <v/>
       </c>
@@ -2904,7 +3110,7 @@
           <t>Y (lu)</t>
         </is>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="35">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,5,FALSE),0.67)</f>
         <v/>
       </c>
@@ -2915,7 +3121,7 @@
           <t>Ke (lu)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="35">
         <f>IFERROR(VLOOKUP(B13,$E$7:$J$9,6,FALSE),0.5)</f>
         <v/>
       </c>
@@ -2953,10 +3159,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="n">
+      <c r="A24" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="B24" s="27">
+      <c r="B24" s="29">
         <f>$B$9+A24</f>
         <v/>
       </c>
@@ -2978,10 +3184,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="n">
+      <c r="A25" s="29" t="n">
         <v>0.05</v>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="29">
         <f>$B$9+A25</f>
         <v/>
       </c>
@@ -3003,10 +3209,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="n">
+      <c r="A26" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="B26" s="27">
+      <c r="B26" s="29">
         <f>$B$9+A26</f>
         <v/>
       </c>
@@ -3028,10 +3234,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="n">
+      <c r="A27" s="29" t="n">
         <v>0.15</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="29">
         <f>$B$9+A27</f>
         <v/>
       </c>
@@ -3053,10 +3259,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="n">
+      <c r="A28" s="29" t="n">
         <v>0.2</v>
       </c>
-      <c r="B28" s="27">
+      <c r="B28" s="29">
         <f>$B$9+A28</f>
         <v/>
       </c>
@@ -3078,10 +3284,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="n">
+      <c r="A29" s="29" t="n">
         <v>0.25</v>
       </c>
-      <c r="B29" s="27">
+      <c r="B29" s="29">
         <f>$B$9+A29</f>
         <v/>
       </c>
@@ -3103,10 +3309,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="n">
+      <c r="A30" s="29" t="n">
         <v>0.3</v>
       </c>
-      <c r="B30" s="27">
+      <c r="B30" s="29">
         <f>$B$9+A30</f>
         <v/>
       </c>
@@ -3128,10 +3334,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="n">
+      <c r="A31" s="29" t="n">
         <v>0.35</v>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="29">
         <f>$B$9+A31</f>
         <v/>
       </c>
@@ -3153,10 +3359,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="n">
+      <c r="A32" s="29" t="n">
         <v>0.4</v>
       </c>
-      <c r="B32" s="27">
+      <c r="B32" s="29">
         <f>$B$9+A32</f>
         <v/>
       </c>
@@ -3178,10 +3384,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="n">
+      <c r="A33" s="29" t="n">
         <v>0.45</v>
       </c>
-      <c r="B33" s="27">
+      <c r="B33" s="29">
         <f>$B$9+A33</f>
         <v/>
       </c>
@@ -3203,10 +3409,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="n">
+      <c r="A34" s="29" t="n">
         <v>0.5</v>
       </c>
-      <c r="B34" s="27">
+      <c r="B34" s="29">
         <f>$B$9+A34</f>
         <v/>
       </c>
@@ -3228,10 +3434,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="n">
+      <c r="A35" s="29" t="n">
         <v>0.55</v>
       </c>
-      <c r="B35" s="27">
+      <c r="B35" s="29">
         <f>$B$9+A35</f>
         <v/>
       </c>
@@ -3253,10 +3459,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="n">
+      <c r="A36" s="29" t="n">
         <v>0.6</v>
       </c>
-      <c r="B36" s="27">
+      <c r="B36" s="29">
         <f>$B$9+A36</f>
         <v/>
       </c>
@@ -3278,10 +3484,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="27" t="n">
+      <c r="A37" s="29" t="n">
         <v>0.65</v>
       </c>
-      <c r="B37" s="27">
+      <c r="B37" s="29">
         <f>$B$9+A37</f>
         <v/>
       </c>
@@ -3303,10 +3509,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="n">
+      <c r="A38" s="29" t="n">
         <v>0.7</v>
       </c>
-      <c r="B38" s="27">
+      <c r="B38" s="29">
         <f>$B$9+A38</f>
         <v/>
       </c>
@@ -3328,10 +3534,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="n">
+      <c r="A39" s="29" t="n">
         <v>0.75</v>
       </c>
-      <c r="B39" s="27">
+      <c r="B39" s="29">
         <f>$B$9+A39</f>
         <v/>
       </c>
@@ -3353,10 +3559,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="27" t="n">
+      <c r="A40" s="29" t="n">
         <v>0.8</v>
       </c>
-      <c r="B40" s="27">
+      <c r="B40" s="29">
         <f>$B$9+A40</f>
         <v/>
       </c>
@@ -3378,10 +3584,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="n">
+      <c r="A41" s="29" t="n">
         <v>0.85</v>
       </c>
-      <c r="B41" s="27">
+      <c r="B41" s="29">
         <f>$B$9+A41</f>
         <v/>
       </c>
@@ -3403,10 +3609,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="n">
+      <c r="A42" s="29" t="n">
         <v>0.9</v>
       </c>
-      <c r="B42" s="27">
+      <c r="B42" s="29">
         <f>$B$9+A42</f>
         <v/>
       </c>
@@ -3428,10 +3634,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="n">
+      <c r="A43" s="29" t="n">
         <v>0.95</v>
       </c>
-      <c r="B43" s="27">
+      <c r="B43" s="29">
         <f>$B$9+A43</f>
         <v/>
       </c>
@@ -3453,10 +3659,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="27" t="n">
+      <c r="A44" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="27">
+      <c r="B44" s="29">
         <f>$B$9+A44</f>
         <v/>
       </c>
@@ -3478,10 +3684,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="n">
+      <c r="A45" s="29" t="n">
         <v>1.05</v>
       </c>
-      <c r="B45" s="27">
+      <c r="B45" s="29">
         <f>$B$9+A45</f>
         <v/>
       </c>
@@ -3503,10 +3709,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="27" t="n">
+      <c r="A46" s="29" t="n">
         <v>1.1</v>
       </c>
-      <c r="B46" s="27">
+      <c r="B46" s="29">
         <f>$B$9+A46</f>
         <v/>
       </c>
@@ -3528,10 +3734,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="27" t="n">
+      <c r="A47" s="29" t="n">
         <v>1.15</v>
       </c>
-      <c r="B47" s="27">
+      <c r="B47" s="29">
         <f>$B$9+A47</f>
         <v/>
       </c>
@@ -3553,10 +3759,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="27" t="n">
+      <c r="A48" s="29" t="n">
         <v>1.2</v>
       </c>
-      <c r="B48" s="27">
+      <c r="B48" s="29">
         <f>$B$9+A48</f>
         <v/>
       </c>
@@ -3578,10 +3784,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="27" t="n">
+      <c r="A49" s="29" t="n">
         <v>1.25</v>
       </c>
-      <c r="B49" s="27">
+      <c r="B49" s="29">
         <f>$B$9+A49</f>
         <v/>
       </c>
@@ -3603,10 +3809,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="27" t="n">
+      <c r="A50" s="29" t="n">
         <v>1.3</v>
       </c>
-      <c r="B50" s="27">
+      <c r="B50" s="29">
         <f>$B$9+A50</f>
         <v/>
       </c>
@@ -3628,10 +3834,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="27" t="n">
+      <c r="A51" s="29" t="n">
         <v>1.35</v>
       </c>
-      <c r="B51" s="27">
+      <c r="B51" s="29">
         <f>$B$9+A51</f>
         <v/>
       </c>
@@ -3653,10 +3859,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="27" t="n">
+      <c r="A52" s="29" t="n">
         <v>1.4</v>
       </c>
-      <c r="B52" s="27">
+      <c r="B52" s="29">
         <f>$B$9+A52</f>
         <v/>
       </c>
@@ -3678,10 +3884,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="27" t="n">
+      <c r="A53" s="29" t="n">
         <v>1.45</v>
       </c>
-      <c r="B53" s="27">
+      <c r="B53" s="29">
         <f>$B$9+A53</f>
         <v/>
       </c>
@@ -3703,10 +3909,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="27" t="n">
+      <c r="A54" s="29" t="n">
         <v>1.5</v>
       </c>
-      <c r="B54" s="27">
+      <c r="B54" s="29">
         <f>$B$9+A54</f>
         <v/>
       </c>
@@ -3728,10 +3934,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="27" t="n">
+      <c r="A55" s="29" t="n">
         <v>1.55</v>
       </c>
-      <c r="B55" s="27">
+      <c r="B55" s="29">
         <f>$B$9+A55</f>
         <v/>
       </c>
@@ -3753,10 +3959,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="27" t="n">
+      <c r="A56" s="29" t="n">
         <v>1.6</v>
       </c>
-      <c r="B56" s="27">
+      <c r="B56" s="29">
         <f>$B$9+A56</f>
         <v/>
       </c>
@@ -3778,10 +3984,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="27" t="n">
+      <c r="A57" s="29" t="n">
         <v>1.65</v>
       </c>
-      <c r="B57" s="27">
+      <c r="B57" s="29">
         <f>$B$9+A57</f>
         <v/>
       </c>
@@ -3803,10 +4009,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="n">
+      <c r="A58" s="29" t="n">
         <v>1.7</v>
       </c>
-      <c r="B58" s="27">
+      <c r="B58" s="29">
         <f>$B$9+A58</f>
         <v/>
       </c>
@@ -3828,10 +4034,10 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="27" t="n">
+      <c r="A59" s="29" t="n">
         <v>1.75</v>
       </c>
-      <c r="B59" s="27">
+      <c r="B59" s="29">
         <f>$B$9+A59</f>
         <v/>
       </c>
@@ -3853,10 +4059,10 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="27" t="n">
+      <c r="A60" s="29" t="n">
         <v>1.8</v>
       </c>
-      <c r="B60" s="27">
+      <c r="B60" s="29">
         <f>$B$9+A60</f>
         <v/>
       </c>
@@ -3878,10 +4084,10 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="27" t="n">
+      <c r="A61" s="29" t="n">
         <v>1.85</v>
       </c>
-      <c r="B61" s="27">
+      <c r="B61" s="29">
         <f>$B$9+A61</f>
         <v/>
       </c>
@@ -3903,10 +4109,10 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="27" t="n">
+      <c r="A62" s="29" t="n">
         <v>1.9</v>
       </c>
-      <c r="B62" s="27">
+      <c r="B62" s="29">
         <f>$B$9+A62</f>
         <v/>
       </c>
@@ -3928,10 +4134,10 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="27" t="n">
+      <c r="A63" s="29" t="n">
         <v>1.95</v>
       </c>
-      <c r="B63" s="27">
+      <c r="B63" s="29">
         <f>$B$9+A63</f>
         <v/>
       </c>
@@ -3953,10 +4159,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="27" t="n">
+      <c r="A64" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="B64" s="27">
+      <c r="B64" s="29">
         <f>$B$9+A64</f>
         <v/>
       </c>
@@ -3978,10 +4184,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="27" t="n">
+      <c r="A65" s="29" t="n">
         <v>2.05</v>
       </c>
-      <c r="B65" s="27">
+      <c r="B65" s="29">
         <f>$B$9+A65</f>
         <v/>
       </c>
@@ -4003,10 +4209,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="27" t="n">
+      <c r="A66" s="29" t="n">
         <v>2.1</v>
       </c>
-      <c r="B66" s="27">
+      <c r="B66" s="29">
         <f>$B$9+A66</f>
         <v/>
       </c>
@@ -4028,10 +4234,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="27" t="n">
+      <c r="A67" s="29" t="n">
         <v>2.15</v>
       </c>
-      <c r="B67" s="27">
+      <c r="B67" s="29">
         <f>$B$9+A67</f>
         <v/>
       </c>
@@ -4053,10 +4259,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="27" t="n">
+      <c r="A68" s="29" t="n">
         <v>2.2</v>
       </c>
-      <c r="B68" s="27">
+      <c r="B68" s="29">
         <f>$B$9+A68</f>
         <v/>
       </c>
@@ -4078,10 +4284,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="27" t="n">
+      <c r="A69" s="29" t="n">
         <v>2.25</v>
       </c>
-      <c r="B69" s="27">
+      <c r="B69" s="29">
         <f>$B$9+A69</f>
         <v/>
       </c>
@@ -4103,10 +4309,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="27" t="n">
+      <c r="A70" s="29" t="n">
         <v>2.3</v>
       </c>
-      <c r="B70" s="27">
+      <c r="B70" s="29">
         <f>$B$9+A70</f>
         <v/>
       </c>
@@ -4128,10 +4334,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="27" t="n">
+      <c r="A71" s="29" t="n">
         <v>2.35</v>
       </c>
-      <c r="B71" s="27">
+      <c r="B71" s="29">
         <f>$B$9+A71</f>
         <v/>
       </c>
@@ -4153,10 +4359,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="34" t="n">
+      <c r="A72" s="36" t="n">
         <v>2.4</v>
       </c>
-      <c r="B72" s="34">
+      <c r="B72" s="36">
         <f>$B$9+A72</f>
         <v/>
       </c>
@@ -4178,10 +4384,10 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="27" t="n">
+      <c r="A73" s="29" t="n">
         <v>2.45</v>
       </c>
-      <c r="B73" s="27">
+      <c r="B73" s="29">
         <f>$B$9+A73</f>
         <v/>
       </c>
@@ -4203,10 +4409,10 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="27" t="n">
+      <c r="A74" s="29" t="n">
         <v>2.5</v>
       </c>
-      <c r="B74" s="27">
+      <c r="B74" s="29">
         <f>$B$9+A74</f>
         <v/>
       </c>
@@ -4228,10 +4434,10 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="27" t="n">
+      <c r="A75" s="29" t="n">
         <v>2.55</v>
       </c>
-      <c r="B75" s="27">
+      <c r="B75" s="29">
         <f>$B$9+A75</f>
         <v/>
       </c>
@@ -4253,10 +4459,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="27" t="n">
+      <c r="A76" s="29" t="n">
         <v>2.6</v>
       </c>
-      <c r="B76" s="27">
+      <c r="B76" s="29">
         <f>$B$9+A76</f>
         <v/>
       </c>
@@ -4278,10 +4484,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="27" t="n">
+      <c r="A77" s="29" t="n">
         <v>2.65</v>
       </c>
-      <c r="B77" s="27">
+      <c r="B77" s="29">
         <f>$B$9+A77</f>
         <v/>
       </c>
@@ -4303,10 +4509,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="27" t="n">
+      <c r="A78" s="29" t="n">
         <v>2.7</v>
       </c>
-      <c r="B78" s="27">
+      <c r="B78" s="29">
         <f>$B$9+A78</f>
         <v/>
       </c>
@@ -4328,10 +4534,10 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="27" t="n">
+      <c r="A79" s="29" t="n">
         <v>2.75</v>
       </c>
-      <c r="B79" s="27">
+      <c r="B79" s="29">
         <f>$B$9+A79</f>
         <v/>
       </c>
@@ -4353,10 +4559,10 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="27" t="n">
+      <c r="A80" s="29" t="n">
         <v>2.8</v>
       </c>
-      <c r="B80" s="27">
+      <c r="B80" s="29">
         <f>$B$9+A80</f>
         <v/>
       </c>
@@ -4378,10 +4584,10 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="27" t="n">
+      <c r="A81" s="29" t="n">
         <v>2.85</v>
       </c>
-      <c r="B81" s="27">
+      <c r="B81" s="29">
         <f>$B$9+A81</f>
         <v/>
       </c>
@@ -4403,10 +4609,10 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="27" t="n">
+      <c r="A82" s="29" t="n">
         <v>2.9</v>
       </c>
-      <c r="B82" s="27">
+      <c r="B82" s="29">
         <f>$B$9+A82</f>
         <v/>
       </c>
@@ -4428,10 +4634,10 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="27" t="n">
+      <c r="A83" s="29" t="n">
         <v>2.95</v>
       </c>
-      <c r="B83" s="27">
+      <c r="B83" s="29">
         <f>$B$9+A83</f>
         <v/>
       </c>
@@ -4453,10 +4659,10 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="27" t="n">
+      <c r="A84" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="B84" s="27">
+      <c r="B84" s="29">
         <f>$B$9+A84</f>
         <v/>
       </c>
@@ -4505,14 +4711,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Méthode B — routage avec Qout = f(H) depuis Courbe_QH_900 (FHWA)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="35" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>H = V / Aire_bassin. Qout interpolé sur Courbe_QH_900!E (Q gouvernant). Si V≈0, Qout = MIN(Qin, Q_plein). ΔV = (Qin_moy - Qout)*Δt. La courbe Courbe_QH_900 est en formules live (changer n/L/entrée/TW).</t>
         </is>
@@ -4525,7 +4731,7 @@
           <t>Aire (m²)</t>
         </is>
       </c>
-      <c r="B5" s="36">
+      <c r="B5" s="38">
         <f>Parametres!B24</f>
         <v/>
       </c>
@@ -4536,7 +4742,7 @@
           <t>Q_plein réf. (m³/s)</t>
         </is>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="38">
         <f>Parametres!B22</f>
         <v/>
       </c>
@@ -4547,7 +4753,7 @@
           <t>Vmax_B (m³)</t>
         </is>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="28">
         <f>MAX(G12:G24)</f>
         <v/>
       </c>
@@ -4619,10 +4825,10 @@
         <f>MIN(B12,$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F12" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="29" t="n">
+      <c r="G12" s="31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4647,11 +4853,11 @@
         <f>IF(G12&lt;=0.01,MIN(0.5*(B12+B13),$B$6),D13)</f>
         <v/>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="24">
         <f>(A13-A12)*60</f>
         <v/>
       </c>
-      <c r="G13" s="29">
+      <c r="G13" s="31">
         <f>MAX(0,G12+(0.5*(B12+B13)-E13)*F13)</f>
         <v/>
       </c>
@@ -4677,11 +4883,11 @@
         <f>IF(G13&lt;=0.01,MIN(0.5*(B13+B14),$B$6),D14)</f>
         <v/>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="24">
         <f>(A14-A13)*60</f>
         <v/>
       </c>
-      <c r="G14" s="29">
+      <c r="G14" s="31">
         <f>MAX(0,G13+(0.5*(B13+B14)-E14)*F14)</f>
         <v/>
       </c>
@@ -4707,11 +4913,11 @@
         <f>IF(G14&lt;=0.01,MIN(0.5*(B14+B15),$B$6),D15)</f>
         <v/>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="24">
         <f>(A15-A14)*60</f>
         <v/>
       </c>
-      <c r="G15" s="29">
+      <c r="G15" s="31">
         <f>MAX(0,G14+(0.5*(B14+B15)-E15)*F15)</f>
         <v/>
       </c>
@@ -4737,11 +4943,11 @@
         <f>IF(G15&lt;=0.01,MIN(0.5*(B15+B16),$B$6),D16)</f>
         <v/>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="24">
         <f>(A16-A15)*60</f>
         <v/>
       </c>
-      <c r="G16" s="29">
+      <c r="G16" s="31">
         <f>MAX(0,G15+(0.5*(B15+B16)-E16)*F16)</f>
         <v/>
       </c>
@@ -4767,11 +4973,11 @@
         <f>IF(G16&lt;=0.01,MIN(0.5*(B16+B17),$B$6),D17)</f>
         <v/>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="24">
         <f>(A17-A16)*60</f>
         <v/>
       </c>
-      <c r="G17" s="29">
+      <c r="G17" s="31">
         <f>MAX(0,G16+(0.5*(B16+B17)-E17)*F17)</f>
         <v/>
       </c>
@@ -4797,11 +5003,11 @@
         <f>IF(G17&lt;=0.01,MIN(0.5*(B17+B18),$B$6),D18)</f>
         <v/>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="24">
         <f>(A18-A17)*60</f>
         <v/>
       </c>
-      <c r="G18" s="29">
+      <c r="G18" s="31">
         <f>MAX(0,G17+(0.5*(B17+B18)-E18)*F18)</f>
         <v/>
       </c>
@@ -4827,11 +5033,11 @@
         <f>IF(G18&lt;=0.01,MIN(0.5*(B18+B19),$B$6),D19)</f>
         <v/>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="24">
         <f>(A19-A18)*60</f>
         <v/>
       </c>
-      <c r="G19" s="29">
+      <c r="G19" s="31">
         <f>MAX(0,G18+(0.5*(B18+B19)-E19)*F19)</f>
         <v/>
       </c>
@@ -4857,11 +5063,11 @@
         <f>IF(G19&lt;=0.01,MIN(0.5*(B19+B20),$B$6),D20)</f>
         <v/>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="24">
         <f>(A20-A19)*60</f>
         <v/>
       </c>
-      <c r="G20" s="29">
+      <c r="G20" s="31">
         <f>MAX(0,G19+(0.5*(B19+B20)-E20)*F20)</f>
         <v/>
       </c>
@@ -4887,11 +5093,11 @@
         <f>IF(G20&lt;=0.01,MIN(0.5*(B20+B21),$B$6),D21)</f>
         <v/>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="24">
         <f>(A21-A20)*60</f>
         <v/>
       </c>
-      <c r="G21" s="29">
+      <c r="G21" s="31">
         <f>MAX(0,G20+(0.5*(B20+B21)-E21)*F21)</f>
         <v/>
       </c>
@@ -4917,11 +5123,11 @@
         <f>IF(G21&lt;=0.01,MIN(0.5*(B21+B22),$B$6),D22)</f>
         <v/>
       </c>
-      <c r="F22" s="22">
+      <c r="F22" s="24">
         <f>(A22-A21)*60</f>
         <v/>
       </c>
-      <c r="G22" s="29">
+      <c r="G22" s="31">
         <f>MAX(0,G21+(0.5*(B21+B22)-E22)*F22)</f>
         <v/>
       </c>
@@ -4947,11 +5153,11 @@
         <f>IF(G22&lt;=0.01,MIN(0.5*(B22+B23),$B$6),D23)</f>
         <v/>
       </c>
-      <c r="F23" s="22">
+      <c r="F23" s="24">
         <f>(A23-A22)*60</f>
         <v/>
       </c>
-      <c r="G23" s="29">
+      <c r="G23" s="31">
         <f>MAX(0,G22+(0.5*(B22+B23)-E23)*F23)</f>
         <v/>
       </c>
@@ -4977,11 +5183,11 @@
         <f>IF(G23&lt;=0.01,MIN(0.5*(B23+B24),$B$6),D24)</f>
         <v/>
       </c>
-      <c r="F24" s="22">
+      <c r="F24" s="24">
         <f>(A24-A23)*60</f>
         <v/>
       </c>
-      <c r="G24" s="29">
+      <c r="G24" s="31">
         <f>MAX(0,G23+(0.5*(B23+B24)-E24)*F24)</f>
         <v/>
       </c>
@@ -5000,130 +5206,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="inlineStr">
-        <is>
-          <t>Où sont les fichiers HY-8 / capacité ?</t>
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>Stage–storage du levé — V = f(WSE) → lire le niveau max</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ce classeur (rétention Ø900) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>PROCÉDURE (dans CE fichier): 1) Routage → Vmax sur Parametres (Calcul_A ou B). 2) Cette feuille calcule V cumulé vs NSE/WSE à partir des surfaces du levé (jaune). 3) Parametres!B30 interpolates Vmax → WSEmax. Remplacez les surfaces jaunes par vos polygones; 543 m² @ 37.28 et 1932 m² @ 39.5 sont vos mesures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Courbe Q=f(H) FHWA pour CE Ø900 : feuille Courbe_QH_900 (ci-dessus).</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Formule d'un pas</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>V_pas (m³) = (A_basse + A_haute) / 2 × (WSE_haute − WSE_basse)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ancien Excel « type HY-8 / inlet-outlet » (autre projet / Ste-Thérèse) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  engineering/drainage-design/Ponceau_Capacite_Inlet_Outlet.xlsx</t>
+          <t>V_cumulatif = somme des V_pas depuis le radier</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Branche git: cursor/culvert-excel-capacity-model-d87f</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>WSE / NSE (m)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Surface A (m²) ← ÉDITER</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ΔWSE (m)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>V_pas (m³)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>V_cumulatif (m³)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Rôle</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" s="29" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Radier Ø900 — départ</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Modèle composé ponceau Ø1050 + fossé (FHWA + remblai) — PAS le Ø900 de rétention :</t>
+      <c r="A12" s="29" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="C12" s="29">
+        <f>A12-A11</f>
+        <v/>
+      </c>
+      <c r="D12" s="24">
+        <f>0.5*(B11+B12)*C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="31">
+        <f>E11+D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder — remplacer par levé</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx</t>
+      <c r="A13" s="29" t="n">
+        <v>36</v>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>180</v>
+      </c>
+      <c r="C13" s="29">
+        <f>A13-A12</f>
+        <v/>
+      </c>
+      <c r="D13" s="24">
+        <f>0.5*(B12+B13)*C13</f>
+        <v/>
+      </c>
+      <c r="E13" s="31">
+        <f>E12+D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder — remplacer par levé</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Branche git: cursor/ponceau-fosse-hydraulic-model-d87f</t>
+      <c r="A14" s="29" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="B14" s="17" t="n">
+        <v>320</v>
+      </c>
+      <c r="C14" s="29">
+        <f>A14-A13</f>
+        <v/>
+      </c>
+      <c r="D14" s="24">
+        <f>0.5*(B13+B14)*C14</f>
+        <v/>
+      </c>
+      <c r="E14" s="31">
+        <f>E13+D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder — remplacer par levé</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" s="29" t="n">
+        <v>37</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>480</v>
+      </c>
+      <c r="C15" s="29">
+        <f>A15-A14</f>
+        <v/>
+      </c>
+      <c r="D15" s="24">
+        <f>0.5*(B14+B15)*C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="31">
+        <f>E14+D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder — remplacer par levé</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>HEC-RAS : pas de projet .ras/.hdf pour ce Ø900. Un DEM Ste-Thérèse est dans</t>
+      <c r="A16" s="36" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>543</v>
+      </c>
+      <c r="C16" s="36">
+        <f>A16-A15</f>
+        <v/>
+      </c>
+      <c r="D16" s="39">
+        <f>0.5*(B15+B16)*C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="39">
+        <f>E15+D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>LIMITE PATRON (+1.5 m crown) — votre levé</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  engineering/hec-ras-data/ (données topo seulement).</t>
+      <c r="A17" s="29" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>700</v>
+      </c>
+      <c r="C17" s="29">
+        <f>A17-A16</f>
+        <v/>
+      </c>
+      <c r="D17" s="24">
+        <f>0.5*(B16+B17)*C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="31">
+        <f>E16+D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder — remplacer par levé</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Donc: on n'avait pas perdu un HY-8 pour ce bassin Ø900 — on avait des outils</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>similaires pour d'autres sites. La courbe de CE classeur remplace ça pour le Ø900.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A18" s="29" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>1932</v>
+      </c>
+      <c r="C18" s="29">
+        <f>A18-A17</f>
+        <v/>
+      </c>
+      <c r="D18" s="24">
+        <f>0.5*(B17+B18)*C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="31">
+        <f>E17+D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Votre levé 1932 m² — niveau optionnel plus haut</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Vmax (depuis Calcul_A)</t>
+        </is>
+      </c>
+      <c r="B21" s="18">
+        <f>Parametres!B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>WSEmax correspondant (m)</t>
+        </is>
+      </c>
+      <c r="B22" s="21">
+        <f>Parametres!B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>V disponible à 37.28 m (m³)</t>
+        </is>
+      </c>
+      <c r="B23" s="40">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Si Vmax &gt; cette valeur → le niveau dépasse la limite patron</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Comment lire le résultat</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="37" t="inlineStr">
+        <is>
+          <t>Exemple: si Vmax = 5609 m³ et V(37.28)≈558 m³, alors WSEmax est au-dessus de 37.28 m (la table ira vers 39.5 m ou 'Hors table'). Affinez en entrant les vraies surfaces aux cotes intermédiaires (jaune).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A2:G4"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A26:F28"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5133,14 +5555,147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>Où sont les fichiers HY-8 / capacité ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ce classeur (rétention Ø900) :</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/drainage-design/retention_volume/Volume_Retention_Ponceau_900.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Courbe Q=f(H) FHWA pour CE Ø900 : feuille Courbe_QH_900 (ci-dessus).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ancien Excel « type HY-8 / inlet-outlet » (autre projet / Ste-Thérèse) :</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/drainage-design/Ponceau_Capacite_Inlet_Outlet.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Branche git: cursor/culvert-excel-capacity-model-d87f</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Modèle composé ponceau Ø1050 + fossé (FHWA + remblai) — PAS le Ø900 de rétention :</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/drainage-design/ponceau_fosse_model/Ponceau_Fosse_Modele_Hydraulique.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Branche git: cursor/ponceau-fosse-hydraulic-model-d87f</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>HEC-RAS : pas de projet .ras/.hdf pour ce Ø900. Un DEM Ste-Thérèse est dans</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  engineering/hec-ras-data/ (données topo seulement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Donc: on n'avait pas perdu un HY-8 pour ce bassin Ø900 — on avait des outils</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>similaires pour d'autres sites. La courbe de CE classeur remplace ça pour le Ø900.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>Méthode — volume de rétention</t>
         </is>
@@ -5217,6 +5772,16 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>8. Niveau d'eau max: Stage_Storage (surfaces levé) + Parametres!B30 = WSEmax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Fichiers liés / anciens Excel: voir feuille Fichiers_lies.</t>
         </is>

</xml_diff>